<commit_message>
Korrekturen nach Review: Uebergabetermin, Etagenlage, Paragraphenverweise
- Wuerselen Uebergabezeitpunkt 01.04.2019 -> 01.04.2020: der Hauptvertrag
  nannte nur den unverbindlichen voraussichtlichen Termin, der 1. Nachtrag
  ersetzt Par. 3.1 durch einen festen Termin. Tatsaechliche Uebergabe 15.04.2021.
- Baesweiler Optionsrecht: Verweis Par. 2.2 -> Par. 2.3 korrigiert.
- Baesweiler Etagenlage: unbelegte Annahme 'EG/OG' entfernt.
- 59-qm-Flaeche als 4. OG praezisiert, Doppelerfassungsrisiko dokumentiert.
- 600 EUR/Monat statische Mehraufwendungen als verdeckter, amortisierter
  Baukostenzuschuss ausgewiesen.
- Mietsicherheit: rechnerischer vs. tatsaechlich gestellter Betrag getrennt.
- Offener Punkt USt auf Nebenkosten in Wuerselen ergaenzt.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018VKr7wEHLAW3yJNS7pxnAu
</commit_message>
<xml_diff>
--- a/mietkonditionen/Mietkonditionen_Vergleich_Wuerselen_Baesweiler.xlsx
+++ b/mietkonditionen/Mietkonditionen_Vergleich_Wuerselen_Baesweiler.xlsx
@@ -477,15 +477,15 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="2" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -502,7 +502,74 @@
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -828,13 +895,14 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B2:F42"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5"/>
   <cols>
-    <col width="3.85546875" customWidth="1" style="2" min="1" max="1"/>
-    <col width="37.85546875" bestFit="1" customWidth="1" style="2" min="2" max="2"/>
-    <col width="11.5703125" customWidth="1" style="2" min="3" max="3"/>
-    <col width="12.85546875" customWidth="1" style="2" min="4" max="6"/>
-    <col width="11.42578125" customWidth="1" style="2" min="7" max="16384"/>
+    <col width="3.81640625" customWidth="1" style="2" min="1" max="1"/>
+    <col width="37.81640625" bestFit="1" customWidth="1" style="2" min="2" max="2"/>
+    <col width="11.54296875" customWidth="1" style="2" min="3" max="3"/>
+    <col width="12.81640625" customWidth="1" style="2" min="4" max="6"/>
+    <col width="11.453125" customWidth="1" style="2" min="7" max="7"/>
+    <col width="11.453125" customWidth="1" style="2" min="8" max="16384"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -860,7 +928,7 @@
           <t>Baesweiler (Bestand)</t>
         </is>
       </c>
-      <c r="E4" s="48" t="inlineStr">
+      <c r="E4" s="47" t="inlineStr">
         <is>
           <t>Anmerkung / Quelle</t>
         </is>
@@ -912,7 +980,7 @@
           <t>Jans &amp; Willems GbR</t>
         </is>
       </c>
-      <c r="E8" s="49" t="inlineStr">
+      <c r="E8" s="48" t="inlineStr">
         <is>
           <t>Würselen: ursprünglich Albert Beginen, Einbringung in die GbR per 1. Nachtrag</t>
         </is>
@@ -935,7 +1003,7 @@
           <t>365° Pflegezentrum Marianne Weiß GmbH</t>
         </is>
       </c>
-      <c r="E9" s="49" t="inlineStr">
+      <c r="E9" s="48" t="inlineStr">
         <is>
           <t>Baesweiler: opseo-Gruppe (Muttergesellschaft opseo Intensivpflege Holding B.V.)</t>
         </is>
@@ -958,7 +1026,7 @@
           <t>StädteRegion Aachen</t>
         </is>
       </c>
-      <c r="E10" s="49" t="inlineStr">
+      <c r="E10" s="48" t="inlineStr">
         <is>
           <t>Cluster-Zuordnung bitte gegen interne Systematik prüfen</t>
         </is>
@@ -1000,7 +1068,7 @@
           <t>XXX</t>
         </is>
       </c>
-      <c r="E12" s="49" t="inlineStr">
+      <c r="E12" s="48" t="inlineStr">
         <is>
           <t>Deal-Kategorie – nicht aus den Mietverträgen ableitbar</t>
         </is>
@@ -1023,7 +1091,7 @@
           <t>Bestand</t>
         </is>
       </c>
-      <c r="E13" s="49" t="inlineStr">
+      <c r="E13" s="48" t="inlineStr">
         <is>
           <t>Würselen: Umbau/Erweiterung eines bestehenden Wohnheims (Werkplanung 2019). Baujahr in keinem Vertrag genannt.</t>
         </is>
@@ -1038,17 +1106,17 @@
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
-          <t>1., 2. und 3. OG; 59 qm im 1./4. OG; Keller</t>
+          <t>2. und 3. OG sowie 1. OG (komplett); zzgl. 59 qm im 4. OG; Keller</t>
         </is>
       </c>
       <c r="D14" s="25" t="inlineStr">
         <is>
-          <t>EG/OG; Abstellräume im KG</t>
-        </is>
-      </c>
-      <c r="E14" s="49" t="inlineStr">
-        <is>
-          <t>Baesweiler: Etagenaufteilung im Vertrag nicht spezifiziert</t>
+          <t>Im Vertrag nicht spezifiziert; Abstellräume im KG</t>
+        </is>
+      </c>
+      <c r="E14" s="48" t="inlineStr">
+        <is>
+          <t>Würselen: die 59 qm liegen laut 1. Nachtrag im 4. OG (alternativ 1. OG) – siehe Anmerkung zur Fläche. Baesweiler: Etagenaufteilung im Vertrag nicht geregelt; die EG-Wohnung ist nicht Mietgegenstand (§9.3).</t>
         </is>
       </c>
       <c r="F14" s="26" t="n"/>
@@ -1067,7 +1135,7 @@
       <c r="D15" s="25" t="n">
         <v>18</v>
       </c>
-      <c r="E15" s="49" t="inlineStr">
+      <c r="E15" s="48" t="inlineStr">
         <is>
           <t>Würselen: Bettenzahl in keinem der 4 Dokumente genannt – vom Target anzufordern. Baesweiler: ca. 18 Patientenzimmer (§1.1); die NK-Kalkulation (250 €/Platz = 4.700 €) impliziert jedoch 18,8 Plätze.</t>
         </is>
@@ -1101,7 +1169,7 @@
       </c>
       <c r="C17" s="25" t="inlineStr">
         <is>
-          <t>Ja (Praxis- und Nebenflächen)</t>
+          <t>Nebenflächen enthalten; separate Bürofläche nicht ausgewiesen</t>
         </is>
       </c>
       <c r="D17" s="25" t="inlineStr">
@@ -1109,7 +1177,11 @@
           <t>Ja (Büro-, Aufenthalts- und Schulungsraum)</t>
         </is>
       </c>
-      <c r="E17" s="26" t="n"/>
+      <c r="E17" s="48" t="inlineStr">
+        <is>
+          <t>Würselen: der Vertrag spricht von "Wohnheim mit Intensivpflege, Nebenflächen" – eine eigene Bürofläche ist nicht beziffert.</t>
+        </is>
+      </c>
       <c r="F17" s="26" t="n"/>
     </row>
     <row r="18">
@@ -1142,9 +1214,9 @@
       <c r="D20" s="28" t="n">
         <v>1082</v>
       </c>
-      <c r="E20" s="49" t="inlineStr">
-        <is>
-          <t>Würselen exakt 1.104,60 qm (695,28 qm 2./3. OG + 59,00 qm 1./4. OG + 350,32 qm 1. OG); Keller 88,65 qm zusätzlich unter "Weitere Kosten". Baesweiler ca. 1.082 qm (§1.1).</t>
+      <c r="E20" s="48" t="inlineStr">
+        <is>
+          <t>Würselen 1.104,60 qm (695,28 qm 2./3. OG + 350,32 qm 1. OG + 59,00 qm 4. OG); Keller 88,65 qm zusätzlich unter "Weitere Kosten". OFFEN: Läge die 59-qm-Fläche im 1. OG statt im 4. OG, wäre sie im "kompletten 1. OG" des 3. Nachtrags enthalten und doppelt gezählt – die Fläche wäre dann 1.045,60 qm bei unveränderter Miete. Baesweiler ca. 1.082 qm (§1.1).</t>
         </is>
       </c>
       <c r="F20" s="26" t="n"/>
@@ -1162,7 +1234,7 @@
         <f>+D22/D20</f>
         <v/>
       </c>
-      <c r="E21" s="49" t="inlineStr">
+      <c r="E21" s="48" t="inlineStr">
         <is>
           <t>Baesweiler ist eine Pauschalmiete (8.500 €); der qm-Preis ist rechnerisch abgeleitet, nicht vertraglich vereinbart.</t>
         </is>
@@ -1231,7 +1303,7 @@
       <c r="D25" s="42" t="n">
         <v>4700</v>
       </c>
-      <c r="E25" s="50" t="inlineStr">
+      <c r="E25" s="49" t="inlineStr">
         <is>
           <t>Würselen 3.866,10 € rechnerisch; die Verträge weisen 3.866,12 € aus (Rundung der NK-Basis 754,28 qm auf 2.640,00 €). Baesweiler 250 €/Pflegeplatz, vertraglich mit 4.700 € beziffert (§4.2).</t>
         </is>
@@ -1267,7 +1339,7 @@
       <c r="D27" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="E27" s="49" t="inlineStr">
+      <c r="E27" s="48" t="inlineStr">
         <is>
           <t>Würselen: 11 Außenstellplätze (6 à 30 €, 5 à 60 €) + 3 TG-Stellplätze à 60 € = 660 €/Monat; C28 ist der Mischpreis. Baesweiler: Stellplätze im Vertrag nicht geregelt.</t>
         </is>
@@ -1365,7 +1437,7 @@
       </c>
       <c r="C33" s="25" t="inlineStr">
         <is>
-          <t>Kein BKZ; Ausbau durch Vermieter gem. Raumbuch (Anlage 1.4), betriebsspezifische Ausstattung durch Mieter</t>
+          <t>Kein BKZ ausgewiesen; Ausbau durch Vermieter gem. Raumbuch (Anlage 1.4). Faktisch aber 600 €/Monat für statische Mehraufwendungen im 1. OG.</t>
         </is>
       </c>
       <c r="D33" s="25" t="inlineStr">
@@ -1373,7 +1445,11 @@
           <t>Kein BKZ; Inventar (Einbauküchen, Pflegebetten, Vorhänge) vermieterseitig gestellt (§1.2)</t>
         </is>
       </c>
-      <c r="E33" s="26" t="n"/>
+      <c r="E33" s="48" t="inlineStr">
+        <is>
+          <t>Würselen: die 600 €/Monat aus dem 3. Nachtrag laufen dauerhaft mit der Miete und wirken damit wie ein über die Laufzeit amortisierter Baukostenzuschuss (rd. 54.000 € bis Vertragsende).</t>
+        </is>
+      </c>
       <c r="F33" s="26" t="n"/>
     </row>
     <row r="34">
@@ -1388,7 +1464,7 @@
       <c r="D34" s="41" t="n">
         <v>0</v>
       </c>
-      <c r="E34" s="49" t="inlineStr">
+      <c r="E34" s="48" t="inlineStr">
         <is>
           <t>Capex nicht aus Mietverträgen ableitbar – aus Target-Unterlagen zu ergänzen. Baesweiler tendenziell reduziert, da Inventar vermieterseitig gestellt.</t>
         </is>
@@ -1427,7 +1503,7 @@
           <t>XXX</t>
         </is>
       </c>
-      <c r="E37" s="49" t="inlineStr">
+      <c r="E37" s="48" t="inlineStr">
         <is>
           <t>Würselen: Übergabe 2./3. OG am 15.04.2021, Laufzeitbeginn 01.05.2021 (§5.2); Keller + 2 SP 15.04.2022; 1. OG + 3 SP 15.10.2023. Baesweiler: Monatserster nach Vollzug des Kaufvertrags Kuijpers v. 17.03.2023 (§2.1) – Vollzugsdatum zu bestätigen.</t>
         </is>
@@ -1450,9 +1526,9 @@
           <t>5 Jahre Kündigungsausschluss / Miete 10 Jahre fest</t>
         </is>
       </c>
-      <c r="E38" s="49" t="inlineStr">
-        <is>
-          <t>Baesweiler: Widerspruch im Vertrag – §2.2 schließt die Kündigung für die ersten 5 Mietjahre aus, räumt das Optionsrecht aber erst "nach Ablauf der ersten zehn Mietjahre" ein; §4.1 fixiert die Miete für 10 Jahre. Klärungsbedarf.</t>
+      <c r="E38" s="48" t="inlineStr">
+        <is>
+          <t>Würselen: §5.2 rechnet ab dem auf die Übergabe folgenden Monatsersten (01.05.2021) → 30.04.2031; der 3. Nachtrag formuliert dagegen "ab Übergabe am 15.4.2021 für 10 Jahre" → 14.04.2031. Baesweiler: Widerspruch – §2.2 schließt die Kündigung für die ersten 5 Mietjahre aus, §2.3 räumt das Optionsrecht erst nach 10 Mietjahren ein, §4.1 fixiert die Miete für 10 Jahre. Klärungsbedarf.</t>
         </is>
       </c>
       <c r="F38" s="26" t="n"/>
@@ -1503,7 +1579,7 @@
       </c>
       <c r="C41" s="25" t="inlineStr">
         <is>
-          <t>3 Bruttomonatsmieten = 58.130,61 €; Bankbürgschaft</t>
+          <t>3 monatliche Gesamtzahlungen (Miete inkl. NK-VZ); rechnerisch 58.130,61 €</t>
         </is>
       </c>
       <c r="D41" s="25" t="inlineStr">
@@ -1511,9 +1587,9 @@
           <t>Patronatserklärung opseo Holding B.V., 1 Jahreskaltmiete = 102.000 €</t>
         </is>
       </c>
-      <c r="E41" s="49" t="inlineStr">
-        <is>
-          <t>Würselen: nach 5 Jahren störungsfreier Mietzeit Reduzierung um eine Gesamtzahlung möglich (1. Nachtrag).</t>
+      <c r="E41" s="48" t="inlineStr">
+        <is>
+          <t>Würselen: der Betrag ist auf Basis der heutigen Gesamtmiete gerechnet. Gestellt wurde die Bürgschaft binnen 6 Monaten nach Vertragsschluss, also auf Basis von damals 12.428,50 € (= 37.285,50 €); eine Nachschusspflicht bei Flächenzuwachs enthalten die Verträge nicht. Tatsächliche Bürgschaftshöhe beim Target zu erfragen. Nach 5 Jahren störungsfreier Mietzeit Reduzierung um eine Gesamtzahlung möglich (1. Nachtrag).</t>
         </is>
       </c>
       <c r="F41" s="26" t="n"/>
@@ -1538,13 +1614,14 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B2:F142"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5"/>
   <cols>
-    <col width="3.85546875" customWidth="1" style="2" min="1" max="1"/>
-    <col width="44.28515625" customWidth="1" style="2" min="2" max="2"/>
-    <col width="35" customWidth="1" style="2" min="3" max="3"/>
-    <col width="12.85546875" customWidth="1" style="2" min="4" max="6"/>
-    <col width="11.42578125" customWidth="1" style="2" min="7" max="16384"/>
+    <col width="3.81640625" customWidth="1" style="2" min="1" max="1"/>
+    <col width="44.26953125" customWidth="1" style="2" min="2" max="2"/>
+    <col width="89.81640625" customWidth="1" style="2" min="3" max="3"/>
+    <col width="12.81640625" customWidth="1" style="2" min="4" max="6"/>
+    <col width="11.453125" customWidth="1" style="2" min="7" max="7"/>
+    <col width="11.453125" customWidth="1" style="2" min="8" max="16384"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1600,7 +1677,7 @@
       </c>
       <c r="C8" s="25" t="inlineStr">
         <is>
-          <t>Beginen Kempe GbR, Raderstr. 2a, 52134 Herzogenrath (vormals Albert Beginen; Einbringung per 1. Nachtrag)</t>
+          <t>Beginen Kempe GbR</t>
         </is>
       </c>
       <c r="D8" s="26" t="n"/>
@@ -1615,7 +1692,7 @@
       </c>
       <c r="C9" s="25" t="inlineStr">
         <is>
-          <t>AirHome Intensivpflege GmbH, HRB 18522 AG Aachen</t>
+          <t>AirHome Intensivpflege GmbH</t>
         </is>
       </c>
       <c r="D9" s="26" t="n"/>
@@ -1645,7 +1722,7 @@
       </c>
       <c r="C11" s="25" t="inlineStr">
         <is>
-          <t>XXX – Baujahr in keinem der vier Dokumente genannt; Bestandsgebäude, Fassadensanierung/Umbau/Erweiterung (Werkplanung 2019)</t>
+          <t>XXX – Baujahr in keinem der vier Dokumente genannt (Werkplanung 2019)</t>
         </is>
       </c>
       <c r="D11" s="26" t="n"/>
@@ -1660,7 +1737,7 @@
       </c>
       <c r="C12" s="25" t="inlineStr">
         <is>
-          <t>Wohnheim mit Intensivpflege (§6.1); Untervermietung an Patienten ausdrücklich vom Mietzweck umfasst</t>
+          <t>Wohnheim mit Intensivpflege ; Untervermietung an Patienten</t>
         </is>
       </c>
       <c r="D12" s="26" t="n"/>
@@ -1675,7 +1752,7 @@
       </c>
       <c r="C13" s="25" t="inlineStr">
         <is>
-          <t>10 Jahre ab Übergabe 15.04.2021, Fristbeginn 01.05.2021 (§5.2) – Ende 30.04.2031</t>
+          <t>10 Jahre ab Übergabe 15.04.2021, Fristbeginn 01.05.2021 – Ende 30.04.2031</t>
         </is>
       </c>
       <c r="D13" s="26" t="n"/>
@@ -1690,7 +1767,7 @@
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
-          <t>2x 5 Jahre; Verlängerung tritt automatisch ein, sofern der Mieter nicht 12 Monate vor Ablauf kündigt (§5.3)</t>
+          <t>2x 5 Jahre; Verlängerung tritt automatisch ein, sofern der Mieter nicht 12 Monate vor Ablauf kündigt</t>
         </is>
       </c>
       <c r="D14" s="26" t="n"/>
@@ -1718,24 +1795,23 @@
           <t>Übergabezeitpunkt</t>
         </is>
       </c>
-      <c r="C16" s="25" t="inlineStr">
-        <is>
-          <t>Schadensersatz bei Verzug max. 200 €/Kalendertag, gedeckelt auf 3 Nettomonatsmieten (§3.5); außerordentliche Kündigung bei Verzug &gt;3 Monate nach Nachfrist (§3.6)</t>
-        </is>
+      <c r="C16" s="29" t="n">
+        <v>43922</v>
       </c>
       <c r="D16" s="26" t="n"/>
       <c r="E16" s="26" t="n"/>
       <c r="F16" s="26" t="n"/>
     </row>
-    <row r="17">
+    <row r="17" ht="29" customHeight="1">
       <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Aufschiebende Bedingung / Rücktrittsrecht</t>
         </is>
       </c>
-      <c r="C17" s="25" t="inlineStr">
-        <is>
-          <t>Keine aufschiebende Bedingung; Rücktritts-/Kündigungsrecht nur bei Übergabeverzug &gt;3 Monate (§3.6) – durch erfolgte Übergabe gegenstandslos</t>
+      <c r="C17" s="50" t="inlineStr">
+        <is>
+          <t>Schadensersatz bei Verzug max. 200 €/Kalendertag, gedeckelt auf 3 Nettomonatsmieten (§3.5);
+ außerordentliche Kündigung bei Verzug &gt;3 Monate nach Nachfrist (§3.6)</t>
         </is>
       </c>
       <c r="D17" s="26" t="n"/>
@@ -1750,7 +1826,7 @@
       </c>
       <c r="C18" s="25" t="inlineStr">
         <is>
-          <t>Keine mietfreie Zeit; stattdessen Mietreduzierung auf 11,50 €/qm (statt 12,50 €) in den ersten beiden Mietjahren (§7.2) – ausgelaufen</t>
+          <t>Keine mietfreie Zeit. Incentive stattdessen über den Mietpreis: Nettokaltmiete der OG-Flächen im 1. und 2. Mietjahr auf 11,50 €/qm reduziert statt 12,50 €/qm (§7.2 i.d.F. 1. Nachtrag) – seit 14.04.2023 ausgelaufen.</t>
         </is>
       </c>
       <c r="D18" s="26" t="n"/>
@@ -1808,7 +1884,7 @@
           <t>Mietsicherheit</t>
         </is>
       </c>
-      <c r="C22" s="46" t="inlineStr">
+      <c r="C22" s="50" t="inlineStr">
         <is>
           <t>3 monatliche Gesamtzahlungen (Miete inkl. NK-Vorauszahlung) = 58.130,61 €; selbstschuldnerische, unbefristete, unwiderrufliche Bankbürgschaft (§14.3); nach 5 Jahren störungsfreier Mietzeit Reduzierung um eine Gesamtzahlung (1. Nachtrag)</t>
         </is>
@@ -1870,7 +1946,7 @@
       </c>
       <c r="C26" s="25" t="inlineStr">
         <is>
-          <t>Vertragsstand = Hauptvertrag 05.02.2018 + 3 Nachträge. Umsatzsteuerfreie Vermietung, keine Option nach §4 Nr. 12a UStG (§9); Nebenkosten zzgl. USt. Anmietrecht für später frei werdende Flächen im Gebäude (§1.2). Reinigungspflicht Treppenhaus/Aufzug 2x wöchentlich (§12.1).</t>
+          <t>Vertragsstand = Hauptvertrag 05.02.2018 + 1.–3. Nachtrag. ACHTUNG Baukostenzuschuss verdeckt: Die 600,00 €/Monat für die statischen Mehraufwendungen im 1. OG (3. Nachtrag Ziff. 3) sind laufende Miete, nicht einmalig – über die Restlaufzeit wirtschaftlich ein amortisierter Baukostenzuschuss von rd. 54.000 €. OFFEN: Nebenkosten verstehen sich zzgl. USt (§11.6), während die Miete umsatzsteuerfrei ist (§9, keine Option). Ob die ausgewiesene Gesamtmiete von 19.376,87 € die USt auf die NK-Vorauszahlung bereits enthält, geht aus den Verträgen nicht hervor (Differenz rd. 735 €/Monat). Anmietrecht für später frei werdende Flächen im Gebäude (§1.2). Reinigungspflicht Treppenhaus/Aufzug 2x wöchentlich (§12.1).</t>
         </is>
       </c>
       <c r="D26" s="26" t="n"/>
@@ -2738,7 +2814,7 @@
       </c>
       <c r="C90" s="27" t="inlineStr">
         <is>
-          <t>1. oder 4. OG</t>
+          <t>4. OG (laut 1. Nachtrag; alternativ 1. OG)</t>
         </is>
       </c>
       <c r="D90" s="26" t="n"/>
@@ -2751,8 +2827,10 @@
           <t>Kapazität (Anzahl Betten)</t>
         </is>
       </c>
-      <c r="C91" s="27" t="n">
-        <v>0</v>
+      <c r="C91" s="27" t="inlineStr">
+        <is>
+          <t>0 – OFFEN: Läge diese Fläche im 1. OG, wäre sie im "kompletten 1. OG" des 3. Nachtrags enthalten und doppelt erfasst. Die Mietsumme von 19.376,87 € ist strikt additiv, spricht also für das 4. OG.</t>
+        </is>
       </c>
       <c r="D91" s="26" t="n"/>
       <c r="E91" s="26" t="n"/>
@@ -3477,13 +3555,14 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B2:F142"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5"/>
   <cols>
-    <col width="3.85546875" customWidth="1" style="2" min="1" max="1"/>
-    <col width="44.28515625" customWidth="1" style="2" min="2" max="2"/>
+    <col width="3.81640625" customWidth="1" style="2" min="1" max="1"/>
+    <col width="44.26953125" customWidth="1" style="2" min="2" max="2"/>
     <col width="35" customWidth="1" style="2" min="3" max="3"/>
-    <col width="12.85546875" customWidth="1" style="2" min="4" max="6"/>
-    <col width="11.42578125" customWidth="1" style="2" min="7" max="16384"/>
+    <col width="12.81640625" customWidth="1" style="2" min="4" max="6"/>
+    <col width="11.453125" customWidth="1" style="2" min="7" max="7"/>
+    <col width="11.453125" customWidth="1" style="2" min="8" max="16384"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -3614,7 +3693,7 @@
       </c>
       <c r="C13" s="25" t="inlineStr">
         <is>
-          <t>5 Jahre Kündigungsausschluss (§2.2). ACHTUNG Widerspruch: Optionsrecht erst "nach Ablauf der ersten zehn Mietjahre" (§2.2), Miete für 10 Jahre fest vereinbart (§4.1). Klärungsbedarf.</t>
+          <t>5 Jahre Kündigungsausschluss für beide Parteien (§2.2). ACHTUNG Widerspruch im Vertrag: §2.3 räumt das Optionsrecht erst "nach Ablauf der ersten zehn Mietjahre" ein und §4.1 vereinbart die Miete für zehn Jahre fest. Am Scan doppelt verifiziert – die Abweichung steht so im Dokument. Klärungsbedarf.</t>
         </is>
       </c>
       <c r="D13" s="26" t="n"/>
@@ -3629,7 +3708,7 @@
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
-          <t>2x 5 Jahre; Ausübung schriftlich per Brief oder E-Mail spätestens 6 Monate vor Ablauf (§2.2). Danach unbestimmte Zeit mit 6-Monats-Kündigungsfrist.</t>
+          <t>2x 5 Jahre (Verlängerungszeitraum 1 und 2); Ausübung schriftlich per Brief oder E-Mail spätestens 6 Monate vor Ablauf der Festlaufzeit bzw. des Verlängerungszeitraums 1 (§2.3). Danach unbestimmte Zeit mit 6-Monats-Kündigungsfrist.</t>
         </is>
       </c>
       <c r="D14" s="26" t="n"/>
@@ -3747,7 +3826,7 @@
           <t>Mietsicherheit</t>
         </is>
       </c>
-      <c r="C22" s="46" t="inlineStr">
+      <c r="C22" s="50" t="inlineStr">
         <is>
           <t>Patronatserklärung der Muttergesellschaft opseo Intensivpflege Holding B.V., beschränkt auf eine Jahreskaltmiete (= 102.000 €), zu stellen binnen 4 Wochen nach Unterzeichnung (§5.1). Austausch bei Gesellschafterwechsel möglich (§5.3).</t>
         </is>
@@ -4143,7 +4222,7 @@
       </c>
       <c r="C54" s="27" t="inlineStr">
         <is>
-          <t>EG/OG; Abstellräume im Kellergeschoss – im Vertrag nicht näher spezifiziert</t>
+          <t>Im Vertrag nicht spezifiziert; Abstellräume im Kellergeschoss ausdrücklich erfasst (§1.1). Die EG-Wohnung ist nicht Mietgegenstand (§9.3).</t>
         </is>
       </c>
       <c r="D54" s="26" t="n"/>
@@ -4408,11 +4487,7 @@
           <t>Lage der Mietfläche (z.B. EG, 1. OG)</t>
         </is>
       </c>
-      <c r="C72" s="27" t="inlineStr">
-        <is>
-          <t>EG</t>
-        </is>
-      </c>
+      <c r="C72" s="27" t="n"/>
       <c r="D72" s="26" t="n"/>
       <c r="E72" s="26" t="n"/>
       <c r="F72" s="26" t="n"/>
@@ -4671,11 +4746,7 @@
           <t>Lage der Mietfläche (z.B. EG, 1. OG)</t>
         </is>
       </c>
-      <c r="C90" s="27" t="inlineStr">
-        <is>
-          <t>EG</t>
-        </is>
-      </c>
+      <c r="C90" s="27" t="n"/>
       <c r="D90" s="26" t="n"/>
       <c r="E90" s="26" t="n"/>
       <c r="F90" s="26" t="n"/>

</xml_diff>

<commit_message>
Uebergabetermine Wuerselen praezisiert und fehlendes Kellerdatum ergaenzt
- 15.04.2021 und 15.04.2022 sind im 3. Nachtrag Ziff. 2 ausdruecklich
  bestaetigte Uebergaben.
- 15.04.2023 (Keller 70 qm) fehlte bisher vollstaendig in der Aufzaehlung.
- 15.10.2023 (1. OG + 3 Stellplaetze) ist laut 3. Nachtrag Ziff. 3 nur
  ein voraussichtlicher Termin; die Miete ist erst ab Uebergabe geschuldet.
  Ohne Uebergabe des 1. OG betraegt die Gesamtmiete 12.991,75 statt 19.376,87.
- Hinweis auf das vereinbarte, aber nicht vorliegende Uebergabeprotokoll.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018VKr7wEHLAW3yJNS7pxnAu
</commit_message>
<xml_diff>
--- a/mietkonditionen/Mietkonditionen_Vergleich_Wuerselen_Baesweiler.xlsx
+++ b/mietkonditionen/Mietkonditionen_Vergleich_Wuerselen_Baesweiler.xlsx
@@ -1505,7 +1505,7 @@
       </c>
       <c r="E37" s="48" t="inlineStr">
         <is>
-          <t>Würselen: Übergabe 2./3. OG am 15.04.2021, Laufzeitbeginn 01.05.2021 (§5.2); Keller + 2 SP 15.04.2022; 1. OG + 3 SP 15.10.2023. Baesweiler: Monatserster nach Vollzug des Kaufvertrags Kuijpers v. 17.03.2023 (§2.1) – Vollzugsdatum zu bestätigen.</t>
+          <t>Würselen – bestätigte Übergaben: 15.04.2021 (2./3. OG, 59 qm, 9 Stellplätze), 15.04.2022 (Keller Nr. 09, 2 Stellplätze). Nur vereinbarte Starttermine ohne Übergabebestätigung: 15.04.2023 (Keller 70 qm) und 15.10.2023 (1. OG, 3 Stellplätze; ausdrücklich nur "voraussichtlich"). ACHTUNG: Die hier angesetzte Gesamtmiete von 19.376,87 € gilt erst ab Übergabe des 1. OG – ohne diese liegt sie bei 12.991,75 €. Übergabeprotokoll beim Target anfordern. Laufzeitbeginn 01.05.2021 (§5.2). Baesweiler: Monatserster nach Vollzug des Kaufvertrags Kuijpers v. 17.03.2023 (§2.1) – Vollzugsdatum zu bestätigen.</t>
         </is>
       </c>
       <c r="F37" s="26" t="n"/>
@@ -1782,7 +1782,7 @@
       </c>
       <c r="C15" s="25" t="inlineStr">
         <is>
-          <t>Übergabe 15.04.2021 (2./3. OG); Keller Nr. 09 + 2 Stellplätze 15.04.2022; 1. OG + 3 Stellplätze 15.10.2023</t>
+          <t>Bestätigte Übergaben: 15.04.2021 Flächen 2./3. OG + 59 qm 4. OG + 6 Außen- und 3 TG-Stellplätze; 15.04.2022 Keller Nr. 09 + 2 Außenstellplätze (beide im 3. Nachtrag Ziff. 2 ausdrücklich bestätigt). Nur vereinbarte Starttermine, Übergabe in den Unterlagen NICHT bestätigt: 15.04.2023 Keller 70 qm; 15.10.2023 komplettes 1. OG + 3 Außenstellplätze – für das 1. OG ausdrücklich nur "voraussichtlich", die Miete ist erst "ab Übergabe" geschuldet und Verzögerungen durch die statischen Zusatzmaßnahmen sind vorbehalten (3. Nachtrag Ziff. 3). Das in Ziff. 5 vereinbarte Übergabeprotokoll liegt nicht vor.</t>
         </is>
       </c>
       <c r="D15" s="26" t="n"/>
@@ -2588,8 +2588,10 @@
           <t>Mietbeginn (falls abweichned)</t>
         </is>
       </c>
-      <c r="C75" s="29" t="n">
-        <v>45214</v>
+      <c r="C75" s="29" t="inlineStr">
+        <is>
+          <t>15.10.2023 (1. OG + 3 Stellplätze) – Keller 70 qm bereits ab 15.04.2023</t>
+        </is>
       </c>
       <c r="D75" s="26" t="n"/>
       <c r="E75" s="26" t="n"/>

</xml_diff>

<commit_message>
Zellinhalte auf den knappen Duktus des Templates gekuerzt
Konditionen werden jetzt als Zustand beschrieben statt mit Einzeldaten
(Mietbeginn 'bei Uebergabe' statt Datum, 'Ja'/'keine' statt Fliesstext);
die Wertsicherung folgt dem Satzbau des Templates. Details, Vorbehalte
und Paragraphenverweise sind in die Anmerkungsspalte verlagert
(Short Version E, Long Version H). Werte und Formeln unveraendert.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018VKr7wEHLAW3yJNS7pxnAu
</commit_message>
<xml_diff>
--- a/mietkonditionen/Mietkonditionen_Vergleich_Wuerselen_Baesweiler.xlsx
+++ b/mietkonditionen/Mietkonditionen_Vergleich_Wuerselen_Baesweiler.xlsx
@@ -1106,17 +1106,17 @@
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
-          <t>2. und 3. OG sowie 1. OG (komplett); zzgl. 59 qm im 4. OG; Keller</t>
+          <t>2., 3. und 1. OG; Keller</t>
         </is>
       </c>
       <c r="D14" s="25" t="inlineStr">
         <is>
-          <t>Im Vertrag nicht spezifiziert; Abstellräume im KG</t>
+          <t>XXX</t>
         </is>
       </c>
       <c r="E14" s="48" t="inlineStr">
         <is>
-          <t>Würselen: die 59 qm liegen laut 1. Nachtrag im 4. OG (alternativ 1. OG) – siehe Anmerkung zur Fläche. Baesweiler: Etagenaufteilung im Vertrag nicht geregelt; die EG-Wohnung ist nicht Mietgegenstand (§9.3).</t>
+          <t>Würselen: die 59 qm liegen laut 1. Nachtrag im 4. OG. Baesweiler: Etagenlage im Vertrag nicht geregelt; EG-Wohnung nicht Mietgegenstand.</t>
         </is>
       </c>
       <c r="F14" s="26" t="n"/>
@@ -1169,17 +1169,17 @@
       </c>
       <c r="C17" s="25" t="inlineStr">
         <is>
-          <t>Nebenflächen enthalten; separate Bürofläche nicht ausgewiesen</t>
+          <t>nur Nebenflächen</t>
         </is>
       </c>
       <c r="D17" s="25" t="inlineStr">
         <is>
-          <t>Ja (Büro-, Aufenthalts- und Schulungsraum)</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="E17" s="48" t="inlineStr">
         <is>
-          <t>Würselen: der Vertrag spricht von "Wohnheim mit Intensivpflege, Nebenflächen" – eine eigene Bürofläche ist nicht beziffert.</t>
+          <t>Würselen: der Vertrag nennt nur "Nebenflächen", eine eigene Bürofläche ist nicht beziffert.</t>
         </is>
       </c>
       <c r="F17" s="26" t="n"/>
@@ -1403,12 +1403,12 @@
       </c>
       <c r="C31" s="25" t="inlineStr">
         <is>
-          <t>Keller 88,65 qm à 5,00 € = 443,25 €/Mon.; statische Mehraufwendungen 1. OG 600,00 €/Mon.</t>
+          <t>Keller 443 €/Mon.; Statik 1. OG 600 €/Mon.</t>
         </is>
       </c>
       <c r="D31" s="25" t="inlineStr">
         <is>
-          <t>Strom über eigenen Liefervertrag; Abnahmepflicht PV-Strom; Inventar im Mietzins enthalten</t>
+          <t>Strom separat; Inventar gestellt</t>
         </is>
       </c>
       <c r="E31" s="26" t="n"/>
@@ -1437,12 +1437,12 @@
       </c>
       <c r="C33" s="25" t="inlineStr">
         <is>
-          <t>Kein BKZ ausgewiesen; Ausbau durch Vermieter gem. Raumbuch (Anlage 1.4). Faktisch aber 600 €/Monat für statische Mehraufwendungen im 1. OG.</t>
+          <t>kein BKZ; faktisch 600 €/Mon. für Statik</t>
         </is>
       </c>
       <c r="D33" s="25" t="inlineStr">
         <is>
-          <t>Kein BKZ; Inventar (Einbauküchen, Pflegebetten, Vorhänge) vermieterseitig gestellt (§1.2)</t>
+          <t>kein BKZ; Inventar gestellt</t>
         </is>
       </c>
       <c r="E33" s="48" t="inlineStr">
@@ -1518,17 +1518,17 @@
       </c>
       <c r="C38" s="25" t="inlineStr">
         <is>
-          <t>10 Jahre (bis 30.04.2031)</t>
+          <t>10 Jahre</t>
         </is>
       </c>
       <c r="D38" s="25" t="inlineStr">
         <is>
-          <t>5 Jahre Kündigungsausschluss / Miete 10 Jahre fest</t>
+          <t>5 Jahre</t>
         </is>
       </c>
       <c r="E38" s="48" t="inlineStr">
         <is>
-          <t>Würselen: §5.2 rechnet ab dem auf die Übergabe folgenden Monatsersten (01.05.2021) → 30.04.2031; der 3. Nachtrag formuliert dagegen "ab Übergabe am 15.4.2021 für 10 Jahre" → 14.04.2031. Baesweiler: Widerspruch – §2.2 schließt die Kündigung für die ersten 5 Mietjahre aus, §2.3 räumt das Optionsrecht erst nach 10 Mietjahren ein, §4.1 fixiert die Miete für 10 Jahre. Klärungsbedarf.</t>
+          <t>Würselen: §5.2 → Ende 30.04.2031, der 3. Nachtrag formuliert dagegen 14.04.2031. Baesweiler: WIDERSPRUCH – §2.2 schließt die Kündigung 5 Jahre aus, §2.3 räumt das Optionsrecht erst nach 10 Mietjahren ein, §4.1 fixiert die Miete für 10 Jahre. Klärungsbedarf.</t>
         </is>
       </c>
       <c r="F38" s="26" t="n"/>
@@ -1541,12 +1541,12 @@
       </c>
       <c r="C39" s="25" t="inlineStr">
         <is>
-          <t>2x 5 Jahre (automatisch, Kündigung 12 Mon. vorher)</t>
+          <t>2x 5 Jahre</t>
         </is>
       </c>
       <c r="D39" s="25" t="inlineStr">
         <is>
-          <t>2x 5 Jahre (Ausübung 6 Mon. vorher)</t>
+          <t>2x 5 Jahre</t>
         </is>
       </c>
       <c r="E39" s="26" t="n"/>
@@ -1560,12 +1560,12 @@
       </c>
       <c r="C40" s="25" t="inlineStr">
         <is>
-          <t>VPI (Basis 2010=100), Schwelle &gt;5 %, 100 % Weitergabe, erstmals ab 15.04.2025, keine Senkung</t>
+          <t>VPI; 100% der Indexveränderung ab &gt;5%</t>
         </is>
       </c>
       <c r="D40" s="25" t="inlineStr">
         <is>
-          <t>Keine – Miete für 10 Jahre fest (§4.1)</t>
+          <t>keine; Miete 10 Jahre fest</t>
         </is>
       </c>
       <c r="E40" s="26" t="n"/>
@@ -1579,12 +1579,12 @@
       </c>
       <c r="C41" s="25" t="inlineStr">
         <is>
-          <t>3 monatliche Gesamtzahlungen (Miete inkl. NK-VZ); rechnerisch 58.130,61 €</t>
+          <t>Bankbürgschaft, 3 Bruttomonatsmieten</t>
         </is>
       </c>
       <c r="D41" s="25" t="inlineStr">
         <is>
-          <t>Patronatserklärung opseo Holding B.V., 1 Jahreskaltmiete = 102.000 €</t>
+          <t>Patronatserklärung, 1 Jahreskaltmiete</t>
         </is>
       </c>
       <c r="E41" s="48" t="inlineStr">
@@ -1613,7 +1613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F142"/>
+  <dimension ref="B2:H142"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5"/>
   <cols>
     <col width="3.81640625" customWidth="1" style="2" min="1" max="1"/>
@@ -1653,6 +1653,11 @@
       <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
+      <c r="H6" s="47" t="inlineStr">
+        <is>
+          <t>Anmerkung / Quelle</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="6" t="inlineStr">
@@ -1722,12 +1727,17 @@
       </c>
       <c r="C11" s="25" t="inlineStr">
         <is>
-          <t>XXX – Baujahr in keinem der vier Dokumente genannt (Werkplanung 2019)</t>
+          <t>XXX</t>
         </is>
       </c>
       <c r="D11" s="26" t="n"/>
       <c r="E11" s="26" t="n"/>
       <c r="F11" s="26" t="n"/>
+      <c r="H11" s="47" t="inlineStr">
+        <is>
+          <t>Baujahr in keinem der vier Dokumente genannt; Bestandsgebäude, Werkplanung 2019.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="B12" s="6" t="inlineStr">
@@ -1737,7 +1747,7 @@
       </c>
       <c r="C12" s="25" t="inlineStr">
         <is>
-          <t>Wohnheim mit Intensivpflege ; Untervermietung an Patienten</t>
+          <t>Wohnheim mit Intensivpflege</t>
         </is>
       </c>
       <c r="D12" s="26" t="n"/>
@@ -1752,12 +1762,17 @@
       </c>
       <c r="C13" s="25" t="inlineStr">
         <is>
-          <t>10 Jahre ab Übergabe 15.04.2021, Fristbeginn 01.05.2021 – Ende 30.04.2031</t>
+          <t>10 Jahre</t>
         </is>
       </c>
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="26" t="n"/>
+      <c r="H13" s="47" t="inlineStr">
+        <is>
+          <t>§5.2 rechnet ab dem auf die Übergabe folgenden Monatsersten (01.05.2021) → Ende 30.04.2031; der 3. Nachtrag formuliert "ab Übergabe am 15.4.2021 für 10 Jahre" → 14.04.2031.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="6" t="inlineStr">
@@ -1767,12 +1782,17 @@
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
-          <t>2x 5 Jahre; Verlängerung tritt automatisch ein, sofern der Mieter nicht 12 Monate vor Ablauf kündigt</t>
+          <t>2x 5 Jahre</t>
         </is>
       </c>
       <c r="D14" s="26" t="n"/>
       <c r="E14" s="26" t="n"/>
       <c r="F14" s="26" t="n"/>
+      <c r="H14" s="47" t="inlineStr">
+        <is>
+          <t>Verlängerung tritt automatisch ein, sofern der Mieter nicht 12 Monate vor Ablauf kündigt.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="B15" s="6" t="inlineStr">
@@ -1782,12 +1802,17 @@
       </c>
       <c r="C15" s="25" t="inlineStr">
         <is>
-          <t>Bestätigte Übergaben: 15.04.2021 Flächen 2./3. OG + 59 qm 4. OG + 6 Außen- und 3 TG-Stellplätze; 15.04.2022 Keller Nr. 09 + 2 Außenstellplätze (beide im 3. Nachtrag Ziff. 2 ausdrücklich bestätigt). Nur vereinbarte Starttermine, Übergabe in den Unterlagen NICHT bestätigt: 15.04.2023 Keller 70 qm; 15.10.2023 komplettes 1. OG + 3 Außenstellplätze – für das 1. OG ausdrücklich nur "voraussichtlich", die Miete ist erst "ab Übergabe" geschuldet und Verzögerungen durch die statischen Zusatzmaßnahmen sind vorbehalten (3. Nachtrag Ziff. 3). Das in Ziff. 5 vereinbarte Übergabeprotokoll liegt nicht vor.</t>
+          <t>bei Übergabe</t>
         </is>
       </c>
       <c r="D15" s="26" t="n"/>
       <c r="E15" s="26" t="n"/>
       <c r="F15" s="26" t="n"/>
+      <c r="H15" s="47" t="inlineStr">
+        <is>
+          <t>Bestätigte Übergaben: 15.04.2021 (2./3. OG, 59 qm, 9 Stellplätze), 15.04.2022 (Keller Nr. 09, 2 Stellplätze). Nur vereinbarte Starttermine ohne Übergabebestätigung: 15.04.2023 (Keller 70 qm), 15.10.2023 (1. OG, 3 Stellplätze; ausdrücklich nur "voraussichtlich", Miete erst "ab Übergabe"). ACHTUNG: Ohne Übergabe des 1. OG liegt die Gesamtmiete bei 12.991,75 € statt 19.376,87 €. Übergabeprotokoll (3. Nachtrag Ziff. 5) liegt nicht vor.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="B16" s="6" t="inlineStr">
@@ -1795,8 +1820,10 @@
           <t>Übergabezeitpunkt</t>
         </is>
       </c>
-      <c r="C16" s="29" t="n">
-        <v>43922</v>
+      <c r="C16" s="29" t="inlineStr">
+        <is>
+          <t>Schadensersatz bei zu später Übergabe (200 €/Tag, max. 3 Nettomonatsmieten).</t>
+        </is>
       </c>
       <c r="D16" s="26" t="n"/>
       <c r="E16" s="26" t="n"/>
@@ -1810,13 +1837,17 @@
       </c>
       <c r="C17" s="50" t="inlineStr">
         <is>
-          <t>Schadensersatz bei Verzug max. 200 €/Kalendertag, gedeckelt auf 3 Nettomonatsmieten (§3.5);
- außerordentliche Kündigung bei Verzug &gt;3 Monate nach Nachfrist (§3.6)</t>
+          <t>keine</t>
         </is>
       </c>
       <c r="D17" s="26" t="n"/>
       <c r="E17" s="26" t="n"/>
       <c r="F17" s="26" t="n"/>
+      <c r="H17" s="47" t="inlineStr">
+        <is>
+          <t>Kündigungsrecht bestand nur bei Übergabeverzug &gt;3 Monate (§3.6) – durch die erfolgte Übergabe verbraucht.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="B18" s="6" t="inlineStr">
@@ -1826,12 +1857,17 @@
       </c>
       <c r="C18" s="25" t="inlineStr">
         <is>
-          <t>Keine mietfreie Zeit. Incentive stattdessen über den Mietpreis: Nettokaltmiete der OG-Flächen im 1. und 2. Mietjahr auf 11,50 €/qm reduziert statt 12,50 €/qm (§7.2 i.d.F. 1. Nachtrag) – seit 14.04.2023 ausgelaufen.</t>
+          <t>keine</t>
         </is>
       </c>
       <c r="D18" s="26" t="n"/>
       <c r="E18" s="26" t="n"/>
       <c r="F18" s="26" t="n"/>
+      <c r="H18" s="47" t="inlineStr">
+        <is>
+          <t>Incentive lief stattdessen über den Preis: 11,50 €/qm statt 12,50 €/qm in den ersten beiden Mietjahren (§7.2 i.d.F. 1. Nachtrag), seit 14.04.2023 ausgelaufen.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="B19" s="6" t="inlineStr">
@@ -1841,12 +1877,17 @@
       </c>
       <c r="C19" s="25" t="inlineStr">
         <is>
-          <t>VPI Deutschland, Basis 2010 = 100; bei Veränderung &gt;5 % Anpassung im vollen prozentualen Verhältnis (100 % Weitergabe); erstmals nach Ablauf des 4. Mietjahres, also ab 15.04.2025; Anpassung nach unten ausgeschlossen (§10, 3. Nachtrag Ziff. 10)</t>
+          <t>Anpassung um 100% der Indexveränderung, wenn Indexveränderung &gt;5% (VPI: Basis: 2010 = 100).</t>
         </is>
       </c>
       <c r="D19" s="26" t="n"/>
       <c r="E19" s="26" t="n"/>
       <c r="F19" s="26" t="n"/>
+      <c r="H19" s="47" t="inlineStr">
+        <is>
+          <t>Erstmals nach Ablauf des 4. Mietjahres, also ab 15.04.2025; Anpassung nach unten ausgeschlossen. Basisjahr wird bei Umstellung des VPI automatisch angepasst (§10.3).</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="B20" s="6" t="inlineStr">
@@ -1856,12 +1897,17 @@
       </c>
       <c r="C20" s="25" t="inlineStr">
         <is>
-          <t>Ja – Entfernung eingebrachter Einrichtungen, Rückbau aller Ein-/Umbauten und Wiederherstellung des ursprünglichen Zustands (§18.1); Trockenbauwände und Zusatzanschlüsse müssen nicht entfernt werden (§2.3.4)</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="D20" s="26" t="n"/>
       <c r="E20" s="26" t="n"/>
       <c r="F20" s="26" t="n"/>
+      <c r="H20" s="47" t="inlineStr">
+        <is>
+          <t>Entfernung eingebrachter Einrichtungen und Wiederherstellung des Ursprungszustands (§18.1); Trockenbauwände und Zusatzanschlüsse ausgenommen (§2.3.4).</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="B21" s="6" t="inlineStr">
@@ -1871,12 +1917,17 @@
       </c>
       <c r="C21" s="25" t="inlineStr">
         <is>
-          <t>Ja – generell gestattet im Rahmen des Mietzwecks, ausdrücklich einschließlich Untervermietung an Patienten (§17.1); zusätzlich Recht zur Ersatzmietergestellung (§17.2)</t>
+          <t>Ja, inkl. an Patienten</t>
         </is>
       </c>
       <c r="D21" s="26" t="n"/>
       <c r="E21" s="26" t="n"/>
       <c r="F21" s="26" t="n"/>
+      <c r="H21" s="47" t="inlineStr">
+        <is>
+          <t>Zusätzlich Recht zur Ersatzmietergestellung (§17.2).</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="65.25" customHeight="1">
       <c r="B22" s="6" t="inlineStr">
@@ -1886,12 +1937,17 @@
       </c>
       <c r="C22" s="50" t="inlineStr">
         <is>
-          <t>3 monatliche Gesamtzahlungen (Miete inkl. NK-Vorauszahlung) = 58.130,61 €; selbstschuldnerische, unbefristete, unwiderrufliche Bankbürgschaft (§14.3); nach 5 Jahren störungsfreier Mietzeit Reduzierung um eine Gesamtzahlung (1. Nachtrag)</t>
+          <t>Bankbürgschaft. Größenordnung: 3 Bruttomonatsmieten.</t>
         </is>
       </c>
       <c r="D22" s="51" t="n"/>
       <c r="E22" s="51" t="n"/>
       <c r="F22" s="51" t="n"/>
+      <c r="H22" s="47" t="inlineStr">
+        <is>
+          <t>Rechnerisch 58.130,61 € auf heutiger Basis. Gestellt wurde die Bürgschaft binnen 6 Monaten nach Vertragsschluss auf Basis von damals 12.428,50 € (= 37.285,50 €); eine Nachschusspflicht bei Flächenzuwachs enthalten die Verträge nicht. Tatsächliche Höhe beim Target erfragen. Nach 5 Jahren störungsfreier Mietzeit Reduzierung um eine Gesamtzahlung möglich.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="6" t="inlineStr">
@@ -1901,12 +1957,17 @@
       </c>
       <c r="C23" s="25" t="inlineStr">
         <is>
-          <t>Eingeschränkt – gewährt nur für den Betrieb eines Wohnheims mit Intensivpflege (§6.3), ausdrücklich nicht für andere medizinische Intensivpflege jedweder Ausrichtung (§6.4). Praktische Schutzwirkung fraglich.</t>
+          <t>eingeschränkt</t>
         </is>
       </c>
       <c r="D23" s="26" t="n"/>
       <c r="E23" s="26" t="n"/>
       <c r="F23" s="26" t="n"/>
+      <c r="H23" s="47" t="inlineStr">
+        <is>
+          <t>Nur für den Betrieb eines Wohnheims mit Intensivpflege (§6.3), ausdrücklich nicht für andere medizinische Intensivpflege jedweder Ausrichtung (§6.4). Praktische Schutzwirkung fraglich.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="B24" s="6" t="inlineStr">
@@ -1916,7 +1977,7 @@
       </c>
       <c r="C24" s="25" t="inlineStr">
         <is>
-          <t>Keines – ordentliche Kündigung während Festlaufzeit und Verlängerungszeiträumen ausgeschlossen (§5.4)</t>
+          <t>keines</t>
         </is>
       </c>
       <c r="D24" s="26" t="n"/>
@@ -1931,12 +1992,17 @@
       </c>
       <c r="C25" s="25" t="inlineStr">
         <is>
-          <t>Dach und Fach beim Vermieter; Mietfläche beim Mieter. Kleinreparaturen bis 300 €/Fall, p.a. gedeckelt auf eine Nettomonatsmiete (§12.8). Umlage der Instandhaltung gemeinschaftlicher Flächen auf 5 % der Jahresnettokaltmiete begrenzt (§11.3). Schönheitsreparaturen beim Mieter (§12.2).</t>
+          <t>Dach und Fach beim Vermieter; Fläche beim Mieter</t>
         </is>
       </c>
       <c r="D25" s="26" t="n"/>
       <c r="E25" s="26" t="n"/>
       <c r="F25" s="26" t="n"/>
+      <c r="H25" s="47" t="inlineStr">
+        <is>
+          <t>Kleinreparaturen bis 300 €/Fall, p.a. gedeckelt auf eine Nettomonatsmiete (§12.8). Umlage der Instandhaltung gemeinschaftlicher Flächen auf 5% der Jahresnettokaltmiete begrenzt (§11.3). Schönheitsreparaturen beim Mieter.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="6" t="inlineStr">
@@ -1946,12 +2012,17 @@
       </c>
       <c r="C26" s="25" t="inlineStr">
         <is>
-          <t>Vertragsstand = Hauptvertrag 05.02.2018 + 1.–3. Nachtrag. ACHTUNG Baukostenzuschuss verdeckt: Die 600,00 €/Monat für die statischen Mehraufwendungen im 1. OG (3. Nachtrag Ziff. 3) sind laufende Miete, nicht einmalig – über die Restlaufzeit wirtschaftlich ein amortisierter Baukostenzuschuss von rd. 54.000 €. OFFEN: Nebenkosten verstehen sich zzgl. USt (§11.6), während die Miete umsatzsteuerfrei ist (§9, keine Option). Ob die ausgewiesene Gesamtmiete von 19.376,87 € die USt auf die NK-Vorauszahlung bereits enthält, geht aus den Verträgen nicht hervor (Differenz rd. 735 €/Monat). Anmietrecht für später frei werdende Flächen im Gebäude (§1.2). Reinigungspflicht Treppenhaus/Aufzug 2x wöchentlich (§12.1).</t>
+          <t>umsatzsteuerfrei; Nebenkosten zzgl. USt</t>
         </is>
       </c>
       <c r="D26" s="26" t="n"/>
       <c r="E26" s="26" t="n"/>
       <c r="F26" s="26" t="n"/>
+      <c r="H26" s="47" t="inlineStr">
+        <is>
+          <t>Vertragsstand = Hauptvertrag 05.02.2018 + 1.–3. Nachtrag. Verdeckter Baukostenzuschuss: die 600 €/Monat für die statischen Mehraufwendungen im 1. OG laufen dauerhaft mit der Miete (rd. 54.000 € bis Vertragsende). OFFEN: ob die ausgewiesenen 19.376,87 € die USt auf die NK-Vorauszahlung enthalten, geht aus den Verträgen nicht hervor (rd. 735 €/Monat). Anmietrecht für frei werdende Flächen (§1.2).</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="6.75" customHeight="1" thickBot="1">
       <c r="B27" s="7" t="n"/>
@@ -2295,12 +2366,17 @@
       </c>
       <c r="C55" s="27" t="inlineStr">
         <is>
-          <t>XXX – Bettenzahl im Vertrag nicht genannt</t>
+          <t>XXX</t>
         </is>
       </c>
       <c r="D55" s="26" t="n"/>
       <c r="E55" s="26" t="n"/>
       <c r="F55" s="26" t="n"/>
+      <c r="H55" s="47" t="inlineStr">
+        <is>
+          <t>Bettenzahl in keinem der vier Dokumente genannt – vom Target anzufordern.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="B56" s="6" t="inlineStr">
@@ -2562,12 +2638,17 @@
       </c>
       <c r="C73" s="27" t="inlineStr">
         <is>
-          <t>XXX – Skizze Anlage N 3-1 sieht 5 Bewohner-Apartments vor</t>
+          <t>XXX</t>
         </is>
       </c>
       <c r="D73" s="26" t="n"/>
       <c r="E73" s="26" t="n"/>
       <c r="F73" s="26" t="n"/>
+      <c r="H73" s="47" t="inlineStr">
+        <is>
+          <t>Skizze Anlage N 3-1 sieht 5 Bewohner-Apartments vor.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="B74" s="6" t="inlineStr">
@@ -2590,7 +2671,7 @@
       </c>
       <c r="C75" s="29" t="inlineStr">
         <is>
-          <t>15.10.2023 (1. OG + 3 Stellplätze) – Keller 70 qm bereits ab 15.04.2023</t>
+          <t>15.10.2023 (1. OG); Keller 70 qm ab 15.04.2023</t>
         </is>
       </c>
       <c r="D75" s="26" t="n"/>
@@ -2801,7 +2882,7 @@
       </c>
       <c r="C89" s="27" t="inlineStr">
         <is>
-          <t>WG / Nebenfläche</t>
+          <t>Nebenfläche</t>
         </is>
       </c>
       <c r="D89" s="26" t="n"/>
@@ -2816,12 +2897,17 @@
       </c>
       <c r="C90" s="27" t="inlineStr">
         <is>
-          <t>4. OG (laut 1. Nachtrag; alternativ 1. OG)</t>
+          <t>4. OG</t>
         </is>
       </c>
       <c r="D90" s="26" t="n"/>
       <c r="E90" s="26" t="n"/>
       <c r="F90" s="26" t="n"/>
+      <c r="H90" s="47" t="inlineStr">
+        <is>
+          <t>Laut 1. Nachtrag im 4. OG, alternativ im 1. OG. Läge sie im 1. OG, wäre sie im "kompletten 1. OG" des 3. Nachtrags enthalten und doppelt erfasst; die strikt additive Mietsumme spricht für das 4. OG.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="B91" s="6" t="inlineStr">
@@ -2829,10 +2915,8 @@
           <t>Kapazität (Anzahl Betten)</t>
         </is>
       </c>
-      <c r="C91" s="27" t="inlineStr">
-        <is>
-          <t>0 – OFFEN: Läge diese Fläche im 1. OG, wäre sie im "kompletten 1. OG" des 3. Nachtrags enthalten und doppelt erfasst. Die Mietsumme von 19.376,87 € ist strikt additiv, spricht also für das 4. OG.</t>
-        </is>
+      <c r="C91" s="27" t="n">
+        <v>0</v>
       </c>
       <c r="D91" s="26" t="n"/>
       <c r="E91" s="26" t="n"/>
@@ -3072,7 +3156,7 @@
       </c>
       <c r="C108" s="36" t="inlineStr">
         <is>
-          <t>XXX – nicht aus dem Mietvertrag ableitbar, aus Target-Unterlagen zu ergänzen</t>
+          <t>XXX</t>
         </is>
       </c>
       <c r="D108" s="37" t="n"/>
@@ -3351,7 +3435,7 @@
       </c>
       <c r="C130" s="36" t="inlineStr">
         <is>
-          <t>XXX – nicht aus dem Mietvertrag ableitbar, aus Target-Unterlagen zu ergänzen</t>
+          <t>XXX</t>
         </is>
       </c>
       <c r="D130" s="37" t="n"/>
@@ -3556,7 +3640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F142"/>
+  <dimension ref="B2:H142"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5"/>
   <cols>
     <col width="3.81640625" customWidth="1" style="2" min="1" max="1"/>
@@ -3596,6 +3680,11 @@
       <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
+      <c r="H6" s="47" t="inlineStr">
+        <is>
+          <t>Anmerkung / Quelle</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="6" t="inlineStr">
@@ -3620,12 +3709,17 @@
       </c>
       <c r="C8" s="25" t="inlineStr">
         <is>
-          <t>Jans &amp; Willems GbR, Pfarrer-Hecker-Str. 33, 41849 Wassenberg, vertreten durch Werner Jans</t>
+          <t>Jans &amp; Willems GbR</t>
         </is>
       </c>
       <c r="D8" s="26" t="n"/>
       <c r="E8" s="26" t="n"/>
       <c r="F8" s="26" t="n"/>
+      <c r="H8" s="47" t="inlineStr">
+        <is>
+          <t>Pfarrer-Hecker-Str. 33, 41849 Wassenberg, vertreten durch Werner Jans.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="B9" s="6" t="inlineStr">
@@ -3635,12 +3729,17 @@
       </c>
       <c r="C9" s="25" t="inlineStr">
         <is>
-          <t>365° Pflegezentrum Marianne Weiß GmbH, Alleestraße 68, 42853 Remscheid (opseo-Gruppe)</t>
+          <t>365° Pflegezentrum Marianne Weiß GmbH</t>
         </is>
       </c>
       <c r="D9" s="26" t="n"/>
       <c r="E9" s="26" t="n"/>
       <c r="F9" s="26" t="n"/>
+      <c r="H9" s="47" t="inlineStr">
+        <is>
+          <t>opseo-Gruppe; Sitz Alleestraße 68, 42853 Remscheid.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="B10" s="6" t="inlineStr">
@@ -3665,12 +3764,17 @@
       </c>
       <c r="C11" s="25" t="inlineStr">
         <is>
-          <t>XXX – im Vertrag nicht genannt</t>
+          <t>XXX</t>
         </is>
       </c>
       <c r="D11" s="26" t="n"/>
       <c r="E11" s="26" t="n"/>
       <c r="F11" s="26" t="n"/>
+      <c r="H11" s="47" t="inlineStr">
+        <is>
+          <t>Im Vertrag nicht genannt.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="B12" s="6" t="inlineStr">
@@ -3680,7 +3784,7 @@
       </c>
       <c r="C12" s="25" t="inlineStr">
         <is>
-          <t>Betrieb einer Pflegeeinrichtung zur außerklinischen Versorgung, insbesondere Beatmungs- und Intensivpflege; Nutzung als Intensivpflege-Wohngemeinschaft gem. Baugenehmigung (§1.1, §1.3)</t>
+          <t>Intensivpflege-WG</t>
         </is>
       </c>
       <c r="D12" s="26" t="n"/>
@@ -3695,12 +3799,17 @@
       </c>
       <c r="C13" s="25" t="inlineStr">
         <is>
-          <t>5 Jahre Kündigungsausschluss für beide Parteien (§2.2). ACHTUNG Widerspruch im Vertrag: §2.3 räumt das Optionsrecht erst "nach Ablauf der ersten zehn Mietjahre" ein und §4.1 vereinbart die Miete für zehn Jahre fest. Am Scan doppelt verifiziert – die Abweichung steht so im Dokument. Klärungsbedarf.</t>
+          <t>5 Jahre</t>
         </is>
       </c>
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="26" t="n"/>
+      <c r="H13" s="47" t="inlineStr">
+        <is>
+          <t>Kündigungsausschluss für beide Parteien (§2.2). WIDERSPRUCH: §2.3 räumt das Optionsrecht erst "nach Ablauf der ersten zehn Mietjahre" ein, §4.1 fixiert die Miete für zehn Jahre. Am Scan mit zwei OCR-Verfahren verifiziert – die Abweichung steht so im Dokument. Klärungsbedarf.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="6" t="inlineStr">
@@ -3710,12 +3819,17 @@
       </c>
       <c r="C14" s="25" t="inlineStr">
         <is>
-          <t>2x 5 Jahre (Verlängerungszeitraum 1 und 2); Ausübung schriftlich per Brief oder E-Mail spätestens 6 Monate vor Ablauf der Festlaufzeit bzw. des Verlängerungszeitraums 1 (§2.3). Danach unbestimmte Zeit mit 6-Monats-Kündigungsfrist.</t>
+          <t>2x 5 Jahre</t>
         </is>
       </c>
       <c r="D14" s="26" t="n"/>
       <c r="E14" s="26" t="n"/>
       <c r="F14" s="26" t="n"/>
+      <c r="H14" s="47" t="inlineStr">
+        <is>
+          <t>Ausübung schriftlich spätestens 6 Monate vor Ablauf (§2.3); danach unbestimmte Zeit mit 6-Monats-Kündigungsfrist.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="B15" s="6" t="inlineStr">
@@ -3725,12 +3839,17 @@
       </c>
       <c r="C15" s="25" t="inlineStr">
         <is>
-          <t>Monatserster des auf den Vollzug des Kaufvertrags folgenden Kalendermonats (§2.1) – XXX, Vollzugsdatum des Kaufvertrags Kuijpers v. 17.03.2023 zu bestätigen</t>
+          <t>Monatserster nach Vollzug des Kaufvertrags</t>
         </is>
       </c>
       <c r="D15" s="26" t="n"/>
       <c r="E15" s="26" t="n"/>
       <c r="F15" s="26" t="n"/>
+      <c r="H15" s="47" t="inlineStr">
+        <is>
+          <t>Vollzugsdatum des Kaufvertrags Kuijpers v. 17.03.2023 zu bestätigen.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="B16" s="6" t="inlineStr">
@@ -3740,12 +3859,17 @@
       </c>
       <c r="C16" s="25" t="inlineStr">
         <is>
-          <t>Übergabeanspruch erst nach Stellung der Sicherheit (§3.1); Übernahmepflicht am Übergabetag; geringfügige Mängel hindern die Übergabe nicht (§3.2). Keine Vertragsstrafe geregelt.</t>
+          <t>keine Vertragsstrafe</t>
         </is>
       </c>
       <c r="D16" s="26" t="n"/>
       <c r="E16" s="26" t="n"/>
       <c r="F16" s="26" t="n"/>
+      <c r="H16" s="47" t="inlineStr">
+        <is>
+          <t>Übergabeanspruch erst nach Stellung der Sicherheit (§3.1); geringfügige Mängel hindern die Übergabe nicht (§3.2).</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="B17" s="6" t="inlineStr">
@@ -3755,12 +3879,17 @@
       </c>
       <c r="C17" s="25" t="inlineStr">
         <is>
-          <t>Ja – der gesamte Mietvertrag steht unter der aufschiebenden Bedingung des Vollzugs des Kauf- und Übertragungsvertrags betreffend Kuijpers Ambulante Pflege GmbH und PWH GmbH &amp; Co. KG vom 17.03.2023</t>
+          <t>Vollzug Kaufvertrag Kuijpers</t>
         </is>
       </c>
       <c r="D17" s="26" t="n"/>
       <c r="E17" s="26" t="n"/>
       <c r="F17" s="26" t="n"/>
+      <c r="H17" s="47" t="inlineStr">
+        <is>
+          <t>Der gesamte Mietvertrag steht unter dieser aufschiebenden Bedingung (Kuijpers Ambulante Pflege GmbH / PWH GmbH &amp; Co. KG, Vertrag v. 17.03.2023).</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="B18" s="6" t="inlineStr">
@@ -3770,7 +3899,7 @@
       </c>
       <c r="C18" s="25" t="inlineStr">
         <is>
-          <t>Keine</t>
+          <t>keine</t>
         </is>
       </c>
       <c r="D18" s="26" t="n"/>
@@ -3785,12 +3914,17 @@
       </c>
       <c r="C19" s="25" t="inlineStr">
         <is>
-          <t>Keine Indexierung vereinbart – die Miete ist für den Zeitraum von zehn Jahren fest vereinbart (§4.1). Deutlicher Vorteil gegenüber Würselen.</t>
+          <t>keine; Miete 10 Jahre fest</t>
         </is>
       </c>
       <c r="D19" s="26" t="n"/>
       <c r="E19" s="26" t="n"/>
       <c r="F19" s="26" t="n"/>
+      <c r="H19" s="47" t="inlineStr">
+        <is>
+          <t>Deutlicher Vorteil gegenüber Würselen, das mit 100% der Indexveränderung ab &gt;5% indexiert ist.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="B20" s="6" t="inlineStr">
@@ -3800,12 +3934,17 @@
       </c>
       <c r="C20" s="25" t="inlineStr">
         <is>
-          <t>Keine – ausdrücklich klargestellt, dass gemäß Zustand bei Mietbeginn keine Rückbauverpflichtungen entstehen (§15.1). Der Vermieter kann die Übernahme von Um-/Einbauten gegen Zeitwertentschädigung verlangen (§8.1.1).</t>
+          <t>keine</t>
         </is>
       </c>
       <c r="D20" s="26" t="n"/>
       <c r="E20" s="26" t="n"/>
       <c r="F20" s="26" t="n"/>
+      <c r="H20" s="47" t="inlineStr">
+        <is>
+          <t>§15.1 stellt ausdrücklich klar, dass keine Rückbauverpflichtungen entstehen. Der Vermieter kann die Übernahme von Um-/Einbauten gegen Zeitwertentschädigung verlangen (§8.1.1).</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="B21" s="6" t="inlineStr">
@@ -3815,12 +3954,17 @@
       </c>
       <c r="C21" s="25" t="inlineStr">
         <is>
-          <t>Grundsätzlich zustimmungspflichtig; ohne Zustimmung zulässig an verbundene Unternehmen i.S.d. §§15 ff. AktG sowie die Untervermietung einzelner Räume an pflegebedürftige Bewohner (§6.1)</t>
+          <t>Ja, zustimmungspflichtig</t>
         </is>
       </c>
       <c r="D21" s="26" t="n"/>
       <c r="E21" s="26" t="n"/>
       <c r="F21" s="26" t="n"/>
+      <c r="H21" s="47" t="inlineStr">
+        <is>
+          <t>Ohne Zustimmung zulässig an verbundene Unternehmen i.S.d. §§15 ff. AktG sowie an pflegebedürftige Bewohner (§6.1).</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="65.25" customHeight="1">
       <c r="B22" s="6" t="inlineStr">
@@ -3830,12 +3974,17 @@
       </c>
       <c r="C22" s="50" t="inlineStr">
         <is>
-          <t>Patronatserklärung der Muttergesellschaft opseo Intensivpflege Holding B.V., beschränkt auf eine Jahreskaltmiete (= 102.000 €), zu stellen binnen 4 Wochen nach Unterzeichnung (§5.1). Austausch bei Gesellschafterwechsel möglich (§5.3).</t>
+          <t>Patronatserklärung. Größenordnung: 1 Jahreskaltmiete.</t>
         </is>
       </c>
       <c r="D22" s="51" t="n"/>
       <c r="E22" s="51" t="n"/>
       <c r="F22" s="51" t="n"/>
+      <c r="H22" s="47" t="inlineStr">
+        <is>
+          <t>Patronatserklärung der Muttergesellschaft opseo Intensivpflege Holding B.V. = 102.000 €, binnen 4 Wochen nach Unterzeichnung (§5.1); Austausch bei Gesellschafterwechsel möglich (§5.3).</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="6" t="inlineStr">
@@ -3845,7 +3994,7 @@
       </c>
       <c r="C23" s="25" t="inlineStr">
         <is>
-          <t>Nicht geregelt – kein Konkurrenzschutz vereinbart</t>
+          <t>nein</t>
         </is>
       </c>
       <c r="D23" s="26" t="n"/>
@@ -3860,12 +4009,17 @@
       </c>
       <c r="C24" s="25" t="inlineStr">
         <is>
-          <t>Ja – bei behördlicher Nutzungsuntersagung wegen des baulichen bzw. bau- und brandschutztechnischen Zustands, sofern der Vermieter sie nicht abwenden kann (§1.4)</t>
+          <t>Ja, bei Nutzungsuntersagung</t>
         </is>
       </c>
       <c r="D24" s="26" t="n"/>
       <c r="E24" s="26" t="n"/>
       <c r="F24" s="26" t="n"/>
+      <c r="H24" s="47" t="inlineStr">
+        <is>
+          <t>Bei behördlicher Nutzungsuntersagung wegen des baulichen bzw. bau- und brandschutztechnischen Zustands, sofern der Vermieter sie nicht abwenden kann (§1.4).</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="B25" s="6" t="inlineStr">
@@ -3875,12 +4029,17 @@
       </c>
       <c r="C25" s="25" t="inlineStr">
         <is>
-          <t>Dach und Fach beim Vermieter auf dessen Kosten (§7.1). Übrige Instandhaltung/Instandsetzung des Gebäudes inkl. technischer Anlagen veranlasst der Vermieter; Kosten werden über die Nebenkostenabrechnung umgelegt, begrenzt auf 5 % der jährlichen Nettokaltmiete (§7.2). Schönheitsreparaturen beim Mieter (§7.4).</t>
+          <t>Dach und Fach beim Vermieter; Fläche beim Mieter</t>
         </is>
       </c>
       <c r="D25" s="26" t="n"/>
       <c r="E25" s="26" t="n"/>
       <c r="F25" s="26" t="n"/>
+      <c r="H25" s="47" t="inlineStr">
+        <is>
+          <t>Übrige Instandhaltung veranlasst der Vermieter, Kosten umgelegt bis max. 5% der jährlichen Nettokaltmiete (§7.2). Schönheitsreparaturen beim Mieter.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="6" t="inlineStr">
@@ -3890,12 +4049,17 @@
       </c>
       <c r="C26" s="25" t="inlineStr">
         <is>
-          <t>RED FLAG: Schlussabnahmebescheinigung der Bauaufsicht liegt nicht vor; Nachtragsgenehmigung seit 02.02.2022 beantragt, noch nicht erteilt (§1.1) – in Verbindung mit dem Sonderkündigungsrecht aus §1.4 zu bewerten. Inventar vermieterseitig gestellt (§1.2). Eigener Stromliefervertrag, Abnahmepflicht für den PV-Strom vom Grundstück (§4.2.2). Eintritt in die bestehenden Untermietverträge mit den Patienten (§18). Verkehrssicherung und Winterdienst beim Mieter (§17). Keine USt auf die Miete (§4.1). EG-Wohnung nicht Mietgegenstand, Zugang über den Haupteingang (§9.3). Gerichtsstand Wassenberg (§21).</t>
+          <t>Schlussabnahme fehlt; Inventar vermieterseitig gestellt</t>
         </is>
       </c>
       <c r="D26" s="26" t="n"/>
       <c r="E26" s="26" t="n"/>
       <c r="F26" s="26" t="n"/>
+      <c r="H26" s="47" t="inlineStr">
+        <is>
+          <t>RED FLAG: Schlussabnahmebescheinigung liegt nicht vor, Nachtragsgenehmigung seit 02.02.2022 beantragt (§1.1) – zusammen mit dem Sonderkündigungsrecht aus §1.4 zu bewerten. Eigener Stromliefervertrag mit Abnahmepflicht für PV-Strom (§4.2.2). Eintritt in bestehende Untermietverträge (§18). Verkehrssicherung und Winterdienst beim Mieter (§17). Keine USt auf die Miete (§4.1). Gerichtsstand Wassenberg.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="6.75" customHeight="1" thickBot="1">
       <c r="B27" s="7" t="n"/>
@@ -4224,12 +4388,17 @@
       </c>
       <c r="C54" s="27" t="inlineStr">
         <is>
-          <t>Im Vertrag nicht spezifiziert; Abstellräume im Kellergeschoss ausdrücklich erfasst (§1.1). Die EG-Wohnung ist nicht Mietgegenstand (§9.3).</t>
+          <t>XXX</t>
         </is>
       </c>
       <c r="D54" s="26" t="n"/>
       <c r="E54" s="26" t="n"/>
       <c r="F54" s="26" t="n"/>
+      <c r="H54" s="47" t="inlineStr">
+        <is>
+          <t>Etagenlage im Vertrag nicht spezifiziert; Abstellräume im Kellergeschoss erfasst (§1.1). Die EG-Wohnung ist nicht Mietgegenstand (§9.3).</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="B55" s="6" t="inlineStr">
@@ -4243,6 +4412,11 @@
       <c r="D55" s="26" t="n"/>
       <c r="E55" s="26" t="n"/>
       <c r="F55" s="26" t="n"/>
+      <c r="H55" s="47" t="inlineStr">
+        <is>
+          <t>ca. 18 Patientenzimmer (§1.1); die NK-Kalkulation (250 €/Platz = 4.700 €) impliziert 18,8 Plätze.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="B56" s="6" t="inlineStr">
@@ -4265,7 +4439,7 @@
       </c>
       <c r="C57" s="29" t="inlineStr">
         <is>
-          <t>XXX – siehe Mietbeginn</t>
+          <t>XXX</t>
         </is>
       </c>
       <c r="D57" s="26" t="n"/>
@@ -4318,6 +4492,11 @@
       <c r="F60" s="13">
         <f>+E60*12</f>
         <v/>
+      </c>
+      <c r="H60" s="47" t="inlineStr">
+        <is>
+          <t>Pauschalmiete 8.500 € bzw. NK-Pauschale 4.700 €; die qm-Preise sind rechnerisch abgeleitet.</t>
+        </is>
       </c>
     </row>
     <row r="61">
@@ -4998,13 +5177,18 @@
       </c>
       <c r="C108" s="36" t="inlineStr">
         <is>
-          <t>Inventar (Einbauküchen, Pflegebetten, Vorhänge) vermieterseitig gestellt und im Mietzins enthalten (§1.2)</t>
+          <t>XXX</t>
         </is>
       </c>
       <c r="D108" s="37" t="n"/>
       <c r="E108" s="38" t="n"/>
       <c r="F108" s="33" t="n">
         <v>0</v>
+      </c>
+      <c r="H108" s="47" t="inlineStr">
+        <is>
+          <t>Inventar (Einbauküchen, Pflegebetten, Vorhänge) vermieterseitig gestellt und im Mietzins enthalten (§1.2).</t>
+        </is>
       </c>
     </row>
     <row r="109">
@@ -5277,7 +5461,7 @@
       </c>
       <c r="C130" s="36" t="inlineStr">
         <is>
-          <t>XXX – nicht aus dem Mietvertrag ableitbar, aus internen Unterlagen zu ergänzen</t>
+          <t>XXX</t>
         </is>
       </c>
       <c r="D130" s="37" t="n"/>

</xml_diff>

<commit_message>
Long Version: Baesweiler neben Wuerselen statt darunter
Wuerselen bleibt in C-F, Baesweiler spiegelt es in G-J unter der bereits
in G4 gesetzten Ueberschrift; die vier Kostenspalten Anzahl / EUR pro Einheit /
EUR pro Monat / EUR pro Jahr liegen damit deckungsgleich nebeneinander.
Getrennt durch eine durchgehende senkrechte Linie an der linken Kante von G.
Die Zeilenbeschriftungen in Spalte B gelten fuer beide Bloecke. Anmerkungen
beider Standorte in Spalte L gebuendelt, Spalte H dafuer geraeumt.
Formeln des rechten Blocks um vier Spalten mitverschoben.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018VKr7wEHLAW3yJNS7pxnAu
</commit_message>
<xml_diff>
--- a/mietkonditionen/Mietkonditionen_Vergleich_Wuerselen_Baesweiler.xlsx
+++ b/mietkonditionen/Mietkonditionen_Vergleich_Wuerselen_Baesweiler.xlsx
@@ -18,12 +18,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="165" formatCode="0&quot;qm&quot;"/>
     <numFmt numFmtId="166" formatCode="#,##0\ &quot;€&quot;;[Red]\-#,##0\ &quot;€&quot;"/>
     <numFmt numFmtId="167" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
-    <numFmt numFmtId="168" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -103,7 +102,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="26">
+  <borders count="33">
     <border>
       <left/>
       <right/>
@@ -404,16 +403,90 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="medium"/>
       <right/>
       <top/>
-      <bottom style="medium"/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="medium"/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium"/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium"/>
+      <right/>
+      <top style="thin">
+        <color theme="0" tint="-0.249946592608417"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.249946592608417"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium"/>
+      <right/>
+      <top style="thin">
+        <color theme="0" tint="-0.249946592608417"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium"/>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium"/>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium"/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0" tint="-0.249946592608417"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -585,21 +658,81 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="167" fontId="2" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="167" fontId="2" fillId="4" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="166" fontId="2" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="2" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="4" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="4" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="4" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="4" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="4" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1716,16 +1849,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I288"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B1:L142"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5"/>
   <cols>
-    <col width="3.81640625" customWidth="1" min="1" max="1"/>
-    <col width="44.26953125" customWidth="1" min="2" max="2"/>
-    <col width="66.453125" customWidth="1" min="3" max="3"/>
-    <col width="12.81640625" customWidth="1" min="4" max="4"/>
-    <col width="11.453125" customWidth="1" min="7" max="7"/>
-    <col width="11.453125" customWidth="1" min="8" max="8"/>
-    <col width="11.453125" customWidth="1" min="9" max="9"/>
+    <col width="3.81640625" customWidth="1" style="2" min="1" max="1"/>
+    <col width="44.26953125" customWidth="1" style="2" min="2" max="2"/>
+    <col width="66.453125" customWidth="1" style="2" min="3" max="3"/>
+    <col width="12.81640625" customWidth="1" style="2" min="4" max="6"/>
+    <col width="35" customWidth="1" style="57" min="7" max="7"/>
+    <col width="12.82" customWidth="1" style="2" min="8" max="8"/>
+    <col width="11.453125" customWidth="1" style="2" min="9" max="16384"/>
   </cols>
   <sheetData>
     <row r="1"/>
@@ -1735,30 +1868,37 @@
           <t>Übersicht Mietvertragskonditionen</t>
         </is>
       </c>
-    </row>
-    <row r="3"/>
+      <c r="G2" s="59" t="n"/>
+    </row>
+    <row r="3">
+      <c r="G3" s="59" t="n"/>
+    </row>
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Standort:</t>
         </is>
       </c>
-      <c r="C4" s="59" t="inlineStr">
+      <c r="C4" s="60" t="inlineStr">
         <is>
           <t>Würselen (Target)</t>
         </is>
       </c>
-      <c r="D4" s="60" t="n"/>
-      <c r="E4" s="60" t="n"/>
-      <c r="F4" s="61" t="n"/>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="D4" s="61" t="n"/>
+      <c r="E4" s="61" t="n"/>
+      <c r="F4" s="62" t="n"/>
+      <c r="G4" s="63" t="inlineStr">
         <is>
           <t>Baesweiler (Bestand)</t>
         </is>
       </c>
-      <c r="H4" s="3" t="n"/>
-    </row>
-    <row r="5"/>
+      <c r="H4" s="61" t="n"/>
+      <c r="I4" s="61" t="n"/>
+      <c r="J4" s="62" t="n"/>
+    </row>
+    <row r="5">
+      <c r="G5" s="59" t="n"/>
+    </row>
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
         <is>
@@ -1769,6 +1909,15 @@
       <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
+      <c r="G6" s="64" t="n"/>
+      <c r="H6" s="5" t="n"/>
+      <c r="I6" s="5" t="n"/>
+      <c r="J6" s="5" t="n"/>
+      <c r="L6" s="47" t="inlineStr">
+        <is>
+          <t>Anmerkung / Quelle</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="6" t="inlineStr">
@@ -1784,7 +1933,14 @@
       <c r="D7" s="26" t="n"/>
       <c r="E7" s="26" t="n"/>
       <c r="F7" s="26" t="n"/>
-      <c r="H7" s="47" t="n"/>
+      <c r="G7" s="65" t="inlineStr">
+        <is>
+          <t>Jans &amp; Willems GbR</t>
+        </is>
+      </c>
+      <c r="H7" s="26" t="n"/>
+      <c r="I7" s="26" t="n"/>
+      <c r="J7" s="26" t="n"/>
     </row>
     <row r="8">
       <c r="B8" s="6" t="inlineStr">
@@ -1800,6 +1956,19 @@
       <c r="D8" s="26" t="n"/>
       <c r="E8" s="26" t="n"/>
       <c r="F8" s="26" t="n"/>
+      <c r="G8" s="65" t="inlineStr">
+        <is>
+          <t>Jans &amp; Willems GbR</t>
+        </is>
+      </c>
+      <c r="H8" s="26" t="n"/>
+      <c r="I8" s="26" t="n"/>
+      <c r="J8" s="26" t="n"/>
+      <c r="L8" s="47" t="inlineStr">
+        <is>
+          <t>Baesweiler: Pfarrer-Hecker-Str. 33, 41849 Wassenberg, vertreten durch Werner Jans.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="B9" s="6" t="inlineStr">
@@ -1815,6 +1984,19 @@
       <c r="D9" s="26" t="n"/>
       <c r="E9" s="26" t="n"/>
       <c r="F9" s="26" t="n"/>
+      <c r="G9" s="65" t="inlineStr">
+        <is>
+          <t>365° Pflegezentrum Marianne Weiß GmbH</t>
+        </is>
+      </c>
+      <c r="H9" s="26" t="n"/>
+      <c r="I9" s="26" t="n"/>
+      <c r="J9" s="26" t="n"/>
+      <c r="L9" s="47" t="inlineStr">
+        <is>
+          <t>Baesweiler: opseo-Gruppe; Sitz Alleestraße 68, 42853 Remscheid.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="B10" s="6" t="inlineStr">
@@ -1830,6 +2012,14 @@
       <c r="D10" s="26" t="n"/>
       <c r="E10" s="26" t="n"/>
       <c r="F10" s="26" t="n"/>
+      <c r="G10" s="65" t="inlineStr">
+        <is>
+          <t>Lessingstr. 3, 52499 Baesweiler</t>
+        </is>
+      </c>
+      <c r="H10" s="26" t="n"/>
+      <c r="I10" s="26" t="n"/>
+      <c r="J10" s="26" t="n"/>
     </row>
     <row r="11">
       <c r="B11" s="6" t="inlineStr">
@@ -1845,7 +2035,19 @@
       <c r="D11" s="26" t="n"/>
       <c r="E11" s="26" t="n"/>
       <c r="F11" s="26" t="n"/>
-      <c r="H11" s="47" t="n"/>
+      <c r="G11" s="65" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H11" s="26" t="n"/>
+      <c r="I11" s="26" t="n"/>
+      <c r="J11" s="26" t="n"/>
+      <c r="L11" s="47" t="inlineStr">
+        <is>
+          <t>Baesweiler: Im Vertrag nicht genannt.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="B12" s="6" t="inlineStr">
@@ -1861,6 +2063,14 @@
       <c r="D12" s="26" t="n"/>
       <c r="E12" s="26" t="n"/>
       <c r="F12" s="26" t="n"/>
+      <c r="G12" s="65" t="inlineStr">
+        <is>
+          <t>Intensivpflege-WG</t>
+        </is>
+      </c>
+      <c r="H12" s="26" t="n"/>
+      <c r="I12" s="26" t="n"/>
+      <c r="J12" s="26" t="n"/>
     </row>
     <row r="13">
       <c r="B13" s="6" t="inlineStr">
@@ -1876,7 +2086,19 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="26" t="n"/>
-      <c r="H13" s="47" t="n"/>
+      <c r="G13" s="65" t="inlineStr">
+        <is>
+          <t>5 Jahre</t>
+        </is>
+      </c>
+      <c r="H13" s="26" t="n"/>
+      <c r="I13" s="26" t="n"/>
+      <c r="J13" s="26" t="n"/>
+      <c r="L13" s="47" t="inlineStr">
+        <is>
+          <t>Baesweiler: Kündigungsausschluss für beide Parteien (§2.2). WIDERSPRUCH: §2.3 räumt das Optionsrecht erst "nach Ablauf der ersten zehn Mietjahre" ein, §4.1 fixiert die Miete für zehn Jahre. Am Scan mit zwei OCR-Verfahren verifiziert – die Abweichung steht so im Dokument. Klärungsbedarf.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="29" customHeight="1">
       <c r="B14" s="6" t="inlineStr">
@@ -1893,7 +2115,19 @@
       <c r="D14" s="26" t="n"/>
       <c r="E14" s="26" t="n"/>
       <c r="F14" s="26" t="n"/>
-      <c r="H14" s="47" t="n"/>
+      <c r="G14" s="65" t="inlineStr">
+        <is>
+          <t>2x 5 Jahre</t>
+        </is>
+      </c>
+      <c r="H14" s="26" t="n"/>
+      <c r="I14" s="26" t="n"/>
+      <c r="J14" s="26" t="n"/>
+      <c r="L14" s="47" t="inlineStr">
+        <is>
+          <t>Baesweiler: Ausübung schriftlich spätestens 6 Monate vor Ablauf (§2.3); danach unbestimmte Zeit mit 6-Monats-Kündigungsfrist.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="B15" s="6" t="inlineStr">
@@ -1909,7 +2143,19 @@
       <c r="D15" s="26" t="n"/>
       <c r="E15" s="26" t="n"/>
       <c r="F15" s="26" t="n"/>
-      <c r="H15" s="47" t="n"/>
+      <c r="G15" s="65" t="inlineStr">
+        <is>
+          <t>Monatserster nach Vollzug des Kaufvertrags</t>
+        </is>
+      </c>
+      <c r="H15" s="26" t="n"/>
+      <c r="I15" s="26" t="n"/>
+      <c r="J15" s="26" t="n"/>
+      <c r="L15" s="47" t="inlineStr">
+        <is>
+          <t>Baesweiler: Vollzugsdatum des Kaufvertrags Kuijpers v. 17.03.2023 zu bestätigen.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="B16" s="6" t="inlineStr">
@@ -1925,6 +2171,19 @@
       <c r="D16" s="26" t="n"/>
       <c r="E16" s="26" t="n"/>
       <c r="F16" s="26" t="n"/>
+      <c r="G16" s="65" t="inlineStr">
+        <is>
+          <t>keine Vertragsstrafe</t>
+        </is>
+      </c>
+      <c r="H16" s="26" t="n"/>
+      <c r="I16" s="26" t="n"/>
+      <c r="J16" s="26" t="n"/>
+      <c r="L16" s="47" t="inlineStr">
+        <is>
+          <t>Baesweiler: Übergabeanspruch erst nach Stellung der Sicherheit (§3.1); geringfügige Mängel hindern die Übergabe nicht (§3.2).</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="29" customHeight="1">
       <c r="B17" s="6" t="inlineStr">
@@ -1940,7 +2199,19 @@
       <c r="D17" s="26" t="n"/>
       <c r="E17" s="26" t="n"/>
       <c r="F17" s="26" t="n"/>
-      <c r="H17" s="47" t="n"/>
+      <c r="G17" s="65" t="inlineStr">
+        <is>
+          <t>Vollzug Kaufvertrag Kuijpers</t>
+        </is>
+      </c>
+      <c r="H17" s="26" t="n"/>
+      <c r="I17" s="26" t="n"/>
+      <c r="J17" s="26" t="n"/>
+      <c r="L17" s="47" t="inlineStr">
+        <is>
+          <t>Baesweiler: Der gesamte Mietvertrag steht unter dieser aufschiebenden Bedingung (Kuijpers Ambulante Pflege GmbH / PWH GmbH &amp; Co. KG, Vertrag v. 17.03.2023).</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="B18" s="6" t="inlineStr">
@@ -1956,7 +2227,14 @@
       <c r="D18" s="26" t="n"/>
       <c r="E18" s="26" t="n"/>
       <c r="F18" s="26" t="n"/>
-      <c r="H18" s="47" t="n"/>
+      <c r="G18" s="65" t="inlineStr">
+        <is>
+          <t>keine</t>
+        </is>
+      </c>
+      <c r="H18" s="26" t="n"/>
+      <c r="I18" s="26" t="n"/>
+      <c r="J18" s="26" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="6" t="inlineStr">
@@ -1972,7 +2250,19 @@
       <c r="D19" s="26" t="n"/>
       <c r="E19" s="26" t="n"/>
       <c r="F19" s="26" t="n"/>
-      <c r="H19" s="47" t="n"/>
+      <c r="G19" s="65" t="inlineStr">
+        <is>
+          <t>keine; Miete 10 Jahre fest</t>
+        </is>
+      </c>
+      <c r="H19" s="26" t="n"/>
+      <c r="I19" s="26" t="n"/>
+      <c r="J19" s="26" t="n"/>
+      <c r="L19" s="47" t="inlineStr">
+        <is>
+          <t>Baesweiler: Deutlicher Vorteil gegenüber Würselen, das mit 100% der Indexveränderung ab &gt;5% indexiert ist.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="B20" s="6" t="inlineStr">
@@ -1988,7 +2278,19 @@
       <c r="D20" s="26" t="n"/>
       <c r="E20" s="26" t="n"/>
       <c r="F20" s="26" t="n"/>
-      <c r="H20" s="47" t="n"/>
+      <c r="G20" s="65" t="inlineStr">
+        <is>
+          <t>keine</t>
+        </is>
+      </c>
+      <c r="H20" s="26" t="n"/>
+      <c r="I20" s="26" t="n"/>
+      <c r="J20" s="26" t="n"/>
+      <c r="L20" s="47" t="inlineStr">
+        <is>
+          <t>Baesweiler: §15.1 stellt ausdrücklich klar, dass keine Rückbauverpflichtungen entstehen. Der Vermieter kann die Übernahme von Um-/Einbauten gegen Zeitwertentschädigung verlangen (§8.1.1).</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="B21" s="6" t="inlineStr">
@@ -2004,7 +2306,19 @@
       <c r="D21" s="26" t="n"/>
       <c r="E21" s="26" t="n"/>
       <c r="F21" s="26" t="n"/>
-      <c r="H21" s="47" t="n"/>
+      <c r="G21" s="65" t="inlineStr">
+        <is>
+          <t>Ja, zustimmungspflichtig</t>
+        </is>
+      </c>
+      <c r="H21" s="26" t="n"/>
+      <c r="I21" s="26" t="n"/>
+      <c r="J21" s="26" t="n"/>
+      <c r="L21" s="47" t="inlineStr">
+        <is>
+          <t>Baesweiler: Ohne Zustimmung zulässig an verbundene Unternehmen i.S.d. §§15 ff. AktG sowie an pflegebedürftige Bewohner (§6.1).</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="29.5" customHeight="1">
       <c r="B22" s="6" t="inlineStr">
@@ -2020,7 +2334,19 @@
       <c r="D22" s="52" t="n"/>
       <c r="E22" s="52" t="n"/>
       <c r="F22" s="52" t="n"/>
-      <c r="H22" s="47" t="n"/>
+      <c r="G22" s="66" t="inlineStr">
+        <is>
+          <t>Patronatserklärung. Größenordnung: 1 Jahreskaltmiete.</t>
+        </is>
+      </c>
+      <c r="H22" s="52" t="n"/>
+      <c r="I22" s="52" t="n"/>
+      <c r="J22" s="52" t="n"/>
+      <c r="L22" s="47" t="inlineStr">
+        <is>
+          <t>Baesweiler: Patronatserklärung der Muttergesellschaft opseo Intensivpflege Holding B.V. = 102.000 €, binnen 4 Wochen nach Unterzeichnung (§5.1); Austausch bei Gesellschafterwechsel möglich (§5.3).</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="6" t="inlineStr">
@@ -2036,7 +2362,14 @@
       <c r="D23" s="26" t="n"/>
       <c r="E23" s="26" t="n"/>
       <c r="F23" s="26" t="n"/>
-      <c r="H23" s="47" t="n"/>
+      <c r="G23" s="65" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="H23" s="26" t="n"/>
+      <c r="I23" s="26" t="n"/>
+      <c r="J23" s="26" t="n"/>
     </row>
     <row r="24">
       <c r="B24" s="6" t="inlineStr">
@@ -2052,6 +2385,19 @@
       <c r="D24" s="26" t="n"/>
       <c r="E24" s="26" t="n"/>
       <c r="F24" s="26" t="n"/>
+      <c r="G24" s="65" t="inlineStr">
+        <is>
+          <t>Ja, bei Nutzungsuntersagung</t>
+        </is>
+      </c>
+      <c r="H24" s="26" t="n"/>
+      <c r="I24" s="26" t="n"/>
+      <c r="J24" s="26" t="n"/>
+      <c r="L24" s="47" t="inlineStr">
+        <is>
+          <t>Baesweiler: Bei behördlicher Nutzungsuntersagung wegen des baulichen bzw. bau- und brandschutztechnischen Zustands, sofern der Vermieter sie nicht abwenden kann (§1.4).</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="B25" s="6" t="inlineStr">
@@ -2067,7 +2413,19 @@
       <c r="D25" s="26" t="n"/>
       <c r="E25" s="26" t="n"/>
       <c r="F25" s="26" t="n"/>
-      <c r="H25" s="47" t="n"/>
+      <c r="G25" s="65" t="inlineStr">
+        <is>
+          <t>Dach und Fach beim Vermieter; Fläche beim Mieter</t>
+        </is>
+      </c>
+      <c r="H25" s="26" t="n"/>
+      <c r="I25" s="26" t="n"/>
+      <c r="J25" s="26" t="n"/>
+      <c r="L25" s="47" t="inlineStr">
+        <is>
+          <t>Baesweiler: Übrige Instandhaltung veranlasst der Vermieter, Kosten umgelegt bis max. 5% der jährlichen Nettokaltmiete (§7.2). Schönheitsreparaturen beim Mieter.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="6" t="inlineStr">
@@ -2083,16 +2441,34 @@
       <c r="D26" s="26" t="n"/>
       <c r="E26" s="26" t="n"/>
       <c r="F26" s="26" t="n"/>
-      <c r="H26" s="47" t="n"/>
-    </row>
-    <row r="27" ht="6.75" customHeight="1">
+      <c r="G26" s="65" t="inlineStr">
+        <is>
+          <t>Schlussabnahme fehlt; Inventar vermieterseitig gestellt</t>
+        </is>
+      </c>
+      <c r="H26" s="26" t="n"/>
+      <c r="I26" s="26" t="n"/>
+      <c r="J26" s="26" t="n"/>
+      <c r="L26" s="47" t="inlineStr">
+        <is>
+          <t>Baesweiler: RED FLAG: Schlussabnahmebescheinigung liegt nicht vor, Nachtragsgenehmigung seit 02.02.2022 beantragt (§1.1) – zusammen mit dem Sonderkündigungsrecht aus §1.4 zu bewerten. Eigener Stromliefervertrag mit Abnahmepflicht für PV-Strom (§4.2.2). Eintritt in bestehende Untermietverträge (§18). Verkehrssicherung und Winterdienst beim Mieter (§17). Keine USt auf die Miete (§4.1). Gerichtsstand Wassenberg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="6.75" customHeight="1" thickBot="1">
       <c r="B27" s="7" t="n"/>
       <c r="C27" s="8" t="n"/>
       <c r="D27" s="7" t="n"/>
       <c r="E27" s="7" t="n"/>
       <c r="F27" s="7" t="n"/>
-    </row>
-    <row r="28"/>
+      <c r="G27" s="67" t="n"/>
+      <c r="H27" s="7" t="n"/>
+      <c r="I27" s="7" t="n"/>
+      <c r="J27" s="7" t="n"/>
+    </row>
+    <row r="28">
+      <c r="G28" s="59" t="n"/>
+    </row>
     <row r="29">
       <c r="B29" s="9" t="inlineStr">
         <is>
@@ -2103,6 +2479,10 @@
       <c r="D29" s="9" t="n"/>
       <c r="E29" s="9" t="n"/>
       <c r="F29" s="9" t="n"/>
+      <c r="G29" s="68" t="n"/>
+      <c r="H29" s="9" t="n"/>
+      <c r="I29" s="9" t="n"/>
+      <c r="J29" s="9" t="n"/>
     </row>
     <row r="30">
       <c r="B30" s="6" t="inlineStr">
@@ -2110,12 +2490,18 @@
           <t>Miete/m² (Neubau) - kein BKZ</t>
         </is>
       </c>
-      <c r="C30" s="62" t="n">
+      <c r="C30" s="69" t="n">
         <v>20</v>
       </c>
       <c r="D30" s="26" t="n"/>
       <c r="E30" s="26" t="n"/>
       <c r="F30" s="26" t="n"/>
+      <c r="G30" s="70" t="n">
+        <v>20</v>
+      </c>
+      <c r="H30" s="26" t="n"/>
+      <c r="I30" s="26" t="n"/>
+      <c r="J30" s="26" t="n"/>
     </row>
     <row r="31">
       <c r="B31" s="6" t="inlineStr">
@@ -2123,12 +2509,18 @@
           <t>Miete/m² inkl. BKZ</t>
         </is>
       </c>
-      <c r="C31" s="62" t="n">
+      <c r="C31" s="69" t="n">
         <v>20</v>
       </c>
       <c r="D31" s="26" t="n"/>
       <c r="E31" s="26" t="n"/>
       <c r="F31" s="26" t="n"/>
+      <c r="G31" s="70" t="n">
+        <v>20</v>
+      </c>
+      <c r="H31" s="26" t="n"/>
+      <c r="I31" s="26" t="n"/>
+      <c r="J31" s="26" t="n"/>
     </row>
     <row r="32">
       <c r="B32" s="6" t="inlineStr">
@@ -2136,12 +2528,18 @@
           <t>Nebenkosten/m²</t>
         </is>
       </c>
-      <c r="C32" s="62" t="n">
+      <c r="C32" s="69" t="n">
         <v>3</v>
       </c>
       <c r="D32" s="26" t="n"/>
       <c r="E32" s="26" t="n"/>
       <c r="F32" s="26" t="n"/>
+      <c r="G32" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="H32" s="26" t="n"/>
+      <c r="I32" s="26" t="n"/>
+      <c r="J32" s="26" t="n"/>
     </row>
     <row r="33">
       <c r="B33" s="6" t="inlineStr">
@@ -2149,18 +2547,30 @@
           <t>Fläche pro Bett</t>
         </is>
       </c>
-      <c r="C33" s="63" t="inlineStr">
+      <c r="C33" s="71" t="inlineStr">
         <is>
           <t>50m²</t>
         </is>
       </c>
-      <c r="D33" s="64" t="inlineStr">
+      <c r="D33" s="72" t="inlineStr">
         <is>
           <t xml:space="preserve"> (d.h. 6er WG: 300m²; 12er WG: 600m²)</t>
         </is>
       </c>
       <c r="E33" s="26" t="n"/>
       <c r="F33" s="26" t="n"/>
+      <c r="G33" s="73" t="inlineStr">
+        <is>
+          <t>50m²</t>
+        </is>
+      </c>
+      <c r="H33" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (d.h. 6er WG: 300m²; 12er WG: 600m²)</t>
+        </is>
+      </c>
+      <c r="I33" s="26" t="n"/>
+      <c r="J33" s="26" t="n"/>
     </row>
     <row r="34">
       <c r="B34" s="6" t="inlineStr">
@@ -2168,12 +2578,18 @@
           <t>Miete pro Bett pro Monat (exkl. Baukostenzuschuss)</t>
         </is>
       </c>
-      <c r="C34" s="63" t="n">
+      <c r="C34" s="71" t="n">
         <v>1000</v>
       </c>
       <c r="D34" s="26" t="n"/>
       <c r="E34" s="26" t="n"/>
       <c r="F34" s="26" t="n"/>
+      <c r="G34" s="73" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H34" s="26" t="n"/>
+      <c r="I34" s="26" t="n"/>
+      <c r="J34" s="26" t="n"/>
     </row>
     <row r="35">
       <c r="B35" s="6" t="inlineStr">
@@ -2181,13 +2597,20 @@
           <t>Miete pro Bett pro Monat (inkl. BKZ über 10 Jahre)</t>
         </is>
       </c>
-      <c r="C35" s="63">
+      <c r="C35" s="71">
         <f>+C34</f>
         <v/>
       </c>
       <c r="D35" s="26" t="n"/>
       <c r="E35" s="26" t="n"/>
       <c r="F35" s="26" t="n"/>
+      <c r="G35" s="73">
+        <f>+G34</f>
+        <v/>
+      </c>
+      <c r="H35" s="26" t="n"/>
+      <c r="I35" s="26" t="n"/>
+      <c r="J35" s="26" t="n"/>
     </row>
     <row r="36">
       <c r="B36" s="6" t="inlineStr">
@@ -2195,12 +2618,18 @@
           <t>Baukostenzuschuss pro Bett</t>
         </is>
       </c>
-      <c r="C36" s="63" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" s="64" t="n"/>
+      <c r="C36" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="72" t="n"/>
       <c r="E36" s="26" t="n"/>
       <c r="F36" s="26" t="n"/>
+      <c r="G36" s="73" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="72" t="n"/>
+      <c r="I36" s="26" t="n"/>
+      <c r="J36" s="26" t="n"/>
     </row>
     <row r="37">
       <c r="B37" s="6" t="inlineStr">
@@ -2208,12 +2637,18 @@
           <t>Capex pro Bett (Möbel, Ausstattung, etc.)</t>
         </is>
       </c>
-      <c r="C37" s="63" t="n">
+      <c r="C37" s="71" t="n">
         <v>30000</v>
       </c>
       <c r="D37" s="26" t="n"/>
       <c r="E37" s="26" t="n"/>
       <c r="F37" s="26" t="n"/>
+      <c r="G37" s="73" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H37" s="26" t="n"/>
+      <c r="I37" s="26" t="n"/>
+      <c r="J37" s="26" t="n"/>
     </row>
     <row r="38">
       <c r="B38" s="6" t="inlineStr">
@@ -2229,8 +2664,18 @@
       <c r="D38" s="26" t="n"/>
       <c r="E38" s="26" t="n"/>
       <c r="F38" s="26" t="n"/>
-    </row>
-    <row r="39"/>
+      <c r="G38" s="65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H38" s="26" t="n"/>
+      <c r="I38" s="26" t="n"/>
+      <c r="J38" s="26" t="n"/>
+    </row>
+    <row r="39">
+      <c r="G39" s="59" t="n"/>
+    </row>
     <row r="40">
       <c r="B40" s="9" t="inlineStr">
         <is>
@@ -2241,6 +2686,10 @@
       <c r="D40" s="9" t="n"/>
       <c r="E40" s="9" t="n"/>
       <c r="F40" s="9" t="n"/>
+      <c r="G40" s="68" t="n"/>
+      <c r="H40" s="9" t="n"/>
+      <c r="I40" s="9" t="n"/>
+      <c r="J40" s="9" t="n"/>
     </row>
     <row r="41">
       <c r="B41" s="6" t="inlineStr">
@@ -2248,12 +2697,18 @@
           <t>Miete/m² (Bestand) - kein BKZ</t>
         </is>
       </c>
-      <c r="C41" s="62" t="n">
+      <c r="C41" s="69" t="n">
         <v>20</v>
       </c>
       <c r="D41" s="26" t="n"/>
       <c r="E41" s="26" t="n"/>
       <c r="F41" s="26" t="n"/>
+      <c r="G41" s="70" t="n">
+        <v>20</v>
+      </c>
+      <c r="H41" s="26" t="n"/>
+      <c r="I41" s="26" t="n"/>
+      <c r="J41" s="26" t="n"/>
     </row>
     <row r="42">
       <c r="B42" s="6" t="inlineStr">
@@ -2261,12 +2716,18 @@
           <t>Miete/m² (Bestand) inkl. BKZ</t>
         </is>
       </c>
-      <c r="C42" s="62" t="n">
+      <c r="C42" s="69" t="n">
         <v>25</v>
       </c>
       <c r="D42" s="26" t="n"/>
       <c r="E42" s="26" t="n"/>
       <c r="F42" s="26" t="n"/>
+      <c r="G42" s="70" t="n">
+        <v>25</v>
+      </c>
+      <c r="H42" s="26" t="n"/>
+      <c r="I42" s="26" t="n"/>
+      <c r="J42" s="26" t="n"/>
     </row>
     <row r="43">
       <c r="B43" s="6" t="inlineStr">
@@ -2274,12 +2735,18 @@
           <t>Nebenkosten/m²</t>
         </is>
       </c>
-      <c r="C43" s="62" t="n">
+      <c r="C43" s="69" t="n">
         <v>3</v>
       </c>
       <c r="D43" s="26" t="n"/>
       <c r="E43" s="26" t="n"/>
       <c r="F43" s="26" t="n"/>
+      <c r="G43" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="H43" s="26" t="n"/>
+      <c r="I43" s="26" t="n"/>
+      <c r="J43" s="26" t="n"/>
     </row>
     <row r="44">
       <c r="B44" s="6" t="inlineStr">
@@ -2287,18 +2754,30 @@
           <t>Fläche pro Bett</t>
         </is>
       </c>
-      <c r="C44" s="63" t="inlineStr">
+      <c r="C44" s="71" t="inlineStr">
         <is>
           <t>50m²</t>
         </is>
       </c>
-      <c r="D44" s="64" t="inlineStr">
+      <c r="D44" s="72" t="inlineStr">
         <is>
           <t xml:space="preserve"> (d.h. 6er WG: 300m²; 12er WG: 600m²)</t>
         </is>
       </c>
       <c r="E44" s="26" t="n"/>
       <c r="F44" s="26" t="n"/>
+      <c r="G44" s="73" t="inlineStr">
+        <is>
+          <t>50m²</t>
+        </is>
+      </c>
+      <c r="H44" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> (d.h. 6er WG: 300m²; 12er WG: 600m²)</t>
+        </is>
+      </c>
+      <c r="I44" s="26" t="n"/>
+      <c r="J44" s="26" t="n"/>
     </row>
     <row r="45">
       <c r="B45" s="6" t="inlineStr">
@@ -2306,12 +2785,18 @@
           <t>Miete pro Bett pro Monat (exkl. Baukostenzuschuss)</t>
         </is>
       </c>
-      <c r="C45" s="63" t="n">
+      <c r="C45" s="71" t="n">
         <v>1000</v>
       </c>
       <c r="D45" s="26" t="n"/>
       <c r="E45" s="26" t="n"/>
       <c r="F45" s="26" t="n"/>
+      <c r="G45" s="73" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H45" s="26" t="n"/>
+      <c r="I45" s="26" t="n"/>
+      <c r="J45" s="26" t="n"/>
     </row>
     <row r="46">
       <c r="B46" s="6" t="inlineStr">
@@ -2319,12 +2804,18 @@
           <t>Miete pro Bett pro Monat (inkl. BKZ über 10 Jahre)</t>
         </is>
       </c>
-      <c r="C46" s="63" t="n">
+      <c r="C46" s="71" t="n">
         <v>1250</v>
       </c>
       <c r="D46" s="26" t="n"/>
       <c r="E46" s="26" t="n"/>
       <c r="F46" s="26" t="n"/>
+      <c r="G46" s="73" t="n">
+        <v>1250</v>
+      </c>
+      <c r="H46" s="26" t="n"/>
+      <c r="I46" s="26" t="n"/>
+      <c r="J46" s="26" t="n"/>
     </row>
     <row r="47">
       <c r="B47" s="6" t="inlineStr">
@@ -2332,16 +2823,26 @@
           <t>Baukostenzuschuss pro Bett</t>
         </is>
       </c>
-      <c r="C47" s="63" t="n">
+      <c r="C47" s="71" t="n">
         <v>40000</v>
       </c>
-      <c r="D47" s="64" t="inlineStr">
+      <c r="D47" s="72" t="inlineStr">
         <is>
           <t>(d.h. 6er WG: 180.000 €, 12er WG: 360.000 €)</t>
         </is>
       </c>
       <c r="E47" s="26" t="n"/>
       <c r="F47" s="26" t="n"/>
+      <c r="G47" s="73" t="n">
+        <v>40000</v>
+      </c>
+      <c r="H47" s="72" t="inlineStr">
+        <is>
+          <t>(d.h. 6er WG: 180.000 €, 12er WG: 360.000 €)</t>
+        </is>
+      </c>
+      <c r="I47" s="26" t="n"/>
+      <c r="J47" s="26" t="n"/>
     </row>
     <row r="48">
       <c r="B48" s="6" t="inlineStr">
@@ -2349,12 +2850,18 @@
           <t>Capex pro Bett (Möbel, Ausstattung, etc.)</t>
         </is>
       </c>
-      <c r="C48" s="63" t="n">
+      <c r="C48" s="71" t="n">
         <v>30000</v>
       </c>
       <c r="D48" s="26" t="n"/>
       <c r="E48" s="26" t="n"/>
       <c r="F48" s="26" t="n"/>
+      <c r="G48" s="73" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H48" s="26" t="n"/>
+      <c r="I48" s="26" t="n"/>
+      <c r="J48" s="26" t="n"/>
     </row>
     <row r="49">
       <c r="B49" s="6" t="inlineStr">
@@ -2368,8 +2875,16 @@
       <c r="D49" s="26" t="n"/>
       <c r="E49" s="26" t="n"/>
       <c r="F49" s="26" t="n"/>
-    </row>
-    <row r="50"/>
+      <c r="G49" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="26" t="n"/>
+      <c r="I49" s="26" t="n"/>
+      <c r="J49" s="26" t="n"/>
+    </row>
+    <row r="50">
+      <c r="G50" s="59" t="n"/>
+    </row>
     <row r="51">
       <c r="B51" s="9" t="inlineStr">
         <is>
@@ -2380,6 +2895,10 @@
       <c r="D51" s="9" t="n"/>
       <c r="E51" s="9" t="n"/>
       <c r="F51" s="9" t="n"/>
+      <c r="G51" s="68" t="n"/>
+      <c r="H51" s="9" t="n"/>
+      <c r="I51" s="9" t="n"/>
+      <c r="J51" s="9" t="n"/>
     </row>
     <row r="52">
       <c r="B52" s="10" t="inlineStr">
@@ -2391,6 +2910,10 @@
       <c r="D52" s="10" t="n"/>
       <c r="E52" s="10" t="n"/>
       <c r="F52" s="10" t="n"/>
+      <c r="G52" s="75" t="n"/>
+      <c r="H52" s="10" t="n"/>
+      <c r="I52" s="10" t="n"/>
+      <c r="J52" s="10" t="n"/>
     </row>
     <row r="53">
       <c r="B53" s="6" t="inlineStr">
@@ -2406,6 +2929,14 @@
       <c r="D53" s="26" t="n"/>
       <c r="E53" s="26" t="n"/>
       <c r="F53" s="26" t="n"/>
+      <c r="G53" s="74" t="inlineStr">
+        <is>
+          <t>WG (Intensivpflege-Wohngemeinschaft)</t>
+        </is>
+      </c>
+      <c r="H53" s="26" t="n"/>
+      <c r="I53" s="26" t="n"/>
+      <c r="J53" s="26" t="n"/>
     </row>
     <row r="54">
       <c r="B54" s="6" t="inlineStr">
@@ -2421,6 +2952,19 @@
       <c r="D54" s="26" t="n"/>
       <c r="E54" s="26" t="n"/>
       <c r="F54" s="26" t="n"/>
+      <c r="G54" s="74" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H54" s="26" t="n"/>
+      <c r="I54" s="26" t="n"/>
+      <c r="J54" s="26" t="n"/>
+      <c r="L54" s="47" t="inlineStr">
+        <is>
+          <t>Baesweiler: Etagenlage im Vertrag nicht spezifiziert; Abstellräume im Kellergeschoss erfasst (§1.1). Die EG-Wohnung ist nicht Mietgegenstand (§9.3).</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="B55" s="6" t="inlineStr">
@@ -2436,9 +2980,15 @@
       <c r="D55" s="26" t="n"/>
       <c r="E55" s="26" t="n"/>
       <c r="F55" s="26" t="n"/>
-      <c r="H55" s="47" t="inlineStr">
-        <is>
-          <t>Bettenzahl in keinem der vier Dokumente genannt – vom Target anzufordern.</t>
+      <c r="G55" s="74" t="n">
+        <v>18</v>
+      </c>
+      <c r="H55" s="26" t="n"/>
+      <c r="I55" s="26" t="n"/>
+      <c r="J55" s="26" t="n"/>
+      <c r="L55" s="47" t="inlineStr">
+        <is>
+          <t>Würselen: Bettenzahl in keinem der vier Dokumente genannt – vom Target anzufordern.  |  Baesweiler: ca. 18 Patientenzimmer (§1.1); die NK-Kalkulation (250 €/Platz = 4.700 €) impliziert 18,8 Plätze.</t>
         </is>
       </c>
     </row>
@@ -2454,6 +3004,12 @@
       <c r="D56" s="26" t="n"/>
       <c r="E56" s="26" t="n"/>
       <c r="F56" s="26" t="n"/>
+      <c r="G56" s="76" t="n">
+        <v>1082</v>
+      </c>
+      <c r="H56" s="26" t="n"/>
+      <c r="I56" s="26" t="n"/>
+      <c r="J56" s="26" t="n"/>
     </row>
     <row r="57">
       <c r="B57" s="6" t="inlineStr">
@@ -2467,8 +3023,18 @@
       <c r="D57" s="26" t="n"/>
       <c r="E57" s="26" t="n"/>
       <c r="F57" s="26" t="n"/>
-    </row>
-    <row r="58"/>
+      <c r="G57" s="77" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H57" s="26" t="n"/>
+      <c r="I57" s="26" t="n"/>
+      <c r="J57" s="26" t="n"/>
+    </row>
+    <row r="58">
+      <c r="G58" s="59" t="n"/>
+    </row>
     <row r="59">
       <c r="B59" s="11" t="inlineStr">
         <is>
@@ -2495,6 +3061,26 @@
           <t>€ pro Jahr</t>
         </is>
       </c>
+      <c r="G59" s="78" t="inlineStr">
+        <is>
+          <t>Anzahl</t>
+        </is>
+      </c>
+      <c r="H59" s="12" t="inlineStr">
+        <is>
+          <t>€ pro Einheit</t>
+        </is>
+      </c>
+      <c r="I59" s="12" t="inlineStr">
+        <is>
+          <t>€ pro Monat</t>
+        </is>
+      </c>
+      <c r="J59" s="12" t="inlineStr">
+        <is>
+          <t>€ pro Jahr</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="B60" s="2" t="inlineStr">
@@ -2516,6 +3102,25 @@
         <f>+E60*12</f>
         <v/>
       </c>
+      <c r="G60" s="79" t="n">
+        <v>1082</v>
+      </c>
+      <c r="H60" s="31" t="n">
+        <v>7.855822550831793</v>
+      </c>
+      <c r="I60" s="13">
+        <f>+G60*H60</f>
+        <v/>
+      </c>
+      <c r="J60" s="13">
+        <f>+I60*12</f>
+        <v/>
+      </c>
+      <c r="L60" s="47" t="inlineStr">
+        <is>
+          <t>Baesweiler: Pauschalmiete 8.500 € bzw. NK-Pauschale 4.700 €; die qm-Preise sind rechnerisch abgeleitet.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="B61" s="6" t="inlineStr">
@@ -2538,6 +3143,21 @@
         <f>+E61*12</f>
         <v/>
       </c>
+      <c r="G61" s="80">
+        <f>+G60</f>
+        <v/>
+      </c>
+      <c r="H61" s="33" t="n">
+        <v>4.343807763401109</v>
+      </c>
+      <c r="I61" s="13">
+        <f>+G61*H61</f>
+        <v/>
+      </c>
+      <c r="J61" s="13">
+        <f>+I61*12</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="B62" s="6" t="inlineStr">
@@ -2559,6 +3179,20 @@
         <f>+E62*12</f>
         <v/>
       </c>
+      <c r="G62" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I62" s="13">
+        <f>+G62*H62</f>
+        <v/>
+      </c>
+      <c r="J62" s="13">
+        <f>+I62*12</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="B63" s="6" t="inlineStr">
@@ -2580,6 +3214,20 @@
         <f>+E63*12</f>
         <v/>
       </c>
+      <c r="G63" s="80" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" s="13">
+        <f>+G63*H63</f>
+        <v/>
+      </c>
+      <c r="J63" s="13">
+        <f>+I63*12</f>
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="B64" s="6" t="inlineStr">
@@ -2601,6 +3249,20 @@
         <f>+E64*12</f>
         <v/>
       </c>
+      <c r="G64" s="80" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I64" s="13">
+        <f>+G64*H64</f>
+        <v/>
+      </c>
+      <c r="J64" s="13">
+        <f>+I64*12</f>
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="B65" s="6" t="inlineStr">
@@ -2620,6 +3282,20 @@
       </c>
       <c r="F65" s="13">
         <f>+E65*12</f>
+        <v/>
+      </c>
+      <c r="G65" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I65" s="13">
+        <f>+G65*H65</f>
+        <v/>
+      </c>
+      <c r="J65" s="13">
+        <f>+I65*12</f>
         <v/>
       </c>
     </row>
@@ -2629,8 +3305,12 @@
       <c r="D66" s="16" t="n"/>
       <c r="E66" s="17" t="n"/>
       <c r="F66" s="17" t="n"/>
-    </row>
-    <row r="67">
+      <c r="G66" s="82" t="n"/>
+      <c r="H66" s="16" t="n"/>
+      <c r="I66" s="17" t="n"/>
+      <c r="J66" s="17" t="n"/>
+    </row>
+    <row r="67" customFormat="1" s="1">
       <c r="B67" s="1" t="inlineStr">
         <is>
           <t>Summe</t>
@@ -2646,16 +3326,31 @@
         <f>+SUM(F60:F66)</f>
         <v/>
       </c>
-      <c r="G67" s="58" t="n"/>
-    </row>
-    <row r="68" ht="6.75" customHeight="1">
+      <c r="G67" s="83" t="n"/>
+      <c r="H67" s="19" t="n"/>
+      <c r="I67" s="20">
+        <f>+SUM(I60:I66)</f>
+        <v/>
+      </c>
+      <c r="J67" s="20">
+        <f>+SUM(J60:J66)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68" ht="6.75" customHeight="1" thickBot="1">
       <c r="B68" s="7" t="n"/>
       <c r="C68" s="8" t="n"/>
       <c r="D68" s="7" t="n"/>
       <c r="E68" s="7" t="n"/>
       <c r="F68" s="7" t="n"/>
-    </row>
-    <row r="69"/>
+      <c r="G68" s="67" t="n"/>
+      <c r="H68" s="7" t="n"/>
+      <c r="I68" s="7" t="n"/>
+      <c r="J68" s="7" t="n"/>
+    </row>
+    <row r="69">
+      <c r="G69" s="59" t="n"/>
+    </row>
     <row r="70">
       <c r="B70" s="10" t="inlineStr">
         <is>
@@ -2666,6 +3361,10 @@
       <c r="D70" s="10" t="n"/>
       <c r="E70" s="10" t="n"/>
       <c r="F70" s="10" t="n"/>
+      <c r="G70" s="75" t="n"/>
+      <c r="H70" s="10" t="n"/>
+      <c r="I70" s="10" t="n"/>
+      <c r="J70" s="10" t="n"/>
     </row>
     <row r="71">
       <c r="B71" s="6" t="inlineStr">
@@ -2681,6 +3380,14 @@
       <c r="D71" s="26" t="n"/>
       <c r="E71" s="26" t="n"/>
       <c r="F71" s="26" t="n"/>
+      <c r="G71" s="74" t="inlineStr">
+        <is>
+          <t>entfällt</t>
+        </is>
+      </c>
+      <c r="H71" s="26" t="n"/>
+      <c r="I71" s="26" t="n"/>
+      <c r="J71" s="26" t="n"/>
     </row>
     <row r="72">
       <c r="B72" s="6" t="inlineStr">
@@ -2696,6 +3403,10 @@
       <c r="D72" s="26" t="n"/>
       <c r="E72" s="26" t="n"/>
       <c r="F72" s="26" t="n"/>
+      <c r="G72" s="74" t="n"/>
+      <c r="H72" s="26" t="n"/>
+      <c r="I72" s="26" t="n"/>
+      <c r="J72" s="26" t="n"/>
     </row>
     <row r="73">
       <c r="B73" s="6" t="inlineStr">
@@ -2711,9 +3422,15 @@
       <c r="D73" s="26" t="n"/>
       <c r="E73" s="26" t="n"/>
       <c r="F73" s="26" t="n"/>
-      <c r="H73" s="47" t="inlineStr">
-        <is>
-          <t>Skizze Anlage N 3-1 sieht 5 Bewohner-Apartments vor.</t>
+      <c r="G73" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" s="26" t="n"/>
+      <c r="I73" s="26" t="n"/>
+      <c r="J73" s="26" t="n"/>
+      <c r="L73" s="47" t="inlineStr">
+        <is>
+          <t>Würselen: Skizze Anlage N 3-1 sieht 5 Bewohner-Apartments vor.</t>
         </is>
       </c>
     </row>
@@ -2729,6 +3446,12 @@
       <c r="D74" s="26" t="n"/>
       <c r="E74" s="26" t="n"/>
       <c r="F74" s="26" t="n"/>
+      <c r="G74" s="76" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" s="26" t="n"/>
+      <c r="I74" s="26" t="n"/>
+      <c r="J74" s="26" t="n"/>
     </row>
     <row r="75">
       <c r="B75" s="6" t="inlineStr">
@@ -2744,8 +3467,14 @@
       <c r="D75" s="26" t="n"/>
       <c r="E75" s="26" t="n"/>
       <c r="F75" s="26" t="n"/>
-    </row>
-    <row r="76"/>
+      <c r="G75" s="77" t="n"/>
+      <c r="H75" s="26" t="n"/>
+      <c r="I75" s="26" t="n"/>
+      <c r="J75" s="26" t="n"/>
+    </row>
+    <row r="76">
+      <c r="G76" s="59" t="n"/>
+    </row>
     <row r="77">
       <c r="B77" s="11" t="inlineStr">
         <is>
@@ -2772,6 +3501,26 @@
           <t>€ pro Jahr</t>
         </is>
       </c>
+      <c r="G77" s="78" t="inlineStr">
+        <is>
+          <t>Anzahl</t>
+        </is>
+      </c>
+      <c r="H77" s="12" t="inlineStr">
+        <is>
+          <t>€ pro Einheit</t>
+        </is>
+      </c>
+      <c r="I77" s="12" t="inlineStr">
+        <is>
+          <t>€ pro Monat</t>
+        </is>
+      </c>
+      <c r="J77" s="12" t="inlineStr">
+        <is>
+          <t>€ pro Jahr</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="B78" s="2" t="inlineStr">
@@ -2793,6 +3542,20 @@
         <f>+E78*12</f>
         <v/>
       </c>
+      <c r="G78" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="I78" s="13">
+        <f>+G78*H78</f>
+        <v/>
+      </c>
+      <c r="J78" s="13">
+        <f>+I78*12</f>
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="B79" s="6" t="inlineStr">
@@ -2815,6 +3578,21 @@
         <f>+E79*12</f>
         <v/>
       </c>
+      <c r="G79" s="80">
+        <f>+G78</f>
+        <v/>
+      </c>
+      <c r="H79" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I79" s="13">
+        <f>+G79*H79</f>
+        <v/>
+      </c>
+      <c r="J79" s="13">
+        <f>+I79*12</f>
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="B80" s="6" t="inlineStr">
@@ -2836,6 +3614,20 @@
         <f>+E80*12</f>
         <v/>
       </c>
+      <c r="G80" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="H80" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I80" s="13">
+        <f>+G80*H80</f>
+        <v/>
+      </c>
+      <c r="J80" s="13">
+        <f>+I80*12</f>
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="B81" s="6" t="inlineStr">
@@ -2857,6 +3649,20 @@
         <f>+E81*12</f>
         <v/>
       </c>
+      <c r="G81" s="80" t="n">
+        <v>0</v>
+      </c>
+      <c r="H81" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I81" s="13">
+        <f>+G81*H81</f>
+        <v/>
+      </c>
+      <c r="J81" s="13">
+        <f>+I81*12</f>
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="B82" s="6" t="inlineStr">
@@ -2878,6 +3684,20 @@
         <f>+E82*12</f>
         <v/>
       </c>
+      <c r="G82" s="80" t="n">
+        <v>0</v>
+      </c>
+      <c r="H82" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I82" s="13">
+        <f>+G82*H82</f>
+        <v/>
+      </c>
+      <c r="J82" s="13">
+        <f>+I82*12</f>
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="B83" s="6" t="inlineStr">
@@ -2897,6 +3717,20 @@
       </c>
       <c r="F83" s="13">
         <f>+E83*12</f>
+        <v/>
+      </c>
+      <c r="G83" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I83" s="13">
+        <f>+G83*H83</f>
+        <v/>
+      </c>
+      <c r="J83" s="13">
+        <f>+I83*12</f>
         <v/>
       </c>
     </row>
@@ -2906,8 +3740,12 @@
       <c r="D84" s="16" t="n"/>
       <c r="E84" s="17" t="n"/>
       <c r="F84" s="17" t="n"/>
-    </row>
-    <row r="85">
+      <c r="G84" s="82" t="n"/>
+      <c r="H84" s="16" t="n"/>
+      <c r="I84" s="17" t="n"/>
+      <c r="J84" s="17" t="n"/>
+    </row>
+    <row r="85" customFormat="1" s="1">
       <c r="B85" s="1" t="inlineStr">
         <is>
           <t>Summe</t>
@@ -2923,16 +3761,31 @@
         <f>+SUM(F78:F84)</f>
         <v/>
       </c>
-      <c r="G85" s="58" t="n"/>
-    </row>
-    <row r="86" ht="6.75" customHeight="1">
+      <c r="G85" s="83" t="n"/>
+      <c r="H85" s="19" t="n"/>
+      <c r="I85" s="20">
+        <f>+SUM(I78:I84)</f>
+        <v/>
+      </c>
+      <c r="J85" s="20">
+        <f>+SUM(J78:J84)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86" ht="6.75" customHeight="1" thickBot="1">
       <c r="B86" s="7" t="n"/>
       <c r="C86" s="8" t="n"/>
       <c r="D86" s="7" t="n"/>
       <c r="E86" s="7" t="n"/>
       <c r="F86" s="7" t="n"/>
-    </row>
-    <row r="87"/>
+      <c r="G86" s="67" t="n"/>
+      <c r="H86" s="7" t="n"/>
+      <c r="I86" s="7" t="n"/>
+      <c r="J86" s="7" t="n"/>
+    </row>
+    <row r="87">
+      <c r="G87" s="59" t="n"/>
+    </row>
     <row r="88">
       <c r="B88" s="10" t="inlineStr">
         <is>
@@ -2943,6 +3796,10 @@
       <c r="D88" s="10" t="n"/>
       <c r="E88" s="10" t="n"/>
       <c r="F88" s="10" t="n"/>
+      <c r="G88" s="75" t="n"/>
+      <c r="H88" s="10" t="n"/>
+      <c r="I88" s="10" t="n"/>
+      <c r="J88" s="10" t="n"/>
     </row>
     <row r="89">
       <c r="B89" s="6" t="inlineStr">
@@ -2958,6 +3815,14 @@
       <c r="D89" s="26" t="n"/>
       <c r="E89" s="26" t="n"/>
       <c r="F89" s="26" t="n"/>
+      <c r="G89" s="74" t="inlineStr">
+        <is>
+          <t>entfällt</t>
+        </is>
+      </c>
+      <c r="H89" s="26" t="n"/>
+      <c r="I89" s="26" t="n"/>
+      <c r="J89" s="26" t="n"/>
     </row>
     <row r="90">
       <c r="B90" s="6" t="inlineStr">
@@ -2973,9 +3838,13 @@
       <c r="D90" s="26" t="n"/>
       <c r="E90" s="26" t="n"/>
       <c r="F90" s="26" t="n"/>
-      <c r="H90" s="47" t="inlineStr">
-        <is>
-          <t>Laut 1. Nachtrag im 4. OG, alternativ im 1. OG. Läge sie im 1. OG, wäre sie im "kompletten 1. OG" des 3. Nachtrags enthalten und doppelt erfasst; die strikt additive Mietsumme spricht für das 4. OG.</t>
+      <c r="G90" s="74" t="n"/>
+      <c r="H90" s="26" t="n"/>
+      <c r="I90" s="26" t="n"/>
+      <c r="J90" s="26" t="n"/>
+      <c r="L90" s="47" t="inlineStr">
+        <is>
+          <t>Würselen: Laut 1. Nachtrag im 4. OG, alternativ im 1. OG. Läge sie im 1. OG, wäre sie im "kompletten 1. OG" des 3. Nachtrags enthalten und doppelt erfasst; die strikt additive Mietsumme spricht für das 4. OG.</t>
         </is>
       </c>
     </row>
@@ -2991,6 +3860,12 @@
       <c r="D91" s="26" t="n"/>
       <c r="E91" s="26" t="n"/>
       <c r="F91" s="26" t="n"/>
+      <c r="G91" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="H91" s="26" t="n"/>
+      <c r="I91" s="26" t="n"/>
+      <c r="J91" s="26" t="n"/>
     </row>
     <row r="92">
       <c r="B92" s="6" t="inlineStr">
@@ -3004,6 +3879,12 @@
       <c r="D92" s="26" t="n"/>
       <c r="E92" s="26" t="n"/>
       <c r="F92" s="26" t="n"/>
+      <c r="G92" s="76" t="n">
+        <v>0</v>
+      </c>
+      <c r="H92" s="26" t="n"/>
+      <c r="I92" s="26" t="n"/>
+      <c r="J92" s="26" t="n"/>
     </row>
     <row r="93">
       <c r="B93" s="6" t="inlineStr">
@@ -3017,8 +3898,14 @@
       <c r="D93" s="26" t="n"/>
       <c r="E93" s="26" t="n"/>
       <c r="F93" s="26" t="n"/>
-    </row>
-    <row r="94"/>
+      <c r="G93" s="77" t="n"/>
+      <c r="H93" s="26" t="n"/>
+      <c r="I93" s="26" t="n"/>
+      <c r="J93" s="26" t="n"/>
+    </row>
+    <row r="94">
+      <c r="G94" s="59" t="n"/>
+    </row>
     <row r="95">
       <c r="B95" s="11" t="inlineStr">
         <is>
@@ -3045,6 +3932,26 @@
           <t>€ pro Jahr</t>
         </is>
       </c>
+      <c r="G95" s="78" t="inlineStr">
+        <is>
+          <t>Anzahl</t>
+        </is>
+      </c>
+      <c r="H95" s="12" t="inlineStr">
+        <is>
+          <t>€ pro Einheit</t>
+        </is>
+      </c>
+      <c r="I95" s="12" t="inlineStr">
+        <is>
+          <t>€ pro Monat</t>
+        </is>
+      </c>
+      <c r="J95" s="12" t="inlineStr">
+        <is>
+          <t>€ pro Jahr</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="B96" s="2" t="inlineStr">
@@ -3066,6 +3973,20 @@
         <f>+E96*12</f>
         <v/>
       </c>
+      <c r="G96" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="H96" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="I96" s="13">
+        <f>+G96*H96</f>
+        <v/>
+      </c>
+      <c r="J96" s="13">
+        <f>+I96*12</f>
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="B97" s="6" t="inlineStr">
@@ -3088,6 +4009,21 @@
         <f>+E97*12</f>
         <v/>
       </c>
+      <c r="G97" s="80">
+        <f>+G96</f>
+        <v/>
+      </c>
+      <c r="H97" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I97" s="13">
+        <f>+G97*H97</f>
+        <v/>
+      </c>
+      <c r="J97" s="13">
+        <f>+I97*12</f>
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="B98" s="6" t="inlineStr">
@@ -3109,6 +4045,20 @@
         <f>+E98*12</f>
         <v/>
       </c>
+      <c r="G98" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="H98" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I98" s="13">
+        <f>+G98*H98</f>
+        <v/>
+      </c>
+      <c r="J98" s="13">
+        <f>+I98*12</f>
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="B99" s="6" t="inlineStr">
@@ -3130,6 +4080,20 @@
         <f>+E99*12</f>
         <v/>
       </c>
+      <c r="G99" s="80" t="n">
+        <v>0</v>
+      </c>
+      <c r="H99" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I99" s="13">
+        <f>+G99*H99</f>
+        <v/>
+      </c>
+      <c r="J99" s="13">
+        <f>+I99*12</f>
+        <v/>
+      </c>
     </row>
     <row r="100">
       <c r="B100" s="6" t="inlineStr">
@@ -3151,6 +4115,20 @@
         <f>+E100*12</f>
         <v/>
       </c>
+      <c r="G100" s="80" t="n">
+        <v>0</v>
+      </c>
+      <c r="H100" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I100" s="13">
+        <f>+G100*H100</f>
+        <v/>
+      </c>
+      <c r="J100" s="13">
+        <f>+I100*12</f>
+        <v/>
+      </c>
     </row>
     <row r="101">
       <c r="B101" s="6" t="inlineStr">
@@ -3170,6 +4148,20 @@
       </c>
       <c r="F101" s="13">
         <f>+E101*12</f>
+        <v/>
+      </c>
+      <c r="G101" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="H101" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I101" s="13">
+        <f>+G101*H101</f>
+        <v/>
+      </c>
+      <c r="J101" s="13">
+        <f>+I101*12</f>
         <v/>
       </c>
     </row>
@@ -3179,8 +4171,12 @@
       <c r="D102" s="16" t="n"/>
       <c r="E102" s="17" t="n"/>
       <c r="F102" s="17" t="n"/>
-    </row>
-    <row r="103">
+      <c r="G102" s="82" t="n"/>
+      <c r="H102" s="16" t="n"/>
+      <c r="I102" s="17" t="n"/>
+      <c r="J102" s="17" t="n"/>
+    </row>
+    <row r="103" customFormat="1" s="1">
       <c r="B103" s="1" t="inlineStr">
         <is>
           <t>Summe</t>
@@ -3196,17 +4192,34 @@
         <f>+SUM(F96:F102)</f>
         <v/>
       </c>
-      <c r="G103" s="58" t="n"/>
-    </row>
-    <row r="104" ht="6.75" customHeight="1">
+      <c r="G103" s="83" t="n"/>
+      <c r="H103" s="19" t="n"/>
+      <c r="I103" s="20">
+        <f>+SUM(I96:I102)</f>
+        <v/>
+      </c>
+      <c r="J103" s="20">
+        <f>+SUM(J96:J102)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104" ht="6.75" customHeight="1" thickBot="1">
       <c r="B104" s="7" t="n"/>
       <c r="C104" s="8" t="n"/>
       <c r="D104" s="7" t="n"/>
       <c r="E104" s="7" t="n"/>
       <c r="F104" s="7" t="n"/>
-    </row>
-    <row r="105"/>
-    <row r="106"/>
+      <c r="G104" s="67" t="n"/>
+      <c r="H104" s="7" t="n"/>
+      <c r="I104" s="7" t="n"/>
+      <c r="J104" s="7" t="n"/>
+    </row>
+    <row r="105">
+      <c r="G105" s="59" t="n"/>
+    </row>
+    <row r="106">
+      <c r="G106" s="59" t="n"/>
+    </row>
     <row r="107">
       <c r="B107" s="23" t="inlineStr">
         <is>
@@ -3221,6 +4234,14 @@
       <c r="D107" s="24" t="n"/>
       <c r="E107" s="24" t="n"/>
       <c r="F107" s="24" t="n"/>
+      <c r="G107" s="84" t="inlineStr">
+        <is>
+          <t>Anmerkungen</t>
+        </is>
+      </c>
+      <c r="H107" s="24" t="n"/>
+      <c r="I107" s="24" t="n"/>
+      <c r="J107" s="24" t="n"/>
     </row>
     <row r="108">
       <c r="B108" s="35" t="inlineStr">
@@ -3238,6 +4259,21 @@
       <c r="F108" s="56" t="n">
         <v>0</v>
       </c>
+      <c r="G108" s="85" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H108" s="37" t="n"/>
+      <c r="I108" s="38" t="n"/>
+      <c r="J108" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L108" s="47" t="inlineStr">
+        <is>
+          <t>Baesweiler: Inventar (Einbauküchen, Pflegebetten, Vorhänge) vermieterseitig gestellt und im Mietzins enthalten (§1.2).</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="B109" s="35" t="inlineStr">
@@ -3255,6 +4291,16 @@
       <c r="F109" s="56" t="n">
         <v>0</v>
       </c>
+      <c r="G109" s="65" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H109" s="39" t="n"/>
+      <c r="I109" s="40" t="n"/>
+      <c r="J109" s="33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="110">
       <c r="B110" s="35" t="inlineStr">
@@ -3272,6 +4318,16 @@
       <c r="F110" s="56" t="n">
         <v>0</v>
       </c>
+      <c r="G110" s="65" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H110" s="39" t="n"/>
+      <c r="I110" s="40" t="n"/>
+      <c r="J110" s="33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="111">
       <c r="B111" s="35" t="inlineStr">
@@ -3289,6 +4345,16 @@
       <c r="F111" s="56" t="n">
         <v>0</v>
       </c>
+      <c r="G111" s="65" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H111" s="39" t="n"/>
+      <c r="I111" s="40" t="n"/>
+      <c r="J111" s="33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="112">
       <c r="B112" s="35" t="inlineStr">
@@ -3306,6 +4372,16 @@
       <c r="F112" s="56" t="n">
         <v>0</v>
       </c>
+      <c r="G112" s="65" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H112" s="39" t="n"/>
+      <c r="I112" s="40" t="n"/>
+      <c r="J112" s="33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="113">
       <c r="B113" s="35" t="inlineStr">
@@ -3323,6 +4399,16 @@
       <c r="F113" s="56" t="n">
         <v>0</v>
       </c>
+      <c r="G113" s="65" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H113" s="39" t="n"/>
+      <c r="I113" s="40" t="n"/>
+      <c r="J113" s="33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="114">
       <c r="B114" s="35" t="inlineStr">
@@ -3340,6 +4426,16 @@
       <c r="F114" s="56" t="n">
         <v>0</v>
       </c>
+      <c r="G114" s="65" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H114" s="39" t="n"/>
+      <c r="I114" s="40" t="n"/>
+      <c r="J114" s="33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="115">
       <c r="B115" s="35" t="inlineStr">
@@ -3357,6 +4453,16 @@
       <c r="F115" s="56" t="n">
         <v>0</v>
       </c>
+      <c r="G115" s="65" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H115" s="39" t="n"/>
+      <c r="I115" s="40" t="n"/>
+      <c r="J115" s="33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="116">
       <c r="B116" s="35" t="inlineStr">
@@ -3374,6 +4480,16 @@
       <c r="F116" s="56" t="n">
         <v>0</v>
       </c>
+      <c r="G116" s="65" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H116" s="39" t="n"/>
+      <c r="I116" s="40" t="n"/>
+      <c r="J116" s="33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="117">
       <c r="B117" s="35" t="inlineStr">
@@ -3391,6 +4507,16 @@
       <c r="F117" s="56" t="n">
         <v>0</v>
       </c>
+      <c r="G117" s="65" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H117" s="39" t="n"/>
+      <c r="I117" s="40" t="n"/>
+      <c r="J117" s="33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="118">
       <c r="B118" s="35" t="inlineStr">
@@ -3406,6 +4532,16 @@
       <c r="D118" s="39" t="n"/>
       <c r="E118" s="40" t="n"/>
       <c r="F118" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G118" s="65" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H118" s="39" t="n"/>
+      <c r="I118" s="40" t="n"/>
+      <c r="J118" s="33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3415,8 +4551,12 @@
       <c r="D119" s="16" t="n"/>
       <c r="E119" s="17" t="n"/>
       <c r="F119" s="17" t="n"/>
-    </row>
-    <row r="120">
+      <c r="G119" s="82" t="n"/>
+      <c r="H119" s="16" t="n"/>
+      <c r="I119" s="17" t="n"/>
+      <c r="J119" s="17" t="n"/>
+    </row>
+    <row r="120" customFormat="1" s="1">
       <c r="B120" s="1" t="inlineStr">
         <is>
           <t>Summe</t>
@@ -3429,22 +4569,35 @@
         <f>+SUM(F108:F119)</f>
         <v/>
       </c>
-      <c r="G120" s="58" t="n"/>
-    </row>
-    <row r="121" ht="6.75" customHeight="1">
+      <c r="G120" s="83" t="n"/>
+      <c r="H120" s="19" t="n"/>
+      <c r="I120" s="20" t="n"/>
+      <c r="J120" s="20">
+        <f>+SUM(J108:J119)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="121" ht="6.75" customHeight="1" thickBot="1">
       <c r="B121" s="7" t="n"/>
       <c r="C121" s="8" t="n"/>
       <c r="D121" s="7" t="n"/>
       <c r="E121" s="7" t="n"/>
       <c r="F121" s="7" t="n"/>
-    </row>
-    <row r="122" ht="6.75" customHeight="1"/>
+      <c r="G121" s="67" t="n"/>
+      <c r="H121" s="7" t="n"/>
+      <c r="I121" s="7" t="n"/>
+      <c r="J121" s="7" t="n"/>
+    </row>
+    <row r="122" ht="6.75" customHeight="1">
+      <c r="G122" s="59" t="n"/>
+    </row>
     <row r="123">
       <c r="B123" s="21" t="inlineStr">
         <is>
           <t>davon:</t>
         </is>
       </c>
+      <c r="G123" s="59" t="n"/>
     </row>
     <row r="124">
       <c r="B124" s="22" t="inlineStr">
@@ -3462,6 +4615,16 @@
       <c r="F124" s="56" t="n">
         <v>0</v>
       </c>
+      <c r="G124" s="65" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H124" s="39" t="n"/>
+      <c r="I124" s="40" t="n"/>
+      <c r="J124" s="33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="125">
       <c r="B125" s="22" t="inlineStr">
@@ -3479,16 +4642,34 @@
       <c r="F125" s="56" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="126" ht="6.75" customHeight="1">
+      <c r="G125" s="65" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H125" s="39" t="n"/>
+      <c r="I125" s="40" t="n"/>
+      <c r="J125" s="33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126" ht="6.75" customHeight="1" thickBot="1">
       <c r="B126" s="7" t="n"/>
       <c r="C126" s="8" t="n"/>
       <c r="D126" s="7" t="n"/>
       <c r="E126" s="7" t="n"/>
       <c r="F126" s="7" t="n"/>
-    </row>
-    <row r="127"/>
-    <row r="128"/>
+      <c r="G126" s="67" t="n"/>
+      <c r="H126" s="7" t="n"/>
+      <c r="I126" s="7" t="n"/>
+      <c r="J126" s="7" t="n"/>
+    </row>
+    <row r="127">
+      <c r="G127" s="59" t="n"/>
+    </row>
+    <row r="128">
+      <c r="G128" s="59" t="n"/>
+    </row>
     <row r="129">
       <c r="B129" s="23" t="inlineStr">
         <is>
@@ -3503,6 +4684,14 @@
       <c r="D129" s="24" t="n"/>
       <c r="E129" s="24" t="n"/>
       <c r="F129" s="24" t="n"/>
+      <c r="G129" s="84" t="inlineStr">
+        <is>
+          <t>Anmerkungen</t>
+        </is>
+      </c>
+      <c r="H129" s="24" t="n"/>
+      <c r="I129" s="24" t="n"/>
+      <c r="J129" s="24" t="n"/>
     </row>
     <row r="130">
       <c r="B130" s="35" t="inlineStr">
@@ -3520,6 +4709,16 @@
       <c r="F130" s="56" t="n">
         <v>0</v>
       </c>
+      <c r="G130" s="85" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H130" s="37" t="n"/>
+      <c r="I130" s="38" t="n"/>
+      <c r="J130" s="33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="131">
       <c r="B131" s="35" t="inlineStr">
@@ -3537,6 +4736,16 @@
       <c r="F131" s="56" t="n">
         <v>0</v>
       </c>
+      <c r="G131" s="65" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H131" s="39" t="n"/>
+      <c r="I131" s="40" t="n"/>
+      <c r="J131" s="33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="132">
       <c r="B132" s="35" t="inlineStr">
@@ -3554,6 +4763,16 @@
       <c r="F132" s="56" t="n">
         <v>0</v>
       </c>
+      <c r="G132" s="65" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H132" s="39" t="n"/>
+      <c r="I132" s="40" t="n"/>
+      <c r="J132" s="33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="133">
       <c r="B133" s="35" t="inlineStr">
@@ -3571,6 +4790,16 @@
       <c r="F133" s="56" t="n">
         <v>0</v>
       </c>
+      <c r="G133" s="65" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H133" s="39" t="n"/>
+      <c r="I133" s="40" t="n"/>
+      <c r="J133" s="33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="134">
       <c r="B134" s="35" t="inlineStr">
@@ -3588,6 +4817,16 @@
       <c r="F134" s="56" t="n">
         <v>0</v>
       </c>
+      <c r="G134" s="65" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H134" s="39" t="n"/>
+      <c r="I134" s="40" t="n"/>
+      <c r="J134" s="33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="135">
       <c r="B135" s="35" t="inlineStr">
@@ -3605,6 +4844,16 @@
       <c r="F135" s="56" t="n">
         <v>0</v>
       </c>
+      <c r="G135" s="65" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H135" s="39" t="n"/>
+      <c r="I135" s="40" t="n"/>
+      <c r="J135" s="33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="136">
       <c r="B136" s="35" t="inlineStr">
@@ -3622,6 +4871,16 @@
       <c r="F136" s="56" t="n">
         <v>0</v>
       </c>
+      <c r="G136" s="65" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H136" s="39" t="n"/>
+      <c r="I136" s="40" t="n"/>
+      <c r="J136" s="33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="137">
       <c r="B137" s="35" t="inlineStr">
@@ -3639,6 +4898,16 @@
       <c r="F137" s="56" t="n">
         <v>0</v>
       </c>
+      <c r="G137" s="65" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H137" s="39" t="n"/>
+      <c r="I137" s="40" t="n"/>
+      <c r="J137" s="33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="138">
       <c r="B138" s="35" t="inlineStr">
@@ -3656,6 +4925,16 @@
       <c r="F138" s="56" t="n">
         <v>0</v>
       </c>
+      <c r="G138" s="65" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H138" s="39" t="n"/>
+      <c r="I138" s="40" t="n"/>
+      <c r="J138" s="33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="139">
       <c r="B139" s="35" t="inlineStr">
@@ -3671,6 +4950,16 @@
       <c r="D139" s="39" t="n"/>
       <c r="E139" s="40" t="n"/>
       <c r="F139" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G139" s="65" t="inlineStr">
+        <is>
+          <t>XXX</t>
+        </is>
+      </c>
+      <c r="H139" s="39" t="n"/>
+      <c r="I139" s="40" t="n"/>
+      <c r="J139" s="33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3680,8 +4969,12 @@
       <c r="D140" s="16" t="n"/>
       <c r="E140" s="17" t="n"/>
       <c r="F140" s="17" t="n"/>
-    </row>
-    <row r="141">
+      <c r="G140" s="82" t="n"/>
+      <c r="H140" s="16" t="n"/>
+      <c r="I140" s="17" t="n"/>
+      <c r="J140" s="17" t="n"/>
+    </row>
+    <row r="141" customFormat="1" s="1">
       <c r="B141" s="1" t="inlineStr">
         <is>
           <t>Summe</t>
@@ -3694,2043 +4987,33 @@
         <f>+SUM(F130:F140)</f>
         <v/>
       </c>
-      <c r="G141" s="58" t="n"/>
-    </row>
-    <row r="142" ht="6.75" customHeight="1">
+      <c r="G141" s="83" t="n"/>
+      <c r="H141" s="19" t="n"/>
+      <c r="I141" s="20" t="n"/>
+      <c r="J141" s="20">
+        <f>+SUM(J130:J140)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="142" ht="6.75" customHeight="1" thickBot="1">
       <c r="B142" s="7" t="n"/>
       <c r="C142" s="8" t="n"/>
       <c r="D142" s="7" t="n"/>
       <c r="E142" s="7" t="n"/>
       <c r="F142" s="7" t="n"/>
-    </row>
-    <row r="145">
-      <c r="B145" s="65" t="n"/>
-      <c r="C145" s="65" t="n"/>
-      <c r="D145" s="65" t="n"/>
-      <c r="E145" s="65" t="n"/>
-      <c r="F145" s="65" t="n"/>
-    </row>
-    <row r="147"/>
-    <row r="148">
-      <c r="B148" s="1" t="inlineStr">
-        <is>
-          <t>Übersicht Mietvertragskonditionen</t>
-        </is>
-      </c>
-    </row>
-    <row r="149"/>
-    <row r="150">
-      <c r="B150" s="3" t="inlineStr">
-        <is>
-          <t>Standort:</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>Baesweiler (Bestand)</t>
-        </is>
-      </c>
-    </row>
-    <row r="151"/>
-    <row r="152">
-      <c r="B152" s="4" t="inlineStr">
-        <is>
-          <t>Eckdaten</t>
-        </is>
-      </c>
-      <c r="C152" s="5" t="n"/>
-      <c r="D152" s="5" t="n"/>
-      <c r="E152" s="5" t="n"/>
-      <c r="F152" s="5" t="n"/>
-      <c r="H152" s="47" t="inlineStr">
-        <is>
-          <t>Anmerkung / Quelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="B153" s="6" t="inlineStr">
-        <is>
-          <t>Eigentümer</t>
-        </is>
-      </c>
-      <c r="C153" s="25" t="inlineStr">
-        <is>
-          <t>Jans &amp; Willems GbR</t>
-        </is>
-      </c>
-      <c r="D153" s="26" t="n"/>
-      <c r="E153" s="26" t="n"/>
-      <c r="F153" s="26" t="n"/>
-    </row>
-    <row r="154">
-      <c r="B154" s="6" t="inlineStr">
-        <is>
-          <t>Vermieter</t>
-        </is>
-      </c>
-      <c r="C154" s="25" t="inlineStr">
-        <is>
-          <t>Jans &amp; Willems GbR</t>
-        </is>
-      </c>
-      <c r="D154" s="26" t="n"/>
-      <c r="E154" s="26" t="n"/>
-      <c r="F154" s="26" t="n"/>
-      <c r="H154" s="47" t="inlineStr">
-        <is>
-          <t>Pfarrer-Hecker-Str. 33, 41849 Wassenberg, vertreten durch Werner Jans.</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="B155" s="6" t="inlineStr">
-        <is>
-          <t>Mieter</t>
-        </is>
-      </c>
-      <c r="C155" s="25" t="inlineStr">
-        <is>
-          <t>365° Pflegezentrum Marianne Weiß GmbH</t>
-        </is>
-      </c>
-      <c r="D155" s="26" t="n"/>
-      <c r="E155" s="26" t="n"/>
-      <c r="F155" s="26" t="n"/>
-      <c r="H155" s="47" t="inlineStr">
-        <is>
-          <t>opseo-Gruppe; Sitz Alleestraße 68, 42853 Remscheid.</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="B156" s="6" t="inlineStr">
-        <is>
-          <t>Adresse</t>
-        </is>
-      </c>
-      <c r="C156" s="25" t="inlineStr">
-        <is>
-          <t>Lessingstr. 3, 52499 Baesweiler</t>
-        </is>
-      </c>
-      <c r="D156" s="26" t="n"/>
-      <c r="E156" s="26" t="n"/>
-      <c r="F156" s="26" t="n"/>
-    </row>
-    <row r="157">
-      <c r="B157" s="6" t="inlineStr">
-        <is>
-          <t>Baujahr der Immobilie</t>
-        </is>
-      </c>
-      <c r="C157" s="25" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D157" s="26" t="n"/>
-      <c r="E157" s="26" t="n"/>
-      <c r="F157" s="26" t="n"/>
-      <c r="H157" s="47" t="inlineStr">
-        <is>
-          <t>Im Vertrag nicht genannt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="B158" s="6" t="inlineStr">
-        <is>
-          <t>Mietzweck</t>
-        </is>
-      </c>
-      <c r="C158" s="25" t="inlineStr">
-        <is>
-          <t>Intensivpflege-WG</t>
-        </is>
-      </c>
-      <c r="D158" s="26" t="n"/>
-      <c r="E158" s="26" t="n"/>
-      <c r="F158" s="26" t="n"/>
-    </row>
-    <row r="159">
-      <c r="B159" s="6" t="inlineStr">
-        <is>
-          <t>Festlaufzeit</t>
-        </is>
-      </c>
-      <c r="C159" s="25" t="inlineStr">
-        <is>
-          <t>5 Jahre</t>
-        </is>
-      </c>
-      <c r="D159" s="26" t="n"/>
-      <c r="E159" s="26" t="n"/>
-      <c r="F159" s="26" t="n"/>
-      <c r="H159" s="47" t="inlineStr">
-        <is>
-          <t>Kündigungsausschluss für beide Parteien (§2.2). WIDERSPRUCH: §2.3 räumt das Optionsrecht erst "nach Ablauf der ersten zehn Mietjahre" ein, §4.1 fixiert die Miete für zehn Jahre. Am Scan mit zwei OCR-Verfahren verifiziert – die Abweichung steht so im Dokument. Klärungsbedarf.</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="B160" s="6" t="inlineStr">
-        <is>
-          <t>Verlängerungsoptionen</t>
-        </is>
-      </c>
-      <c r="C160" s="25" t="inlineStr">
-        <is>
-          <t>2x 5 Jahre</t>
-        </is>
-      </c>
-      <c r="D160" s="26" t="n"/>
-      <c r="E160" s="26" t="n"/>
-      <c r="F160" s="26" t="n"/>
-      <c r="H160" s="47" t="inlineStr">
-        <is>
-          <t>Ausübung schriftlich spätestens 6 Monate vor Ablauf (§2.3); danach unbestimmte Zeit mit 6-Monats-Kündigungsfrist.</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="B161" s="6" t="inlineStr">
-        <is>
-          <t>Mietbeginn</t>
-        </is>
-      </c>
-      <c r="C161" s="25" t="inlineStr">
-        <is>
-          <t>Monatserster nach Vollzug des Kaufvertrags</t>
-        </is>
-      </c>
-      <c r="D161" s="26" t="n"/>
-      <c r="E161" s="26" t="n"/>
-      <c r="F161" s="26" t="n"/>
-      <c r="H161" s="47" t="inlineStr">
-        <is>
-          <t>Vollzugsdatum des Kaufvertrags Kuijpers v. 17.03.2023 zu bestätigen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="B162" s="6" t="inlineStr">
-        <is>
-          <t>Übergabezeitpunkt</t>
-        </is>
-      </c>
-      <c r="C162" s="25" t="inlineStr">
-        <is>
-          <t>keine Vertragsstrafe</t>
-        </is>
-      </c>
-      <c r="D162" s="26" t="n"/>
-      <c r="E162" s="26" t="n"/>
-      <c r="F162" s="26" t="n"/>
-      <c r="H162" s="47" t="inlineStr">
-        <is>
-          <t>Übergabeanspruch erst nach Stellung der Sicherheit (§3.1); geringfügige Mängel hindern die Übergabe nicht (§3.2).</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="B163" s="6" t="inlineStr">
-        <is>
-          <t>Aufschiebende Bedingung / Rücktrittsrecht</t>
-        </is>
-      </c>
-      <c r="C163" s="25" t="inlineStr">
-        <is>
-          <t>Vollzug Kaufvertrag Kuijpers</t>
-        </is>
-      </c>
-      <c r="D163" s="26" t="n"/>
-      <c r="E163" s="26" t="n"/>
-      <c r="F163" s="26" t="n"/>
-      <c r="H163" s="47" t="inlineStr">
-        <is>
-          <t>Der gesamte Mietvertrag steht unter dieser aufschiebenden Bedingung (Kuijpers Ambulante Pflege GmbH / PWH GmbH &amp; Co. KG, Vertrag v. 17.03.2023).</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="B164" s="6" t="inlineStr">
-        <is>
-          <t>Mietfreie Zeit</t>
-        </is>
-      </c>
-      <c r="C164" s="25" t="inlineStr">
-        <is>
-          <t>keine</t>
-        </is>
-      </c>
-      <c r="D164" s="26" t="n"/>
-      <c r="E164" s="26" t="n"/>
-      <c r="F164" s="26" t="n"/>
-    </row>
-    <row r="165">
-      <c r="B165" s="6" t="inlineStr">
-        <is>
-          <t>Wertsicherung (VPI)</t>
-        </is>
-      </c>
-      <c r="C165" s="25" t="inlineStr">
-        <is>
-          <t>keine; Miete 10 Jahre fest</t>
-        </is>
-      </c>
-      <c r="D165" s="26" t="n"/>
-      <c r="E165" s="26" t="n"/>
-      <c r="F165" s="26" t="n"/>
-      <c r="H165" s="47" t="inlineStr">
-        <is>
-          <t>Deutlicher Vorteil gegenüber Würselen, das mit 100% der Indexveränderung ab &gt;5% indexiert ist.</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="B166" s="6" t="inlineStr">
-        <is>
-          <t>Rückbauverpflichtung Mieter</t>
-        </is>
-      </c>
-      <c r="C166" s="25" t="inlineStr">
-        <is>
-          <t>keine</t>
-        </is>
-      </c>
-      <c r="D166" s="26" t="n"/>
-      <c r="E166" s="26" t="n"/>
-      <c r="F166" s="26" t="n"/>
-      <c r="H166" s="47" t="inlineStr">
-        <is>
-          <t>§15.1 stellt ausdrücklich klar, dass keine Rückbauverpflichtungen entstehen. Der Vermieter kann die Übernahme von Um-/Einbauten gegen Zeitwertentschädigung verlangen (§8.1.1).</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="B167" s="6" t="inlineStr">
-        <is>
-          <t>Untervermietung</t>
-        </is>
-      </c>
-      <c r="C167" s="25" t="inlineStr">
-        <is>
-          <t>Ja, zustimmungspflichtig</t>
-        </is>
-      </c>
-      <c r="D167" s="26" t="n"/>
-      <c r="E167" s="26" t="n"/>
-      <c r="F167" s="26" t="n"/>
-      <c r="H167" s="47" t="inlineStr">
-        <is>
-          <t>Ohne Zustimmung zulässig an verbundene Unternehmen i.S.d. §§15 ff. AktG sowie an pflegebedürftige Bewohner (§6.1).</t>
-        </is>
-      </c>
-    </row>
-    <row r="168" ht="65.25" customHeight="1">
-      <c r="B168" s="6" t="inlineStr">
-        <is>
-          <t>Mietsicherheit</t>
-        </is>
-      </c>
-      <c r="C168" s="51" t="inlineStr">
-        <is>
-          <t>Patronatserklärung. Größenordnung: 1 Jahreskaltmiete.</t>
-        </is>
-      </c>
-      <c r="D168" s="52" t="n"/>
-      <c r="E168" s="52" t="n"/>
-      <c r="F168" s="52" t="n"/>
-      <c r="H168" s="47" t="inlineStr">
-        <is>
-          <t>Patronatserklärung der Muttergesellschaft opseo Intensivpflege Holding B.V. = 102.000 €, binnen 4 Wochen nach Unterzeichnung (§5.1); Austausch bei Gesellschafterwechsel möglich (§5.3).</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="B169" s="6" t="inlineStr">
-        <is>
-          <t>Konkurrenzschutz</t>
-        </is>
-      </c>
-      <c r="C169" s="25" t="inlineStr">
-        <is>
-          <t>nein</t>
-        </is>
-      </c>
-      <c r="D169" s="26" t="n"/>
-      <c r="E169" s="26" t="n"/>
-      <c r="F169" s="26" t="n"/>
-    </row>
-    <row r="170">
-      <c r="B170" s="6" t="inlineStr">
-        <is>
-          <t>Sonderkündigungsrecht</t>
-        </is>
-      </c>
-      <c r="C170" s="25" t="inlineStr">
-        <is>
-          <t>Ja, bei Nutzungsuntersagung</t>
-        </is>
-      </c>
-      <c r="D170" s="26" t="n"/>
-      <c r="E170" s="26" t="n"/>
-      <c r="F170" s="26" t="n"/>
-      <c r="H170" s="47" t="inlineStr">
-        <is>
-          <t>Bei behördlicher Nutzungsuntersagung wegen des baulichen bzw. bau- und brandschutztechnischen Zustands, sofern der Vermieter sie nicht abwenden kann (§1.4).</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="B171" s="6" t="inlineStr">
-        <is>
-          <t>Instandhaltung/Instandsetzung</t>
-        </is>
-      </c>
-      <c r="C171" s="25" t="inlineStr">
-        <is>
-          <t>Dach und Fach beim Vermieter; Fläche beim Mieter</t>
-        </is>
-      </c>
-      <c r="D171" s="26" t="n"/>
-      <c r="E171" s="26" t="n"/>
-      <c r="F171" s="26" t="n"/>
-      <c r="H171" s="47" t="inlineStr">
-        <is>
-          <t>Übrige Instandhaltung veranlasst der Vermieter, Kosten umgelegt bis max. 5% der jährlichen Nettokaltmiete (§7.2). Schönheitsreparaturen beim Mieter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="B172" s="6" t="inlineStr">
-        <is>
-          <t>Besonderheiten / Sonstiges</t>
-        </is>
-      </c>
-      <c r="C172" s="25" t="inlineStr">
-        <is>
-          <t>Schlussabnahme fehlt; Inventar vermieterseitig gestellt</t>
-        </is>
-      </c>
-      <c r="D172" s="26" t="n"/>
-      <c r="E172" s="26" t="n"/>
-      <c r="F172" s="26" t="n"/>
-      <c r="H172" s="47" t="inlineStr">
-        <is>
-          <t>RED FLAG: Schlussabnahmebescheinigung liegt nicht vor, Nachtragsgenehmigung seit 02.02.2022 beantragt (§1.1) – zusammen mit dem Sonderkündigungsrecht aus §1.4 zu bewerten. Eigener Stromliefervertrag mit Abnahmepflicht für PV-Strom (§4.2.2). Eintritt in bestehende Untermietverträge (§18). Verkehrssicherung und Winterdienst beim Mieter (§17). Keine USt auf die Miete (§4.1). Gerichtsstand Wassenberg.</t>
-        </is>
-      </c>
-    </row>
-    <row r="173" ht="6.75" customHeight="1">
-      <c r="B173" s="7" t="n"/>
-      <c r="C173" s="8" t="n"/>
-      <c r="D173" s="7" t="n"/>
-      <c r="E173" s="7" t="n"/>
-      <c r="F173" s="7" t="n"/>
-    </row>
-    <row r="174"/>
-    <row r="175">
-      <c r="B175" s="9" t="inlineStr">
-        <is>
-          <t>Benchmarks (Neubau)</t>
-        </is>
-      </c>
-      <c r="C175" s="9" t="n"/>
-      <c r="D175" s="9" t="n"/>
-      <c r="E175" s="9" t="n"/>
-      <c r="F175" s="9" t="n"/>
-    </row>
-    <row r="176">
-      <c r="B176" s="6" t="inlineStr">
-        <is>
-          <t>Miete/m² (Neubau) - kein BKZ</t>
-        </is>
-      </c>
-      <c r="C176" s="62" t="n">
-        <v>20</v>
-      </c>
-      <c r="D176" s="26" t="n"/>
-      <c r="E176" s="26" t="n"/>
-      <c r="F176" s="26" t="n"/>
-    </row>
-    <row r="177">
-      <c r="B177" s="6" t="inlineStr">
-        <is>
-          <t>Miete/m² inkl. BKZ</t>
-        </is>
-      </c>
-      <c r="C177" s="62" t="n">
-        <v>20</v>
-      </c>
-      <c r="D177" s="26" t="n"/>
-      <c r="E177" s="26" t="n"/>
-      <c r="F177" s="26" t="n"/>
-    </row>
-    <row r="178">
-      <c r="B178" s="6" t="inlineStr">
-        <is>
-          <t>Nebenkosten/m²</t>
-        </is>
-      </c>
-      <c r="C178" s="62" t="n">
-        <v>3</v>
-      </c>
-      <c r="D178" s="26" t="n"/>
-      <c r="E178" s="26" t="n"/>
-      <c r="F178" s="26" t="n"/>
-    </row>
-    <row r="179">
-      <c r="B179" s="6" t="inlineStr">
-        <is>
-          <t>Fläche pro Bett</t>
-        </is>
-      </c>
-      <c r="C179" s="63" t="inlineStr">
-        <is>
-          <t>50m²</t>
-        </is>
-      </c>
-      <c r="D179" s="64" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> (d.h. 6er WG: 300m²; 12er WG: 600m²)</t>
-        </is>
-      </c>
-      <c r="E179" s="26" t="n"/>
-      <c r="F179" s="26" t="n"/>
-    </row>
-    <row r="180">
-      <c r="B180" s="6" t="inlineStr">
-        <is>
-          <t>Miete pro Bett pro Monat (exkl. Baukostenzuschuss)</t>
-        </is>
-      </c>
-      <c r="C180" s="63" t="n">
-        <v>1000</v>
-      </c>
-      <c r="D180" s="26" t="n"/>
-      <c r="E180" s="26" t="n"/>
-      <c r="F180" s="26" t="n"/>
-    </row>
-    <row r="181">
-      <c r="B181" s="6" t="inlineStr">
-        <is>
-          <t>Miete pro Bett pro Monat (inkl. BKZ über 10 Jahre)</t>
-        </is>
-      </c>
-      <c r="C181" s="63">
-        <f>+C180</f>
-        <v/>
-      </c>
-      <c r="D181" s="26" t="n"/>
-      <c r="E181" s="26" t="n"/>
-      <c r="F181" s="26" t="n"/>
-    </row>
-    <row r="182">
-      <c r="B182" s="6" t="inlineStr">
-        <is>
-          <t>Baukostenzuschuss pro Bett</t>
-        </is>
-      </c>
-      <c r="C182" s="63" t="n">
-        <v>0</v>
-      </c>
-      <c r="D182" s="64" t="n"/>
-      <c r="E182" s="26" t="n"/>
-      <c r="F182" s="26" t="n"/>
-    </row>
-    <row r="183">
-      <c r="B183" s="6" t="inlineStr">
-        <is>
-          <t>Capex pro Bett (Möbel, Ausstattung, etc.)</t>
-        </is>
-      </c>
-      <c r="C183" s="63" t="n">
-        <v>30000</v>
-      </c>
-      <c r="D183" s="26" t="n"/>
-      <c r="E183" s="26" t="n"/>
-      <c r="F183" s="26" t="n"/>
-    </row>
-    <row r="184">
-      <c r="B184" s="6" t="inlineStr">
-        <is>
-          <t>Baukosten pro qm (Neubau)</t>
-        </is>
-      </c>
-      <c r="C184" s="25" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D184" s="26" t="n"/>
-      <c r="E184" s="26" t="n"/>
-      <c r="F184" s="26" t="n"/>
-    </row>
-    <row r="185"/>
-    <row r="186">
-      <c r="B186" s="9" t="inlineStr">
-        <is>
-          <t>Benchmarks (Bestand)</t>
-        </is>
-      </c>
-      <c r="C186" s="9" t="n"/>
-      <c r="D186" s="9" t="n"/>
-      <c r="E186" s="9" t="n"/>
-      <c r="F186" s="9" t="n"/>
-    </row>
-    <row r="187">
-      <c r="B187" s="6" t="inlineStr">
-        <is>
-          <t>Miete/m² (Bestand) - kein BKZ</t>
-        </is>
-      </c>
-      <c r="C187" s="62" t="n">
-        <v>20</v>
-      </c>
-      <c r="D187" s="26" t="n"/>
-      <c r="E187" s="26" t="n"/>
-      <c r="F187" s="26" t="n"/>
-    </row>
-    <row r="188">
-      <c r="B188" s="6" t="inlineStr">
-        <is>
-          <t>Miete/m² (Bestand) inkl. BKZ</t>
-        </is>
-      </c>
-      <c r="C188" s="62" t="n">
-        <v>25</v>
-      </c>
-      <c r="D188" s="26" t="n"/>
-      <c r="E188" s="26" t="n"/>
-      <c r="F188" s="26" t="n"/>
-    </row>
-    <row r="189">
-      <c r="B189" s="6" t="inlineStr">
-        <is>
-          <t>Nebenkosten/m²</t>
-        </is>
-      </c>
-      <c r="C189" s="62" t="n">
-        <v>3</v>
-      </c>
-      <c r="D189" s="26" t="n"/>
-      <c r="E189" s="26" t="n"/>
-      <c r="F189" s="26" t="n"/>
-    </row>
-    <row r="190">
-      <c r="B190" s="6" t="inlineStr">
-        <is>
-          <t>Fläche pro Bett</t>
-        </is>
-      </c>
-      <c r="C190" s="63" t="inlineStr">
-        <is>
-          <t>50m²</t>
-        </is>
-      </c>
-      <c r="D190" s="64" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> (d.h. 6er WG: 300m²; 12er WG: 600m²)</t>
-        </is>
-      </c>
-      <c r="E190" s="26" t="n"/>
-      <c r="F190" s="26" t="n"/>
-    </row>
-    <row r="191">
-      <c r="B191" s="6" t="inlineStr">
-        <is>
-          <t>Miete pro Bett pro Monat (exkl. Baukostenzuschuss)</t>
-        </is>
-      </c>
-      <c r="C191" s="63" t="n">
-        <v>1000</v>
-      </c>
-      <c r="D191" s="26" t="n"/>
-      <c r="E191" s="26" t="n"/>
-      <c r="F191" s="26" t="n"/>
-    </row>
-    <row r="192">
-      <c r="B192" s="6" t="inlineStr">
-        <is>
-          <t>Miete pro Bett pro Monat (inkl. BKZ über 10 Jahre)</t>
-        </is>
-      </c>
-      <c r="C192" s="63" t="n">
-        <v>1250</v>
-      </c>
-      <c r="D192" s="26" t="n"/>
-      <c r="E192" s="26" t="n"/>
-      <c r="F192" s="26" t="n"/>
-    </row>
-    <row r="193">
-      <c r="B193" s="6" t="inlineStr">
-        <is>
-          <t>Baukostenzuschuss pro Bett</t>
-        </is>
-      </c>
-      <c r="C193" s="63" t="n">
-        <v>40000</v>
-      </c>
-      <c r="D193" s="64" t="inlineStr">
-        <is>
-          <t>(d.h. 6er WG: 180.000 €, 12er WG: 360.000 €)</t>
-        </is>
-      </c>
-      <c r="E193" s="26" t="n"/>
-      <c r="F193" s="26" t="n"/>
-    </row>
-    <row r="194">
-      <c r="B194" s="6" t="inlineStr">
-        <is>
-          <t>Capex pro Bett (Möbel, Ausstattung, etc.)</t>
-        </is>
-      </c>
-      <c r="C194" s="63" t="n">
-        <v>30000</v>
-      </c>
-      <c r="D194" s="26" t="n"/>
-      <c r="E194" s="26" t="n"/>
-      <c r="F194" s="26" t="n"/>
-    </row>
-    <row r="195">
-      <c r="B195" s="6" t="inlineStr">
-        <is>
-          <t>Baukosten pro qm (Neubau)</t>
-        </is>
-      </c>
-      <c r="C195" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D195" s="26" t="n"/>
-      <c r="E195" s="26" t="n"/>
-      <c r="F195" s="26" t="n"/>
-    </row>
-    <row r="196"/>
-    <row r="197">
-      <c r="B197" s="9" t="inlineStr">
-        <is>
-          <t>Mietkosten</t>
-        </is>
-      </c>
-      <c r="C197" s="9" t="n"/>
-      <c r="D197" s="9" t="n"/>
-      <c r="E197" s="9" t="n"/>
-      <c r="F197" s="9" t="n"/>
-    </row>
-    <row r="198">
-      <c r="B198" s="10" t="inlineStr">
-        <is>
-          <t>Einheit 1</t>
-        </is>
-      </c>
-      <c r="C198" s="10" t="n"/>
-      <c r="D198" s="10" t="n"/>
-      <c r="E198" s="10" t="n"/>
-      <c r="F198" s="10" t="n"/>
-    </row>
-    <row r="199">
-      <c r="B199" s="6" t="inlineStr">
-        <is>
-          <t>Art (z.B. WG, Büro, etc.)</t>
-        </is>
-      </c>
-      <c r="C199" s="27" t="inlineStr">
-        <is>
-          <t>WG (Intensivpflege-Wohngemeinschaft)</t>
-        </is>
-      </c>
-      <c r="D199" s="26" t="n"/>
-      <c r="E199" s="26" t="n"/>
-      <c r="F199" s="26" t="n"/>
-    </row>
-    <row r="200">
-      <c r="B200" s="6" t="inlineStr">
-        <is>
-          <t>Lage der Mietfläche (z.B. EG, 1. OG)</t>
-        </is>
-      </c>
-      <c r="C200" s="27" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D200" s="26" t="n"/>
-      <c r="E200" s="26" t="n"/>
-      <c r="F200" s="26" t="n"/>
-      <c r="H200" s="47" t="inlineStr">
-        <is>
-          <t>Etagenlage im Vertrag nicht spezifiziert; Abstellräume im Kellergeschoss erfasst (§1.1). Die EG-Wohnung ist nicht Mietgegenstand (§9.3).</t>
-        </is>
-      </c>
-    </row>
-    <row r="201">
-      <c r="B201" s="6" t="inlineStr">
-        <is>
-          <t>Kapazität (Anzahl Betten)</t>
-        </is>
-      </c>
-      <c r="C201" s="27" t="n">
-        <v>18</v>
-      </c>
-      <c r="D201" s="26" t="n"/>
-      <c r="E201" s="26" t="n"/>
-      <c r="F201" s="26" t="n"/>
-      <c r="H201" s="47" t="inlineStr">
-        <is>
-          <t>ca. 18 Patientenzimmer (§1.1); die NK-Kalkulation (250 €/Platz = 4.700 €) impliziert 18,8 Plätze.</t>
-        </is>
-      </c>
-    </row>
-    <row r="202">
-      <c r="B202" s="6" t="inlineStr">
-        <is>
-          <t>Größe der Fläche (in qm)</t>
-        </is>
-      </c>
-      <c r="C202" s="28" t="n">
-        <v>1082</v>
-      </c>
-      <c r="D202" s="26" t="n"/>
-      <c r="E202" s="26" t="n"/>
-      <c r="F202" s="26" t="n"/>
-    </row>
-    <row r="203">
-      <c r="B203" s="6" t="inlineStr">
-        <is>
-          <t>Mietbeginn (falls abweichned)</t>
-        </is>
-      </c>
-      <c r="C203" s="29" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D203" s="26" t="n"/>
-      <c r="E203" s="26" t="n"/>
-      <c r="F203" s="26" t="n"/>
-    </row>
-    <row r="204"/>
-    <row r="205">
-      <c r="B205" s="11" t="inlineStr">
-        <is>
-          <t>Kosten Einheit 1</t>
-        </is>
-      </c>
-      <c r="C205" s="12" t="inlineStr">
-        <is>
-          <t>Anzahl</t>
-        </is>
-      </c>
-      <c r="D205" s="12" t="inlineStr">
-        <is>
-          <t>€ pro Einheit</t>
-        </is>
-      </c>
-      <c r="E205" s="12" t="inlineStr">
-        <is>
-          <t>€ pro Monat</t>
-        </is>
-      </c>
-      <c r="F205" s="12" t="inlineStr">
-        <is>
-          <t>€ pro Jahr</t>
-        </is>
-      </c>
-    </row>
-    <row r="206">
-      <c r="B206" s="2" t="inlineStr">
-        <is>
-          <t>Nettokaltmiete</t>
-        </is>
-      </c>
-      <c r="C206" s="30" t="n">
-        <v>1082</v>
-      </c>
-      <c r="D206" s="31" t="n">
-        <v>7.855822550831793</v>
-      </c>
-      <c r="E206" s="13">
-        <f>+C206*D206</f>
-        <v/>
-      </c>
-      <c r="F206" s="13">
-        <f>+E206*12</f>
-        <v/>
-      </c>
-      <c r="H206" s="47" t="inlineStr">
-        <is>
-          <t>Pauschalmiete 8.500 € bzw. NK-Pauschale 4.700 €; die qm-Preise sind rechnerisch abgeleitet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="207">
-      <c r="B207" s="6" t="inlineStr">
-        <is>
-          <t>Nebenkostenpauschale</t>
-        </is>
-      </c>
-      <c r="C207" s="32">
-        <f>+C206</f>
-        <v/>
-      </c>
-      <c r="D207" s="33" t="n">
-        <v>4.343807763401109</v>
-      </c>
-      <c r="E207" s="13">
-        <f>+C207*D207</f>
-        <v/>
-      </c>
-      <c r="F207" s="13">
-        <f>+E207*12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="208">
-      <c r="B208" s="6" t="inlineStr">
-        <is>
-          <t>Stellplätze</t>
-        </is>
-      </c>
-      <c r="C208" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="D208" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E208" s="13">
-        <f>+C208*D208</f>
-        <v/>
-      </c>
-      <c r="F208" s="13">
-        <f>+E208*12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="209">
-      <c r="B209" s="6" t="inlineStr">
-        <is>
-          <t>Terasse</t>
-        </is>
-      </c>
-      <c r="C209" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="D209" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E209" s="13">
-        <f>+C209*D209</f>
-        <v/>
-      </c>
-      <c r="F209" s="13">
-        <f>+E209*12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="210">
-      <c r="B210" s="6" t="inlineStr">
-        <is>
-          <t>Keller</t>
-        </is>
-      </c>
-      <c r="C210" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="D210" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E210" s="13">
-        <f>+C210*D210</f>
-        <v/>
-      </c>
-      <c r="F210" s="13">
-        <f>+E210*12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="211">
-      <c r="B211" s="6" t="inlineStr">
-        <is>
-          <t>Sonstiges</t>
-        </is>
-      </c>
-      <c r="C211" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="D211" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E211" s="13">
-        <f>+C211*D211</f>
-        <v/>
-      </c>
-      <c r="F211" s="13">
-        <f>+E211*12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="212" ht="8.25" customHeight="1">
-      <c r="B212" s="14" t="n"/>
-      <c r="C212" s="15" t="n"/>
-      <c r="D212" s="16" t="n"/>
-      <c r="E212" s="17" t="n"/>
-      <c r="F212" s="17" t="n"/>
-    </row>
-    <row r="213">
-      <c r="B213" s="1" t="inlineStr">
-        <is>
-          <t>Summe</t>
-        </is>
-      </c>
-      <c r="C213" s="18" t="n"/>
-      <c r="D213" s="19" t="n"/>
-      <c r="E213" s="20">
-        <f>+SUM(E206:E212)</f>
-        <v/>
-      </c>
-      <c r="F213" s="20">
-        <f>+SUM(F206:F212)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="214" ht="6.75" customHeight="1">
-      <c r="B214" s="7" t="n"/>
-      <c r="C214" s="8" t="n"/>
-      <c r="D214" s="7" t="n"/>
-      <c r="E214" s="7" t="n"/>
-      <c r="F214" s="7" t="n"/>
-    </row>
-    <row r="215"/>
-    <row r="216">
-      <c r="B216" s="10" t="inlineStr">
-        <is>
-          <t>Einheit 2</t>
-        </is>
-      </c>
-      <c r="C216" s="10" t="n"/>
-      <c r="D216" s="10" t="n"/>
-      <c r="E216" s="10" t="n"/>
-      <c r="F216" s="10" t="n"/>
-    </row>
-    <row r="217">
-      <c r="B217" s="6" t="inlineStr">
-        <is>
-          <t>Art (z.B. WG, Büro, etc.)</t>
-        </is>
-      </c>
-      <c r="C217" s="27" t="inlineStr">
-        <is>
-          <t>entfällt</t>
-        </is>
-      </c>
-      <c r="D217" s="26" t="n"/>
-      <c r="E217" s="26" t="n"/>
-      <c r="F217" s="26" t="n"/>
-    </row>
-    <row r="218">
-      <c r="B218" s="6" t="inlineStr">
-        <is>
-          <t>Lage der Mietfläche (z.B. EG, 1. OG)</t>
-        </is>
-      </c>
-      <c r="C218" s="27" t="n"/>
-      <c r="D218" s="26" t="n"/>
-      <c r="E218" s="26" t="n"/>
-      <c r="F218" s="26" t="n"/>
-    </row>
-    <row r="219">
-      <c r="B219" s="6" t="inlineStr">
-        <is>
-          <t>Kapazität (Anzahl Betten)</t>
-        </is>
-      </c>
-      <c r="C219" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D219" s="26" t="n"/>
-      <c r="E219" s="26" t="n"/>
-      <c r="F219" s="26" t="n"/>
-    </row>
-    <row r="220">
-      <c r="B220" s="6" t="inlineStr">
-        <is>
-          <t>Größe der Fläche (in qm)</t>
-        </is>
-      </c>
-      <c r="C220" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="D220" s="26" t="n"/>
-      <c r="E220" s="26" t="n"/>
-      <c r="F220" s="26" t="n"/>
-    </row>
-    <row r="221">
-      <c r="B221" s="6" t="inlineStr">
-        <is>
-          <t>Mietbeginn (falls abweichned)</t>
-        </is>
-      </c>
-      <c r="C221" s="29" t="n"/>
-      <c r="D221" s="26" t="n"/>
-      <c r="E221" s="26" t="n"/>
-      <c r="F221" s="26" t="n"/>
-    </row>
-    <row r="222"/>
-    <row r="223">
-      <c r="B223" s="11" t="inlineStr">
-        <is>
-          <t>Kosten Einheit 2</t>
-        </is>
-      </c>
-      <c r="C223" s="12" t="inlineStr">
-        <is>
-          <t>Anzahl</t>
-        </is>
-      </c>
-      <c r="D223" s="12" t="inlineStr">
-        <is>
-          <t>€ pro Einheit</t>
-        </is>
-      </c>
-      <c r="E223" s="12" t="inlineStr">
-        <is>
-          <t>€ pro Monat</t>
-        </is>
-      </c>
-      <c r="F223" s="12" t="inlineStr">
-        <is>
-          <t>€ pro Jahr</t>
-        </is>
-      </c>
-    </row>
-    <row r="224">
-      <c r="B224" s="2" t="inlineStr">
-        <is>
-          <t>Nettokaltmiete</t>
-        </is>
-      </c>
-      <c r="C224" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D224" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="E224" s="13">
-        <f>+C224*D224</f>
-        <v/>
-      </c>
-      <c r="F224" s="13">
-        <f>+E224*12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="225">
-      <c r="B225" s="6" t="inlineStr">
-        <is>
-          <t>Nebenkostenpauschale</t>
-        </is>
-      </c>
-      <c r="C225" s="32">
-        <f>+C224</f>
-        <v/>
-      </c>
-      <c r="D225" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E225" s="13">
-        <f>+C225*D225</f>
-        <v/>
-      </c>
-      <c r="F225" s="13">
-        <f>+E225*12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="226">
-      <c r="B226" s="6" t="inlineStr">
-        <is>
-          <t>Stellplätze</t>
-        </is>
-      </c>
-      <c r="C226" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="D226" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E226" s="13">
-        <f>+C226*D226</f>
-        <v/>
-      </c>
-      <c r="F226" s="13">
-        <f>+E226*12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="227">
-      <c r="B227" s="6" t="inlineStr">
-        <is>
-          <t>Terasse</t>
-        </is>
-      </c>
-      <c r="C227" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="D227" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E227" s="13">
-        <f>+C227*D227</f>
-        <v/>
-      </c>
-      <c r="F227" s="13">
-        <f>+E227*12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="228">
-      <c r="B228" s="6" t="inlineStr">
-        <is>
-          <t>Keller</t>
-        </is>
-      </c>
-      <c r="C228" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="D228" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E228" s="13">
-        <f>+C228*D228</f>
-        <v/>
-      </c>
-      <c r="F228" s="13">
-        <f>+E228*12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="229">
-      <c r="B229" s="6" t="inlineStr">
-        <is>
-          <t>Sonstiges</t>
-        </is>
-      </c>
-      <c r="C229" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="D229" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E229" s="13">
-        <f>+C229*D229</f>
-        <v/>
-      </c>
-      <c r="F229" s="13">
-        <f>+E229*12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="230" ht="8.25" customHeight="1">
-      <c r="B230" s="14" t="n"/>
-      <c r="C230" s="15" t="n"/>
-      <c r="D230" s="16" t="n"/>
-      <c r="E230" s="17" t="n"/>
-      <c r="F230" s="17" t="n"/>
-    </row>
-    <row r="231">
-      <c r="B231" s="1" t="inlineStr">
-        <is>
-          <t>Summe</t>
-        </is>
-      </c>
-      <c r="C231" s="18" t="n"/>
-      <c r="D231" s="19" t="n"/>
-      <c r="E231" s="20">
-        <f>+SUM(E224:E230)</f>
-        <v/>
-      </c>
-      <c r="F231" s="20">
-        <f>+SUM(F224:F230)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="232" ht="6.75" customHeight="1">
-      <c r="B232" s="7" t="n"/>
-      <c r="C232" s="8" t="n"/>
-      <c r="D232" s="7" t="n"/>
-      <c r="E232" s="7" t="n"/>
-      <c r="F232" s="7" t="n"/>
-    </row>
-    <row r="233"/>
-    <row r="234">
-      <c r="B234" s="10" t="inlineStr">
-        <is>
-          <t>Einheit 3</t>
-        </is>
-      </c>
-      <c r="C234" s="10" t="n"/>
-      <c r="D234" s="10" t="n"/>
-      <c r="E234" s="10" t="n"/>
-      <c r="F234" s="10" t="n"/>
-    </row>
-    <row r="235">
-      <c r="B235" s="6" t="inlineStr">
-        <is>
-          <t>Art (z.B. WG, Büro, etc.)</t>
-        </is>
-      </c>
-      <c r="C235" s="27" t="inlineStr">
-        <is>
-          <t>entfällt</t>
-        </is>
-      </c>
-      <c r="D235" s="26" t="n"/>
-      <c r="E235" s="26" t="n"/>
-      <c r="F235" s="26" t="n"/>
-    </row>
-    <row r="236">
-      <c r="B236" s="6" t="inlineStr">
-        <is>
-          <t>Lage der Mietfläche (z.B. EG, 1. OG)</t>
-        </is>
-      </c>
-      <c r="C236" s="27" t="n"/>
-      <c r="D236" s="26" t="n"/>
-      <c r="E236" s="26" t="n"/>
-      <c r="F236" s="26" t="n"/>
-    </row>
-    <row r="237">
-      <c r="B237" s="6" t="inlineStr">
-        <is>
-          <t>Kapazität (Anzahl Betten)</t>
-        </is>
-      </c>
-      <c r="C237" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D237" s="26" t="n"/>
-      <c r="E237" s="26" t="n"/>
-      <c r="F237" s="26" t="n"/>
-    </row>
-    <row r="238">
-      <c r="B238" s="6" t="inlineStr">
-        <is>
-          <t>Größe der Fläche (in qm)</t>
-        </is>
-      </c>
-      <c r="C238" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="D238" s="26" t="n"/>
-      <c r="E238" s="26" t="n"/>
-      <c r="F238" s="26" t="n"/>
-    </row>
-    <row r="239">
-      <c r="B239" s="6" t="inlineStr">
-        <is>
-          <t>Mietbeginn (falls abweichned)</t>
-        </is>
-      </c>
-      <c r="C239" s="29" t="n"/>
-      <c r="D239" s="26" t="n"/>
-      <c r="E239" s="26" t="n"/>
-      <c r="F239" s="26" t="n"/>
-    </row>
-    <row r="240"/>
-    <row r="241">
-      <c r="B241" s="11" t="inlineStr">
-        <is>
-          <t>Kosten Einheit 3</t>
-        </is>
-      </c>
-      <c r="C241" s="12" t="inlineStr">
-        <is>
-          <t>Anzahl</t>
-        </is>
-      </c>
-      <c r="D241" s="12" t="inlineStr">
-        <is>
-          <t>€ pro Einheit</t>
-        </is>
-      </c>
-      <c r="E241" s="12" t="inlineStr">
-        <is>
-          <t>€ pro Monat</t>
-        </is>
-      </c>
-      <c r="F241" s="12" t="inlineStr">
-        <is>
-          <t>€ pro Jahr</t>
-        </is>
-      </c>
-    </row>
-    <row r="242">
-      <c r="B242" s="2" t="inlineStr">
-        <is>
-          <t>Nettokaltmiete</t>
-        </is>
-      </c>
-      <c r="C242" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D242" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="E242" s="13">
-        <f>+C242*D242</f>
-        <v/>
-      </c>
-      <c r="F242" s="13">
-        <f>+E242*12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="243">
-      <c r="B243" s="6" t="inlineStr">
-        <is>
-          <t>Nebenkostenpauschale</t>
-        </is>
-      </c>
-      <c r="C243" s="32">
-        <f>+C242</f>
-        <v/>
-      </c>
-      <c r="D243" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E243" s="13">
-        <f>+C243*D243</f>
-        <v/>
-      </c>
-      <c r="F243" s="13">
-        <f>+E243*12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="244">
-      <c r="B244" s="6" t="inlineStr">
-        <is>
-          <t>Stellplätze</t>
-        </is>
-      </c>
-      <c r="C244" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="D244" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E244" s="13">
-        <f>+C244*D244</f>
-        <v/>
-      </c>
-      <c r="F244" s="13">
-        <f>+E244*12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="245">
-      <c r="B245" s="6" t="inlineStr">
-        <is>
-          <t>Terasse</t>
-        </is>
-      </c>
-      <c r="C245" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="D245" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E245" s="13">
-        <f>+C245*D245</f>
-        <v/>
-      </c>
-      <c r="F245" s="13">
-        <f>+E245*12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="246">
-      <c r="B246" s="6" t="inlineStr">
-        <is>
-          <t>Keller</t>
-        </is>
-      </c>
-      <c r="C246" s="32" t="n">
-        <v>0</v>
-      </c>
-      <c r="D246" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E246" s="13">
-        <f>+C246*D246</f>
-        <v/>
-      </c>
-      <c r="F246" s="13">
-        <f>+E246*12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="247">
-      <c r="B247" s="6" t="inlineStr">
-        <is>
-          <t>Sonstiges</t>
-        </is>
-      </c>
-      <c r="C247" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="D247" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E247" s="13">
-        <f>+C247*D247</f>
-        <v/>
-      </c>
-      <c r="F247" s="13">
-        <f>+E247*12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="248" ht="8.25" customHeight="1">
-      <c r="B248" s="14" t="n"/>
-      <c r="C248" s="15" t="n"/>
-      <c r="D248" s="16" t="n"/>
-      <c r="E248" s="17" t="n"/>
-      <c r="F248" s="17" t="n"/>
-    </row>
-    <row r="249">
-      <c r="B249" s="1" t="inlineStr">
-        <is>
-          <t>Summe</t>
-        </is>
-      </c>
-      <c r="C249" s="18" t="n"/>
-      <c r="D249" s="19" t="n"/>
-      <c r="E249" s="20">
-        <f>+SUM(E242:E248)</f>
-        <v/>
-      </c>
-      <c r="F249" s="20">
-        <f>+SUM(F242:F248)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="250" ht="6.75" customHeight="1">
-      <c r="B250" s="7" t="n"/>
-      <c r="C250" s="8" t="n"/>
-      <c r="D250" s="7" t="n"/>
-      <c r="E250" s="7" t="n"/>
-      <c r="F250" s="7" t="n"/>
-    </row>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253">
-      <c r="B253" s="23" t="inlineStr">
-        <is>
-          <t>Capex</t>
-        </is>
-      </c>
-      <c r="C253" s="23" t="inlineStr">
-        <is>
-          <t>Anmerkungen</t>
-        </is>
-      </c>
-      <c r="D253" s="24" t="n"/>
-      <c r="E253" s="24" t="n"/>
-      <c r="F253" s="24" t="n"/>
-    </row>
-    <row r="254">
-      <c r="B254" s="35" t="inlineStr">
-        <is>
-          <t>Möbel Patientenzimmer</t>
-        </is>
-      </c>
-      <c r="C254" s="36" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D254" s="37" t="n"/>
-      <c r="E254" s="38" t="n"/>
-      <c r="F254" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="H254" s="47" t="inlineStr">
-        <is>
-          <t>Inventar (Einbauküchen, Pflegebetten, Vorhänge) vermieterseitig gestellt und im Mietzins enthalten (§1.2).</t>
-        </is>
-      </c>
-    </row>
-    <row r="255">
-      <c r="B255" s="35" t="inlineStr">
-        <is>
-          <t>Gemeinschaftsbereich</t>
-        </is>
-      </c>
-      <c r="C255" s="25" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D255" s="39" t="n"/>
-      <c r="E255" s="40" t="n"/>
-      <c r="F255" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="256">
-      <c r="B256" s="35" t="inlineStr">
-        <is>
-          <t>Schwesternrufanlage</t>
-        </is>
-      </c>
-      <c r="C256" s="25" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D256" s="39" t="n"/>
-      <c r="E256" s="40" t="n"/>
-      <c r="F256" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="257">
-      <c r="B257" s="35" t="inlineStr">
-        <is>
-          <t>Pflegebad</t>
-        </is>
-      </c>
-      <c r="C257" s="25" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D257" s="39" t="n"/>
-      <c r="E257" s="40" t="n"/>
-      <c r="F257" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="258">
-      <c r="B258" s="35" t="inlineStr">
-        <is>
-          <t>Fäkalienspüle</t>
-        </is>
-      </c>
-      <c r="C258" s="25" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D258" s="39" t="n"/>
-      <c r="E258" s="40" t="n"/>
-      <c r="F258" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="259">
-      <c r="B259" s="35" t="inlineStr">
-        <is>
-          <t>Umbaukosten</t>
-        </is>
-      </c>
-      <c r="C259" s="25" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D259" s="39" t="n"/>
-      <c r="E259" s="40" t="n"/>
-      <c r="F259" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="260">
-      <c r="B260" s="35" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="C260" s="25" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D260" s="39" t="n"/>
-      <c r="E260" s="40" t="n"/>
-      <c r="F260" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="261">
-      <c r="B261" s="35" t="inlineStr">
-        <is>
-          <t>Waschmaschinen</t>
-        </is>
-      </c>
-      <c r="C261" s="25" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D261" s="39" t="n"/>
-      <c r="E261" s="40" t="n"/>
-      <c r="F261" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="262">
-      <c r="B262" s="35" t="inlineStr">
-        <is>
-          <t>[Platzhalter]</t>
-        </is>
-      </c>
-      <c r="C262" s="25" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D262" s="39" t="n"/>
-      <c r="E262" s="40" t="n"/>
-      <c r="F262" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="263">
-      <c r="B263" s="35" t="inlineStr">
-        <is>
-          <t>[Platzhalter]</t>
-        </is>
-      </c>
-      <c r="C263" s="25" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D263" s="39" t="n"/>
-      <c r="E263" s="40" t="n"/>
-      <c r="F263" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="264">
-      <c r="B264" s="35" t="inlineStr">
-        <is>
-          <t>[Platzhalter]</t>
-        </is>
-      </c>
-      <c r="C264" s="25" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D264" s="39" t="n"/>
-      <c r="E264" s="40" t="n"/>
-      <c r="F264" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="265" ht="8.25" customHeight="1">
-      <c r="B265" s="14" t="n"/>
-      <c r="C265" s="15" t="n"/>
-      <c r="D265" s="16" t="n"/>
-      <c r="E265" s="17" t="n"/>
-      <c r="F265" s="17" t="n"/>
-    </row>
-    <row r="266">
-      <c r="B266" s="1" t="inlineStr">
-        <is>
-          <t>Summe</t>
-        </is>
-      </c>
-      <c r="C266" s="18" t="n"/>
-      <c r="D266" s="19" t="n"/>
-      <c r="E266" s="20" t="n"/>
-      <c r="F266" s="20">
-        <f>+SUM(F254:F265)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="267" ht="6.75" customHeight="1">
-      <c r="B267" s="7" t="n"/>
-      <c r="C267" s="8" t="n"/>
-      <c r="D267" s="7" t="n"/>
-      <c r="E267" s="7" t="n"/>
-      <c r="F267" s="7" t="n"/>
-    </row>
-    <row r="268" ht="6.75" customHeight="1"/>
-    <row r="269">
-      <c r="B269" s="21" t="inlineStr">
-        <is>
-          <t>davon:</t>
-        </is>
-      </c>
-    </row>
-    <row r="270">
-      <c r="B270" s="22" t="inlineStr">
-        <is>
-          <t>Übernahme Vermieter</t>
-        </is>
-      </c>
-      <c r="C270" s="25" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D270" s="39" t="n"/>
-      <c r="E270" s="40" t="n"/>
-      <c r="F270" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="271">
-      <c r="B271" s="22" t="inlineStr">
-        <is>
-          <t>Baukostenzuschuss Mieter</t>
-        </is>
-      </c>
-      <c r="C271" s="25" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D271" s="39" t="n"/>
-      <c r="E271" s="40" t="n"/>
-      <c r="F271" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="272" ht="6.75" customHeight="1">
-      <c r="B272" s="7" t="n"/>
-      <c r="C272" s="8" t="n"/>
-      <c r="D272" s="7" t="n"/>
-      <c r="E272" s="7" t="n"/>
-      <c r="F272" s="7" t="n"/>
-    </row>
-    <row r="273"/>
-    <row r="274"/>
-    <row r="275">
-      <c r="B275" s="23" t="inlineStr">
-        <is>
-          <t>Ramp-up Kosten</t>
-        </is>
-      </c>
-      <c r="C275" s="23" t="inlineStr">
-        <is>
-          <t>Anmerkungen</t>
-        </is>
-      </c>
-      <c r="D275" s="24" t="n"/>
-      <c r="E275" s="24" t="n"/>
-      <c r="F275" s="24" t="n"/>
-    </row>
-    <row r="276">
-      <c r="B276" s="35" t="inlineStr">
-        <is>
-          <t>Betriebsmittel</t>
-        </is>
-      </c>
-      <c r="C276" s="36" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D276" s="37" t="n"/>
-      <c r="E276" s="38" t="n"/>
-      <c r="F276" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="277">
-      <c r="B277" s="35" t="inlineStr">
-        <is>
-          <t>Werbung / Marketing</t>
-        </is>
-      </c>
-      <c r="C277" s="25" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D277" s="39" t="n"/>
-      <c r="E277" s="40" t="n"/>
-      <c r="F277" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="278">
-      <c r="B278" s="35" t="inlineStr">
-        <is>
-          <t>Personalbeschaffung</t>
-        </is>
-      </c>
-      <c r="C278" s="25" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D278" s="39" t="n"/>
-      <c r="E278" s="40" t="n"/>
-      <c r="F278" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="279">
-      <c r="B279" s="35" t="inlineStr">
-        <is>
-          <t>Planungskosten</t>
-        </is>
-      </c>
-      <c r="C279" s="25" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D279" s="39" t="n"/>
-      <c r="E279" s="40" t="n"/>
-      <c r="F279" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="280">
-      <c r="B280" s="35" t="inlineStr">
-        <is>
-          <t>Makler</t>
-        </is>
-      </c>
-      <c r="C280" s="25" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D280" s="39" t="n"/>
-      <c r="E280" s="40" t="n"/>
-      <c r="F280" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="281">
-      <c r="B281" s="35" t="inlineStr">
-        <is>
-          <t>[Platzhalter]</t>
-        </is>
-      </c>
-      <c r="C281" s="25" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D281" s="39" t="n"/>
-      <c r="E281" s="40" t="n"/>
-      <c r="F281" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="282">
-      <c r="B282" s="35" t="inlineStr">
-        <is>
-          <t>[Platzhalter]</t>
-        </is>
-      </c>
-      <c r="C282" s="25" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D282" s="39" t="n"/>
-      <c r="E282" s="40" t="n"/>
-      <c r="F282" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="283">
-      <c r="B283" s="35" t="inlineStr">
-        <is>
-          <t>[Platzhalter]</t>
-        </is>
-      </c>
-      <c r="C283" s="25" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D283" s="39" t="n"/>
-      <c r="E283" s="40" t="n"/>
-      <c r="F283" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="284">
-      <c r="B284" s="35" t="inlineStr">
-        <is>
-          <t>[Platzhalter]</t>
-        </is>
-      </c>
-      <c r="C284" s="25" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D284" s="39" t="n"/>
-      <c r="E284" s="40" t="n"/>
-      <c r="F284" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="285">
-      <c r="B285" s="35" t="inlineStr">
-        <is>
-          <t>[Platzhalter]</t>
-        </is>
-      </c>
-      <c r="C285" s="25" t="inlineStr">
-        <is>
-          <t>XXX</t>
-        </is>
-      </c>
-      <c r="D285" s="39" t="n"/>
-      <c r="E285" s="40" t="n"/>
-      <c r="F285" s="33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="286" ht="8.25" customHeight="1">
-      <c r="B286" s="14" t="n"/>
-      <c r="C286" s="15" t="n"/>
-      <c r="D286" s="16" t="n"/>
-      <c r="E286" s="17" t="n"/>
-      <c r="F286" s="17" t="n"/>
-    </row>
-    <row r="287">
-      <c r="B287" s="1" t="inlineStr">
-        <is>
-          <t>Summe</t>
-        </is>
-      </c>
-      <c r="C287" s="18" t="n"/>
-      <c r="D287" s="19" t="n"/>
-      <c r="E287" s="20" t="n"/>
-      <c r="F287" s="20">
-        <f>+SUM(F276:F286)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="288" ht="6.75" customHeight="1">
-      <c r="B288" s="7" t="n"/>
-      <c r="C288" s="8" t="n"/>
-      <c r="D288" s="7" t="n"/>
-      <c r="E288" s="7" t="n"/>
-      <c r="F288" s="7" t="n"/>
+      <c r="G142" s="67" t="n"/>
+      <c r="H142" s="7" t="n"/>
+      <c r="I142" s="7" t="n"/>
+      <c r="J142" s="7" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="C22:F22"/>
     <mergeCell ref="C4:F4"/>
-    <mergeCell ref="C168:F168"/>
+    <mergeCell ref="G4:J4"/>
+    <mergeCell ref="G22:J22"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.5118110236220472" right="0.5118110236220472" top="0.7874015748031497" bottom="0.7874015748031497" header="0.3149606299212598" footer="0.3149606299212598"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="96"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Baesweiler: Verlaengerung und aufschiebende Bedingung praezisiert
- Keine automatische Verlaengerung: der Vertrag laeuft auf unbestimmte Zeit,
  die Option muss aktiv ausgeuebt werden. Nach der Festlaufzeit beidseitig
  mit 6 Monaten kuendbar (Par. 2.3 Schlusssatz).
- Keine Vertragsstrafe und keine Schadensersatzregelung bei verspaeteter
  Uebergabe; per Volltextsuche bestaetigt.
- Der Vollzug des Kaufvertrags Kuijpers ist eine aufschiebende Bedingung,
  kein Ruecktrittsrecht - Zelle und Anmerkung entsprechend klargestellt.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018VKr7wEHLAW3yJNS7pxnAu
</commit_message>
<xml_diff>
--- a/mietkonditionen/Mietkonditionen_Vergleich_Wuerselen_Baesweiler.xlsx
+++ b/mietkonditionen/Mietkonditionen_Vergleich_Wuerselen_Baesweiler.xlsx
@@ -1849,7 +1849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:L142"/>
+  <dimension ref="B2:L142"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5"/>
   <cols>
     <col width="3.81640625" customWidth="1" style="2" min="1" max="1"/>
@@ -1861,7 +1861,6 @@
     <col width="11.453125" customWidth="1" style="2" min="9" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -2096,7 +2095,7 @@
       <c r="J13" s="26" t="n"/>
       <c r="L13" s="47" t="inlineStr">
         <is>
-          <t>Baesweiler: Kündigungsausschluss für beide Parteien (§2.2). WIDERSPRUCH: §2.3 räumt das Optionsrecht erst "nach Ablauf der ersten zehn Mietjahre" ein, §4.1 fixiert die Miete für zehn Jahre. Am Scan mit zwei OCR-Verfahren verifiziert – die Abweichung steht so im Dokument. Klärungsbedarf.</t>
+          <t>Würselen: 10 Jahre fest ab Übergabe.  |  Baesweiler: Vertrag läuft auf UNBESTIMMTE ZEIT, mit Kündigungsausschluss nur für die ersten 5 Mietjahre (§2.2). WIDERSPRUCH: §2.3 gewährt das Optionsrecht erst "nach Ablauf der ersten zehn Mietjahre", verlangt die Ausübung aber "6 Monate vor Ablauf der Festlaufzeit" – und Festlaufzeit ist in §2.2 als 5 Jahre definiert. §4.1 fixiert die Miete für 10 Jahre. Folge im Worst Case: ab Jahr 6 beidseitig mit 6 Monaten kündbar. Rechtlich prüfen lassen.</t>
         </is>
       </c>
     </row>
@@ -2117,7 +2116,7 @@
       <c r="F14" s="26" t="n"/>
       <c r="G14" s="65" t="inlineStr">
         <is>
-          <t>2x 5 Jahre</t>
+          <t>2x 5 Jahre, nur auf Ausübung</t>
         </is>
       </c>
       <c r="H14" s="26" t="n"/>
@@ -2125,7 +2124,7 @@
       <c r="J14" s="26" t="n"/>
       <c r="L14" s="47" t="inlineStr">
         <is>
-          <t>Baesweiler: Ausübung schriftlich spätestens 6 Monate vor Ablauf (§2.3); danach unbestimmte Zeit mit 6-Monats-Kündigungsfrist.</t>
+          <t>Würselen: Verlängerung tritt AUTOMATISCH ein, sofern der Mieter nicht 12 Monate vor Ablauf kündigt.  |  Baesweiler: KEINE Automatik – die Option muss aktiv schriftlich ausgeübt werden (§2.3). Ohne Ausübung läuft der Vertrag unbefristet weiter, dann aber von beiden Seiten mit 6 Monaten kündbar.</t>
         </is>
       </c>
     </row>
@@ -2181,7 +2180,7 @@
       <c r="J16" s="26" t="n"/>
       <c r="L16" s="47" t="inlineStr">
         <is>
-          <t>Baesweiler: Übergabeanspruch erst nach Stellung der Sicherheit (§3.1); geringfügige Mängel hindern die Übergabe nicht (§3.2).</t>
+          <t>Würselen: Schadensersatz 200 €/Kalendertag, gedeckelt auf 3 Nettomonatsmieten (§3.5).  |  Baesweiler: keinerlei Vertragsstrafe oder Schadensersatzregelung für verspätete Übergabe; Volltextsuche nach Vertragsstrafe/Pönale/Schadensersatz ohne Treffer.</t>
         </is>
       </c>
     </row>
@@ -2201,7 +2200,7 @@
       <c r="F17" s="26" t="n"/>
       <c r="G17" s="65" t="inlineStr">
         <is>
-          <t>Vollzug Kaufvertrag Kuijpers</t>
+          <t>Vollzug Kaufvertrag Kuijpers; kein Rücktrittsrecht</t>
         </is>
       </c>
       <c r="H17" s="26" t="n"/>
@@ -2209,7 +2208,7 @@
       <c r="J17" s="26" t="n"/>
       <c r="L17" s="47" t="inlineStr">
         <is>
-          <t>Baesweiler: Der gesamte Mietvertrag steht unter dieser aufschiebenden Bedingung (Kuijpers Ambulante Pflege GmbH / PWH GmbH &amp; Co. KG, Vertrag v. 17.03.2023).</t>
+          <t>Würselen: keine aufschiebende Bedingung.  |  Baesweiler: der gesamte Mietvertrag steht unter der aufschiebenden Bedingung des Vollzugs (Closing) des Kauf- und Übertragungsvertrags über Kuijpers Ambulante Pflege GmbH und PWH GmbH &amp; Co. KG vom 17.03.2023. Ohne Closing wird der Mietvertrag nie wirksam (§158 Abs. 1 BGB) – das ist KEIN Rücktrittsrecht. Ein Rücktrittsrecht enthält der Vertrag nicht; das Sonderkündigungsrecht steht separat in §1.4.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Baesweiler G14: Option als Kuendigungsausschluss statt Laufzeitverlaengerung
Der Vertrag laeuft ohnehin unbefristet; die Option verlaengert nicht die
Laufzeit, sondern den Kuendigungsausschluss um je 5 Jahre. Formulierung an
das zweizeilige Muster der Wuerselen-Zelle angeglichen.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018VKr7wEHLAW3yJNS7pxnAu
</commit_message>
<xml_diff>
--- a/mietkonditionen/Mietkonditionen_Vergleich_Wuerselen_Baesweiler.xlsx
+++ b/mietkonditionen/Mietkonditionen_Vergleich_Wuerselen_Baesweiler.xlsx
@@ -486,7 +486,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -732,6 +732,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2114,9 +2117,10 @@
       <c r="D14" s="26" t="n"/>
       <c r="E14" s="26" t="n"/>
       <c r="F14" s="26" t="n"/>
-      <c r="G14" s="65" t="inlineStr">
-        <is>
-          <t>2x 5 Jahre, nur auf Ausübung</t>
+      <c r="G14" s="86" t="inlineStr">
+        <is>
+          <t>2x 5 Jahre; 
+nur auf aktive Ausübung, verlängert jeweils den Kündigungsausschluss</t>
         </is>
       </c>
       <c r="H14" s="26" t="n"/>
@@ -2124,7 +2128,7 @@
       <c r="J14" s="26" t="n"/>
       <c r="L14" s="47" t="inlineStr">
         <is>
-          <t>Würselen: Verlängerung tritt AUTOMATISCH ein, sofern der Mieter nicht 12 Monate vor Ablauf kündigt.  |  Baesweiler: KEINE Automatik – die Option muss aktiv schriftlich ausgeübt werden (§2.3). Ohne Ausübung läuft der Vertrag unbefristet weiter, dann aber von beiden Seiten mit 6 Monaten kündbar.</t>
+          <t>Würselen: Verlängerung tritt AUTOMATISCH ein, sofern der Mieter nicht 12 Monate vor Ablauf kündigt.  |  Baesweiler: keine Automatik. Der Vertrag läuft ohnehin auf unbestimmte Zeit weiter – die Option verlängert nicht die Laufzeit, sondern den Kündigungsausschluss um je 5 Jahre (§2.3). Wird sie nicht ausgeübt, bleibt der Vertrag bestehen, ist dann aber von beiden Seiten mit 6 Monaten kündbar. Wirtschaftlich zählt daher nur die gesicherte Laufzeit, nicht die unbefristete Fortsetzung.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Baesweiler Konkurrenzschutz: 'nein' -> 'nicht geregelt'
Der Vertrag enthaelt keine Klausel, schliesst Konkurrenzschutz aber auch
nicht aus; ein vertragsimmanenter Schutz ist damit nicht ausgeschlossen.
Anmerkung mit Pruefauftrag und Hinweis auf den nicht vorliegenden Kaufvertrag.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018VKr7wEHLAW3yJNS7pxnAu
</commit_message>
<xml_diff>
--- a/mietkonditionen/Mietkonditionen_Vergleich_Wuerselen_Baesweiler.xlsx
+++ b/mietkonditionen/Mietkonditionen_Vergleich_Wuerselen_Baesweiler.xlsx
@@ -2367,12 +2367,17 @@
       <c r="F23" s="26" t="n"/>
       <c r="G23" s="65" t="inlineStr">
         <is>
-          <t>nein</t>
+          <t>nicht geregelt</t>
         </is>
       </c>
       <c r="H23" s="26" t="n"/>
       <c r="I23" s="26" t="n"/>
       <c r="J23" s="26" t="n"/>
+      <c r="L23" s="47" t="inlineStr">
+        <is>
+          <t>Würselen: gewährt nur für den Betrieb eines Wohnheims mit Intensivpflege (§6.3), ausdrücklich NICHT für andere medizinische Intensivpflege jedweder Ausrichtung (§6.4) – die Ausnahme hebt die Zusage weitgehend wieder auf.  |  Baesweiler: im Vertrag nicht geregelt. Alle 21 Paragraphen geprüft, Volltextsuche nach Konkurrenz/Wettbewerb/Exklusivität ohne Treffer. ABER: ein vertragsimmanenter Konkurrenzschutz kann sich nach der Rechtsprechung auch ohne Klausel als Nebenpflicht des Vermieters ergeben – da er hier auch nicht ausgeschlossen wurde, ist das anwaltlich zu bewerten. Ein etwaiges Wettbewerbsverbot dürfte zudem eher im Kaufvertrag vom 17.03.2023 stehen, der uns nicht vorliegt.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="B24" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Capex und Ramp-up: Kostentraegerschaft aus den Vertraegen ergaenzt
Die Betraege bleiben offen (nicht aus Mietvertraegen ableitbar), aber die
Anmerkungsspalten weisen jetzt aus, wer welche Position schuldet: Wuerselen
Vermieterausbau nach Raumbuch gegen mieterseitige Betriebsausstattung
(Par. 2.3.2, 2.3.5), Baesweiler vermieterseitig gestelltes Inventar (Par. 1.2)
und bereits vorhandene Schwesternruf-, Brandmelde- und Aufzugsanlage.
Ramp-up: Baesweiler als laufender Betrieb uebernommen (Par. 18).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018VKr7wEHLAW3yJNS7pxnAu
</commit_message>
<xml_diff>
--- a/mietkonditionen/Mietkonditionen_Vergleich_Wuerselen_Baesweiler.xlsx
+++ b/mietkonditionen/Mietkonditionen_Vergleich_Wuerselen_Baesweiler.xlsx
@@ -4250,6 +4250,11 @@
       <c r="H107" s="24" t="n"/>
       <c r="I107" s="24" t="n"/>
       <c r="J107" s="24" t="n"/>
+      <c r="L107" s="47" t="inlineStr">
+        <is>
+          <t>Beträge sind aus Mietverträgen grundsätzlich nicht ableitbar – sie kommen aus Anlagenspiegel bzw. Investitionsplanung des Targets. Die Verträge regeln aber die Kostenträgerschaft, und die steht hier: Würselen baut der Vermieter nach Raumbuch aus, der Mieter trägt die gesamte betriebsspezifische Ausstattung (§2.3.2) einschließlich Medizin-, IT- und Klimatechnik (§2.3.5). Baesweiler stellt der Vermieter das Inventar (§1.2) – Capex dort strukturell deutlich niedriger.</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="B108" s="35" t="inlineStr">
@@ -4259,7 +4264,7 @@
       </c>
       <c r="C108" s="36" t="inlineStr">
         <is>
-          <t>XXX</t>
+          <t>Mieter (§2.3.2 Möblierung)</t>
         </is>
       </c>
       <c r="D108" s="37" t="n"/>
@@ -4269,7 +4274,7 @@
       </c>
       <c r="G108" s="85" t="inlineStr">
         <is>
-          <t>XXX</t>
+          <t>Vermieter – Pflegebetten im Inventar (§1.2)</t>
         </is>
       </c>
       <c r="H108" s="37" t="n"/>
@@ -4291,7 +4296,7 @@
       </c>
       <c r="C109" s="25" t="inlineStr">
         <is>
-          <t>XXX</t>
+          <t>Mieter (§2.3.2)</t>
         </is>
       </c>
       <c r="D109" s="39" t="n"/>
@@ -4301,7 +4306,7 @@
       </c>
       <c r="G109" s="65" t="inlineStr">
         <is>
-          <t>XXX</t>
+          <t>Vermieter – Einbauküchen, Vorhänge (§1.2)</t>
         </is>
       </c>
       <c r="H109" s="39" t="n"/>
@@ -4318,7 +4323,7 @@
       </c>
       <c r="C110" s="25" t="inlineStr">
         <is>
-          <t>XXX</t>
+          <t>Mieter (§2.3.5)</t>
         </is>
       </c>
       <c r="D110" s="39" t="n"/>
@@ -4328,7 +4333,7 @@
       </c>
       <c r="G110" s="65" t="inlineStr">
         <is>
-          <t>XXX</t>
+          <t>vorhanden; nur Unterhaltung als NK (§4.2)</t>
         </is>
       </c>
       <c r="H110" s="39" t="n"/>
@@ -4336,6 +4341,11 @@
       <c r="J110" s="33" t="n">
         <v>0</v>
       </c>
+      <c r="L110" s="47" t="inlineStr">
+        <is>
+          <t>Baesweiler: eine Schwesternrufanlage existiert bereits; §4.2 legt nur deren Unterhaltungskosten als Nebenkosten um. Ebenso vorhanden: Brandmelde- und Aufzugsanlage.</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="B111" s="35" t="inlineStr">
@@ -4345,7 +4355,7 @@
       </c>
       <c r="C111" s="25" t="inlineStr">
         <is>
-          <t>XXX</t>
+          <t>Mieter; Pavillon nur vorgerüstet (§2.3.1)</t>
         </is>
       </c>
       <c r="D111" s="39" t="n"/>
@@ -4355,7 +4365,7 @@
       </c>
       <c r="G111" s="65" t="inlineStr">
         <is>
-          <t>XXX</t>
+          <t>XXX – im Vertrag nicht erwähnt</t>
         </is>
       </c>
       <c r="H111" s="39" t="n"/>
@@ -4363,6 +4373,11 @@
       <c r="J111" s="33" t="n">
         <v>0</v>
       </c>
+      <c r="L111" s="47" t="inlineStr">
+        <is>
+          <t>Würselen: der Eingangspavillon ist laut §2.3.1 nur so vorgerichtet, dass der spätere Einbau eines Pflegebades MÖGLICH ist – das Pflegebad selbst schuldet der Vermieter nicht.</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="B112" s="35" t="inlineStr">
@@ -4372,7 +4387,7 @@
       </c>
       <c r="C112" s="25" t="inlineStr">
         <is>
-          <t>XXX</t>
+          <t>XXX – Raumbuch (Anlage 1.4) liegt nicht vor</t>
         </is>
       </c>
       <c r="D112" s="39" t="n"/>
@@ -4382,7 +4397,7 @@
       </c>
       <c r="G112" s="65" t="inlineStr">
         <is>
-          <t>XXX</t>
+          <t>XXX – im Vertrag nicht erwähnt</t>
         </is>
       </c>
       <c r="H112" s="39" t="n"/>
@@ -4399,7 +4414,7 @@
       </c>
       <c r="C113" s="25" t="inlineStr">
         <is>
-          <t>XXX</t>
+          <t>Vermieter baut aus; Sonderwünsche zu Lasten Mieter</t>
         </is>
       </c>
       <c r="D113" s="39" t="n"/>
@@ -4409,7 +4424,7 @@
       </c>
       <c r="G113" s="65" t="inlineStr">
         <is>
-          <t>XXX</t>
+          <t>kein Umbau – laufender Betrieb übernommen</t>
         </is>
       </c>
       <c r="H113" s="39" t="n"/>
@@ -4426,7 +4441,7 @@
       </c>
       <c r="C114" s="25" t="inlineStr">
         <is>
-          <t>XXX</t>
+          <t>Mieter (§2.3.5)</t>
         </is>
       </c>
       <c r="D114" s="39" t="n"/>
@@ -4436,7 +4451,7 @@
       </c>
       <c r="G114" s="65" t="inlineStr">
         <is>
-          <t>XXX</t>
+          <t>Mieter</t>
         </is>
       </c>
       <c r="H114" s="39" t="n"/>
@@ -4615,7 +4630,7 @@
       </c>
       <c r="C124" s="25" t="inlineStr">
         <is>
-          <t>XXX</t>
+          <t>Ausbau nach Raumbuch (Anlage 1.4)</t>
         </is>
       </c>
       <c r="D124" s="39" t="n"/>
@@ -4625,7 +4640,7 @@
       </c>
       <c r="G124" s="65" t="inlineStr">
         <is>
-          <t>XXX</t>
+          <t>Inventar vermieterseitig gestellt (§1.2)</t>
         </is>
       </c>
       <c r="H124" s="39" t="n"/>
@@ -4642,7 +4657,7 @@
       </c>
       <c r="C125" s="25" t="inlineStr">
         <is>
-          <t>XXX</t>
+          <t>kein BKZ; faktisch 600 €/Mon. für Statik 1. OG</t>
         </is>
       </c>
       <c r="D125" s="39" t="n"/>
@@ -4652,7 +4667,7 @@
       </c>
       <c r="G125" s="65" t="inlineStr">
         <is>
-          <t>XXX</t>
+          <t>kein BKZ</t>
         </is>
       </c>
       <c r="H125" s="39" t="n"/>
@@ -4700,6 +4715,11 @@
       <c r="H129" s="24" t="n"/>
       <c r="I129" s="24" t="n"/>
       <c r="J129" s="24" t="n"/>
+      <c r="L129" s="47" t="inlineStr">
+        <is>
+          <t>Aus Mietverträgen nicht ableitbar. Ein struktureller Unterschied ergibt sich dennoch: Baesweiler wurde als laufender Betrieb übernommen – die Mieterin tritt nach §18 in die bestehenden Untermietverträge mit den Patienten ein, die Belegung besteht also bereits. Ein Belegungsaufbau entfällt damit weitgehend. Personalthemen hängen am Kaufvertrag vom 17.03.2023, der nicht vorliegt.</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="B130" s="35" t="inlineStr">
@@ -4709,7 +4729,7 @@
       </c>
       <c r="C130" s="36" t="inlineStr">
         <is>
-          <t>XXX</t>
+          <t>XXX – aus Target-Unterlagen</t>
         </is>
       </c>
       <c r="D130" s="37" t="n"/>
@@ -4719,7 +4739,7 @@
       </c>
       <c r="G130" s="85" t="inlineStr">
         <is>
-          <t>XXX</t>
+          <t>gering – Betrieb läuft bereits</t>
         </is>
       </c>
       <c r="H130" s="37" t="n"/>
@@ -4763,7 +4783,7 @@
       </c>
       <c r="C132" s="25" t="inlineStr">
         <is>
-          <t>XXX</t>
+          <t>XXX – aus Target-Unterlagen</t>
         </is>
       </c>
       <c r="D132" s="39" t="n"/>
@@ -4773,7 +4793,7 @@
       </c>
       <c r="G132" s="65" t="inlineStr">
         <is>
-          <t>XXX</t>
+          <t>XXX – abhängig vom Kaufvertrag (liegt nicht vor)</t>
         </is>
       </c>
       <c r="H132" s="39" t="n"/>

</xml_diff>

<commit_message>
Statik-Zuschlag 1. OG: Rechenbeleg und offene Punkte dokumentiert
Die 600 EUR sind rechnerisch als monatlicher Bestandteil der Gesamtmiete
belegt (5.605,12 + 600,00 = 6.205,12; Gesamtmiete 19.376,87). Ergaenzt um
Volumen bis Ende Festlaufzeit bzw. bei Optionsausuebung sowie die offenen
Fragen zu tatsaechlichen Statikkosten, Indexierung und Fortgeltung.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018VKr7wEHLAW3yJNS7pxnAu
</commit_message>
<xml_diff>
--- a/mietkonditionen/Mietkonditionen_Vergleich_Wuerselen_Baesweiler.xlsx
+++ b/mietkonditionen/Mietkonditionen_Vergleich_Wuerselen_Baesweiler.xlsx
@@ -4675,6 +4675,11 @@
       <c r="J125" s="33" t="n">
         <v>0</v>
       </c>
+      <c r="L125" s="47" t="inlineStr">
+        <is>
+          <t>Würselen: die 600 €/Monat für die statischen Mehraufwendungen im 1. OG (3. Nachtrag Ziff. 3) sind laufende Miete, nicht einmalig – belegt durch die Rechnung des Nachtrags selbst: 350,32 qm x 12,50 € = 4.379,00 zzgl. 350,32 qm x 3,50 € = 1.226,12, macht 5.605,12; plus 600,00 ergibt die im Vertrag genannten 6.205,12, und die gehen in der monatlichen Gesamtmiete von 19.376,87 € auf. Volumen: 7.200 €/Jahr, rd. 54.300 € bis Ende der Festlaufzeit (30.04.2031), rd. 126.300 € bei Ausübung beider Verlängerungsoptionen. Wirtschaftlich ein amortisierter Baukostenzuschuss. OFFEN: (1) tatsächliche Höhe der Statikkosten beim Vermieter erfragen – daraus ergibt sich der implizite Zins; (2) ob der Betrag der VPI-Wertsicherung unterliegt, ist unklar – §10 indexiert "die Miete", der 3. Nachtrag erstreckt die Klausel aber auf zusätzlich angemietete FLÄCHEN, und die 600 € sind keine Fläche; (3) ob er in den Verlängerungszeiträumen weiterläuft, ist nicht geregelt.</t>
+        </is>
+      </c>
     </row>
     <row r="126" ht="6.75" customHeight="1" thickBot="1">
       <c r="B126" s="7" t="n"/>

</xml_diff>

<commit_message>
Long Version: Kategoriespalte und Standortueberschriften fixiert
freeze_panes C5 haelt die Spalten A/B mit den Kategorien beim seitlichen
Scrollen und die Zeilen 1-4 mit Titel und Standortnamen beim vertikalen
Scrollen sichtbar. Short Version behaelt ihren bestehenden Punkt C7.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018VKr7wEHLAW3yJNS7pxnAu
</commit_message>
<xml_diff>
--- a/mietkonditionen/Mietkonditionen_Vergleich_Wuerselen_Baesweiler.xlsx
+++ b/mietkonditionen/Mietkonditionen_Vergleich_Wuerselen_Baesweiler.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Short Version" sheetId="1" state="visible" r:id="rId1"/>
@@ -497,7 +497,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -719,6 +719,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="2" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -1132,18 +1135,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:F45"/>
+  <dimension ref="B2:F42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5"/>
   <cols>
     <col width="3.81640625" customWidth="1" style="2" min="1" max="1"/>
     <col width="37.81640625" bestFit="1" customWidth="1" style="2" min="2" max="2"/>
-    <col width="11.54296875" customWidth="1" style="2" min="3" max="3"/>
+    <col width="34.90625" bestFit="1" customWidth="1" style="2" min="3" max="3"/>
     <col width="12.81640625" customWidth="1" style="2" min="4" max="6"/>
-    <col width="11.453125" customWidth="1" style="2" min="7" max="9"/>
-    <col width="11.453125" customWidth="1" style="2" min="10" max="16384"/>
+    <col width="11.453125" customWidth="1" style="2" min="7" max="10"/>
+    <col width="11.453125" customWidth="1" style="2" min="11" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -1151,7 +1153,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
@@ -1160,17 +1161,16 @@
       </c>
       <c r="C4" s="25" t="inlineStr">
         <is>
-          <t>Würselen (Target)</t>
+          <t xml:space="preserve">Würselen </t>
         </is>
       </c>
       <c r="D4" s="25" t="inlineStr">
         <is>
-          <t>Baesweiler (Bestand)</t>
+          <t>Baesweiler</t>
         </is>
       </c>
       <c r="E4" s="47" t="n"/>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
         <is>
@@ -1285,7 +1285,7 @@
       </c>
       <c r="C12" s="25" t="inlineStr">
         <is>
-          <t>XXX</t>
+          <t>Expansion</t>
         </is>
       </c>
       <c r="D12" s="25" t="inlineStr">
@@ -1345,7 +1345,7 @@
           <t>XXX</t>
         </is>
       </c>
-      <c r="D15" s="25" t="n">
+      <c r="D15" s="27" t="n">
         <v>18</v>
       </c>
       <c r="E15" s="48" t="n"/>
@@ -1439,7 +1439,7 @@
       <c r="F21" s="26" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="22" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Nettokaltmiete pro Monat</t>
         </is>
@@ -1455,7 +1455,7 @@
       <c r="F22" s="6" t="n"/>
     </row>
     <row r="23">
-      <c r="B23" s="22" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>Nettokaltmiete pro Jahr</t>
         </is>
@@ -1488,7 +1488,7 @@
       <c r="F24" s="26" t="n"/>
     </row>
     <row r="25">
-      <c r="B25" s="22" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>Nebenkosten pro Monat</t>
         </is>
@@ -1504,7 +1504,7 @@
       <c r="F25" s="6" t="n"/>
     </row>
     <row r="26">
-      <c r="B26" s="22" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>Nebenkosten pro Jahr</t>
         </is>
@@ -1551,7 +1551,7 @@
       <c r="F28" s="26" t="n"/>
     </row>
     <row r="29">
-      <c r="B29" s="22" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>Kosten Stellplätze pro Monat</t>
         </is>
@@ -1568,7 +1568,7 @@
       <c r="F29" s="6" t="n"/>
     </row>
     <row r="30">
-      <c r="B30" s="22" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>Kosten Stellplätze pro Jahr</t>
         </is>
@@ -1592,7 +1592,7 @@
       </c>
       <c r="C31" s="25" t="inlineStr">
         <is>
-          <t>Keller 443 €/Mon.; Statik 1. OG 600 €/Mon.</t>
+          <t>Keller 443 €/Mon.</t>
         </is>
       </c>
       <c r="D31" s="25" t="inlineStr">
@@ -1609,8 +1609,10 @@
           <t>Baukostenzuschuss in €</t>
         </is>
       </c>
-      <c r="C32" s="41" t="n">
-        <v>0</v>
+      <c r="C32" s="41" t="inlineStr">
+        <is>
+          <t>Statik 1. OG 600 €/Mon.</t>
+        </is>
       </c>
       <c r="D32" s="41" t="n">
         <v>0</v>
@@ -1626,7 +1628,7 @@
       </c>
       <c r="C33" s="25" t="inlineStr">
         <is>
-          <t>kein BKZ; faktisch 600 €/Mon. für Statik</t>
+          <t xml:space="preserve"> faktisch 600 €/Mon. für Statik = BKZ?</t>
         </is>
       </c>
       <c r="D33" s="25" t="inlineStr">
@@ -1733,7 +1735,7 @@
       </c>
       <c r="C40" s="25" t="inlineStr">
         <is>
-          <t>VPI; 100% der Indexveränderung ab &gt;5%</t>
+          <t>volle Indexveränderung ab &gt;5%</t>
         </is>
       </c>
       <c r="D40" s="25" t="inlineStr">
@@ -1770,12 +1772,9 @@
       <c r="E42" s="7" t="n"/>
       <c r="F42" s="7" t="n"/>
     </row>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
   </sheetData>
   <pageMargins left="0.5118110236220472" right="0.5118110236220472" top="0.7874015748031497" bottom="0.7874015748031497" header="0.3149606299212598" footer="0.3149606299212598"/>
-  <pageSetup orientation="portrait" paperSize="9"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="83"/>
 </worksheet>
 </file>
 
@@ -1785,20 +1784,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:L144"/>
+  <dimension ref="B2:L142"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5"/>
   <cols>
     <col width="3.81640625" customWidth="1" style="2" min="1" max="1"/>
     <col width="44.26953125" customWidth="1" style="2" min="2" max="2"/>
     <col width="42.1796875" customWidth="1" style="2" min="3" max="3"/>
     <col width="12.81640625" customWidth="1" style="2" min="4" max="6"/>
-    <col width="35" customWidth="1" style="51" min="7" max="7"/>
+    <col width="35.453125" customWidth="1" style="51" min="7" max="7"/>
     <col width="12.81640625" customWidth="1" style="2" min="8" max="8"/>
-    <col width="11.453125" customWidth="1" style="2" min="9" max="9"/>
-    <col width="11.453125" customWidth="1" style="2" min="10" max="16384"/>
+    <col width="11.453125" customWidth="1" style="2" min="9" max="10"/>
+    <col width="11.453125" customWidth="1" style="2" min="11" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -2017,7 +2015,7 @@
       <c r="J13" s="26" t="n"/>
       <c r="L13" s="47" t="n"/>
     </row>
-    <row r="14">
+    <row r="14" ht="29" customHeight="1">
       <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Verlängerungsoptionen</t>
@@ -2032,10 +2030,10 @@
       <c r="D14" s="26" t="n"/>
       <c r="E14" s="26" t="n"/>
       <c r="F14" s="26" t="n"/>
-      <c r="G14" s="54" t="inlineStr">
+      <c r="G14" s="78" t="inlineStr">
         <is>
           <t>2x 5 Jahre; 
-nur auf aktive Ausübung, keine Automatik</t>
+nur auf aktive Ausübung</t>
         </is>
       </c>
       <c r="H14" s="26" t="n"/>
@@ -2313,7 +2311,7 @@
       </c>
       <c r="C26" s="25" t="inlineStr">
         <is>
-          <t>umsatzsteuerfrei; Nebenkosten zzgl. USt; Reinigung Treppenhaus/Aufzug 2x wöchentlich durch Mieter</t>
+          <t>Nebenkosten zzgl. USt; Reinigung Treppenhaus/Aufzug 2x wöchentlich durch Mieter</t>
         </is>
       </c>
       <c r="D26" s="26" t="n"/>
@@ -2321,7 +2319,7 @@
       <c r="F26" s="26" t="n"/>
       <c r="G26" s="54" t="inlineStr">
         <is>
-          <t>Schlussabnahme fehlt; Inventar vermieterseitig gestellt; Umstellung auf gewerbliche Wärmelieferung möglich; Zustimmungsfiktion nach 4 Wochen</t>
+          <t>Inventar vermieterseitig gestellt; Umstellung auf gewerbliche Wärmelieferung möglich</t>
         </is>
       </c>
       <c r="H26" s="26" t="n"/>
@@ -2364,13 +2362,13 @@
           <t>Miete/m² (Neubau) - kein BKZ</t>
         </is>
       </c>
-      <c r="C30" s="78" t="n">
+      <c r="C30" s="79" t="n">
         <v>20</v>
       </c>
       <c r="D30" s="26" t="n"/>
       <c r="E30" s="26" t="n"/>
       <c r="F30" s="26" t="n"/>
-      <c r="G30" s="79" t="n">
+      <c r="G30" s="80" t="n">
         <v>20</v>
       </c>
       <c r="H30" s="26" t="n"/>
@@ -2383,13 +2381,13 @@
           <t>Miete/m² inkl. BKZ</t>
         </is>
       </c>
-      <c r="C31" s="78" t="n">
+      <c r="C31" s="79" t="n">
         <v>20</v>
       </c>
       <c r="D31" s="26" t="n"/>
       <c r="E31" s="26" t="n"/>
       <c r="F31" s="26" t="n"/>
-      <c r="G31" s="79" t="n">
+      <c r="G31" s="80" t="n">
         <v>20</v>
       </c>
       <c r="H31" s="26" t="n"/>
@@ -2402,13 +2400,13 @@
           <t>Nebenkosten/m²</t>
         </is>
       </c>
-      <c r="C32" s="78" t="n">
+      <c r="C32" s="79" t="n">
         <v>3</v>
       </c>
       <c r="D32" s="26" t="n"/>
       <c r="E32" s="26" t="n"/>
       <c r="F32" s="26" t="n"/>
-      <c r="G32" s="79" t="n">
+      <c r="G32" s="80" t="n">
         <v>3</v>
       </c>
       <c r="H32" s="26" t="n"/>
@@ -2421,24 +2419,24 @@
           <t>Fläche pro Bett</t>
         </is>
       </c>
-      <c r="C33" s="80" t="inlineStr">
+      <c r="C33" s="81" t="inlineStr">
         <is>
           <t>50m²</t>
         </is>
       </c>
-      <c r="D33" s="81" t="inlineStr">
+      <c r="D33" s="82" t="inlineStr">
         <is>
           <t xml:space="preserve"> (d.h. 6er WG: 300m²; 12er WG: 600m²)</t>
         </is>
       </c>
       <c r="E33" s="26" t="n"/>
       <c r="F33" s="26" t="n"/>
-      <c r="G33" s="82" t="inlineStr">
+      <c r="G33" s="83" t="inlineStr">
         <is>
           <t>50m²</t>
         </is>
       </c>
-      <c r="H33" s="81" t="inlineStr">
+      <c r="H33" s="82" t="inlineStr">
         <is>
           <t xml:space="preserve"> (d.h. 6er WG: 300m²; 12er WG: 600m²)</t>
         </is>
@@ -2452,13 +2450,13 @@
           <t>Miete pro Bett pro Monat (exkl. Baukostenzuschuss)</t>
         </is>
       </c>
-      <c r="C34" s="80" t="n">
+      <c r="C34" s="81" t="n">
         <v>1000</v>
       </c>
       <c r="D34" s="26" t="n"/>
       <c r="E34" s="26" t="n"/>
       <c r="F34" s="26" t="n"/>
-      <c r="G34" s="82" t="n">
+      <c r="G34" s="83" t="n">
         <v>1000</v>
       </c>
       <c r="H34" s="26" t="n"/>
@@ -2471,14 +2469,14 @@
           <t>Miete pro Bett pro Monat (inkl. BKZ über 10 Jahre)</t>
         </is>
       </c>
-      <c r="C35" s="80">
+      <c r="C35" s="81">
         <f>+C34</f>
         <v/>
       </c>
       <c r="D35" s="26" t="n"/>
       <c r="E35" s="26" t="n"/>
       <c r="F35" s="26" t="n"/>
-      <c r="G35" s="82">
+      <c r="G35" s="83">
         <f>+G34</f>
         <v/>
       </c>
@@ -2492,16 +2490,16 @@
           <t>Baukostenzuschuss pro Bett</t>
         </is>
       </c>
-      <c r="C36" s="80" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" s="81" t="n"/>
+      <c r="C36" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="82" t="n"/>
       <c r="E36" s="26" t="n"/>
       <c r="F36" s="26" t="n"/>
-      <c r="G36" s="82" t="n">
-        <v>0</v>
-      </c>
-      <c r="H36" s="81" t="n"/>
+      <c r="G36" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="82" t="n"/>
       <c r="I36" s="26" t="n"/>
       <c r="J36" s="26" t="n"/>
     </row>
@@ -2511,13 +2509,13 @@
           <t>Capex pro Bett (Möbel, Ausstattung, etc.)</t>
         </is>
       </c>
-      <c r="C37" s="80" t="n">
+      <c r="C37" s="81" t="n">
         <v>30000</v>
       </c>
       <c r="D37" s="26" t="n"/>
       <c r="E37" s="26" t="n"/>
       <c r="F37" s="26" t="n"/>
-      <c r="G37" s="82" t="n">
+      <c r="G37" s="83" t="n">
         <v>30000</v>
       </c>
       <c r="H37" s="26" t="n"/>
@@ -2571,13 +2569,13 @@
           <t>Miete/m² (Bestand) - kein BKZ</t>
         </is>
       </c>
-      <c r="C41" s="78" t="n">
+      <c r="C41" s="79" t="n">
         <v>20</v>
       </c>
       <c r="D41" s="26" t="n"/>
       <c r="E41" s="26" t="n"/>
       <c r="F41" s="26" t="n"/>
-      <c r="G41" s="79" t="n">
+      <c r="G41" s="80" t="n">
         <v>20</v>
       </c>
       <c r="H41" s="26" t="n"/>
@@ -2590,13 +2588,13 @@
           <t>Miete/m² (Bestand) inkl. BKZ</t>
         </is>
       </c>
-      <c r="C42" s="78" t="n">
+      <c r="C42" s="79" t="n">
         <v>25</v>
       </c>
       <c r="D42" s="26" t="n"/>
       <c r="E42" s="26" t="n"/>
       <c r="F42" s="26" t="n"/>
-      <c r="G42" s="79" t="n">
+      <c r="G42" s="80" t="n">
         <v>25</v>
       </c>
       <c r="H42" s="26" t="n"/>
@@ -2609,13 +2607,13 @@
           <t>Nebenkosten/m²</t>
         </is>
       </c>
-      <c r="C43" s="78" t="n">
+      <c r="C43" s="79" t="n">
         <v>3</v>
       </c>
       <c r="D43" s="26" t="n"/>
       <c r="E43" s="26" t="n"/>
       <c r="F43" s="26" t="n"/>
-      <c r="G43" s="79" t="n">
+      <c r="G43" s="80" t="n">
         <v>3</v>
       </c>
       <c r="H43" s="26" t="n"/>
@@ -2628,24 +2626,24 @@
           <t>Fläche pro Bett</t>
         </is>
       </c>
-      <c r="C44" s="80" t="inlineStr">
+      <c r="C44" s="81" t="inlineStr">
         <is>
           <t>50m²</t>
         </is>
       </c>
-      <c r="D44" s="81" t="inlineStr">
+      <c r="D44" s="82" t="inlineStr">
         <is>
           <t xml:space="preserve"> (d.h. 6er WG: 300m²; 12er WG: 600m²)</t>
         </is>
       </c>
       <c r="E44" s="26" t="n"/>
       <c r="F44" s="26" t="n"/>
-      <c r="G44" s="82" t="inlineStr">
+      <c r="G44" s="83" t="inlineStr">
         <is>
           <t>50m²</t>
         </is>
       </c>
-      <c r="H44" s="81" t="inlineStr">
+      <c r="H44" s="82" t="inlineStr">
         <is>
           <t xml:space="preserve"> (d.h. 6er WG: 300m²; 12er WG: 600m²)</t>
         </is>
@@ -2659,13 +2657,13 @@
           <t>Miete pro Bett pro Monat (exkl. Baukostenzuschuss)</t>
         </is>
       </c>
-      <c r="C45" s="80" t="n">
+      <c r="C45" s="81" t="n">
         <v>1000</v>
       </c>
       <c r="D45" s="26" t="n"/>
       <c r="E45" s="26" t="n"/>
       <c r="F45" s="26" t="n"/>
-      <c r="G45" s="82" t="n">
+      <c r="G45" s="83" t="n">
         <v>1000</v>
       </c>
       <c r="H45" s="26" t="n"/>
@@ -2678,13 +2676,13 @@
           <t>Miete pro Bett pro Monat (inkl. BKZ über 10 Jahre)</t>
         </is>
       </c>
-      <c r="C46" s="80" t="n">
+      <c r="C46" s="81" t="n">
         <v>1250</v>
       </c>
       <c r="D46" s="26" t="n"/>
       <c r="E46" s="26" t="n"/>
       <c r="F46" s="26" t="n"/>
-      <c r="G46" s="82" t="n">
+      <c r="G46" s="83" t="n">
         <v>1250</v>
       </c>
       <c r="H46" s="26" t="n"/>
@@ -2697,20 +2695,20 @@
           <t>Baukostenzuschuss pro Bett</t>
         </is>
       </c>
-      <c r="C47" s="80" t="n">
+      <c r="C47" s="81" t="n">
         <v>40000</v>
       </c>
-      <c r="D47" s="81" t="inlineStr">
+      <c r="D47" s="82" t="inlineStr">
         <is>
           <t>(d.h. 6er WG: 180.000 €, 12er WG: 360.000 €)</t>
         </is>
       </c>
       <c r="E47" s="26" t="n"/>
       <c r="F47" s="26" t="n"/>
-      <c r="G47" s="82" t="n">
+      <c r="G47" s="83" t="n">
         <v>40000</v>
       </c>
-      <c r="H47" s="81" t="inlineStr">
+      <c r="H47" s="82" t="inlineStr">
         <is>
           <t>(d.h. 6er WG: 180.000 €, 12er WG: 360.000 €)</t>
         </is>
@@ -2724,13 +2722,13 @@
           <t>Capex pro Bett (Möbel, Ausstattung, etc.)</t>
         </is>
       </c>
-      <c r="C48" s="80" t="n">
+      <c r="C48" s="81" t="n">
         <v>30000</v>
       </c>
       <c r="D48" s="26" t="n"/>
       <c r="E48" s="26" t="n"/>
       <c r="F48" s="26" t="n"/>
-      <c r="G48" s="82" t="n">
+      <c r="G48" s="83" t="n">
         <v>30000</v>
       </c>
       <c r="H48" s="26" t="n"/>
@@ -4181,7 +4179,7 @@
       </c>
       <c r="C111" s="25" t="inlineStr">
         <is>
-          <t>Mieter; Pavillon nur vorgerüstet</t>
+          <t>XXX</t>
         </is>
       </c>
       <c r="D111" s="39" t="n"/>
@@ -4850,8 +4848,6 @@
       <c r="I142" s="7" t="n"/>
       <c r="J142" s="7" t="n"/>
     </row>
-    <row r="143"/>
-    <row r="144"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="C22:F22"/>

</xml_diff>